<commit_message>
refactor(tests+thermal): clean up unused mappings and constants, streamline thermal type filtering logic (delete dropna filter on key)
</commit_message>
<xml_diff>
--- a/tests/antares/resources/MAIN_PARAMS_2025.xlsx
+++ b/tests/antares/resources/MAIN_PARAMS_2025.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1529" uniqueCount="566">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1517" uniqueCount="564">
   <si>
     <t xml:space="preserve">dossier PEMMDB</t>
   </si>
@@ -1052,12 +1052,6 @@
   </si>
   <si>
     <t xml:space="preserve">Lignite old 2 CHP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gas pcomp CCS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gas pcomp H2</t>
   </si>
   <si>
     <t xml:space="preserve">Nuclear/-</t>
@@ -1971,10 +1965,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1984,6 +1974,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2118,9 +2112,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
-      <xdr:colOff>109440</xdr:colOff>
+      <xdr:colOff>109080</xdr:colOff>
       <xdr:row>10</xdr:row>
-      <xdr:rowOff>127440</xdr:rowOff>
+      <xdr:rowOff>127080</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -2129,8 +2123,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7523640" y="952560"/>
-          <a:ext cx="7632720" cy="1080000"/>
+          <a:off x="7528680" y="952560"/>
+          <a:ext cx="7637400" cy="1079640"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2230,9 +2224,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
-      <xdr:colOff>311040</xdr:colOff>
+      <xdr:colOff>310680</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>176040</xdr:rowOff>
+      <xdr:rowOff>175680</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -2241,8 +2235,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="11264040" y="429480"/>
-          <a:ext cx="8258400" cy="1080000"/>
+          <a:off x="11264760" y="429480"/>
+          <a:ext cx="8263440" cy="1079640"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2333,9 +2327,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>243000</xdr:colOff>
+      <xdr:colOff>242640</xdr:colOff>
       <xdr:row>26</xdr:row>
-      <xdr:rowOff>49320</xdr:rowOff>
+      <xdr:rowOff>48960</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -2344,8 +2338,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13868640" y="560160"/>
-          <a:ext cx="6840360" cy="4400280"/>
+          <a:off x="13867920" y="560160"/>
+          <a:ext cx="6843240" cy="4399920"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2778,9 +2772,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>550800</xdr:colOff>
+      <xdr:colOff>550440</xdr:colOff>
       <xdr:row>25</xdr:row>
-      <xdr:rowOff>111960</xdr:rowOff>
+      <xdr:rowOff>111600</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -2789,8 +2783,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13863600" y="771480"/>
-          <a:ext cx="7153200" cy="4061160"/>
+          <a:off x="13862880" y="771480"/>
+          <a:ext cx="7156080" cy="4060800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3232,9 +3226,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>318600</xdr:colOff>
+      <xdr:colOff>318240</xdr:colOff>
       <xdr:row>17</xdr:row>
-      <xdr:rowOff>128160</xdr:rowOff>
+      <xdr:rowOff>127800</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -3244,7 +3238,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="6582240" y="409320"/>
-          <a:ext cx="10342080" cy="2957400"/>
+          <a:ext cx="10347480" cy="2957040"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3558,7 +3552,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B25"/>
-  <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.5859375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="65.43"/>
@@ -3632,7 +3626,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D27"/>
-  <sheetFormatPr defaultColWidth="10.8671875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="8" width="10.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.57"/>
@@ -3648,152 +3642,152 @@
         <v>247</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="20" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="20" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="20" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="20" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="20" t="s">
+        <v>378</v>
+      </c>
+      <c r="B6" s="0" t="s">
         <v>380</v>
       </c>
-      <c r="B6" s="0" t="s">
-        <v>382</v>
-      </c>
       <c r="C6" s="0" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="20" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="C7" s="0" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="20" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="20" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="20" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="C10" s="0" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="B11" s="0" t="s">
+        <v>515</v>
+      </c>
+      <c r="C11" s="0" t="s">
+        <v>516</v>
+      </c>
+      <c r="D11" s="0" t="s">
         <v>517</v>
-      </c>
-      <c r="C11" s="0" t="s">
-        <v>518</v>
-      </c>
-      <c r="D11" s="0" t="s">
-        <v>519</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="20" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="B12" s="0" t="s">
+        <v>518</v>
+      </c>
+      <c r="C12" s="0" t="s">
+        <v>519</v>
+      </c>
+      <c r="D12" s="0" t="s">
         <v>520</v>
-      </c>
-      <c r="C12" s="0" t="s">
-        <v>521</v>
-      </c>
-      <c r="D12" s="0" t="s">
-        <v>522</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3863,7 +3857,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C71"/>
-  <sheetFormatPr defaultColWidth="10.8671875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="31"/>
@@ -3886,10 +3880,10 @@
         <v>15</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3897,10 +3891,10 @@
         <v>15</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3908,10 +3902,10 @@
         <v>15</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3919,10 +3913,10 @@
         <v>15</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3930,10 +3924,10 @@
         <v>15</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="C6" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3944,7 +3938,7 @@
         <v>331</v>
       </c>
       <c r="C7" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3955,7 +3949,7 @@
         <v>336</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3966,7 +3960,7 @@
         <v>326</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3974,10 +3968,10 @@
         <v>15</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
       <c r="C10" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3988,7 +3982,7 @@
         <v>288</v>
       </c>
       <c r="C11" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3999,7 +3993,7 @@
         <v>294</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4010,7 +4004,7 @@
         <v>278</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4021,7 +4015,7 @@
         <v>282</v>
       </c>
       <c r="C14" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4032,7 +4026,7 @@
         <v>266</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4043,7 +4037,7 @@
         <v>272</v>
       </c>
       <c r="C16" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4054,7 +4048,7 @@
         <v>261</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4065,7 +4059,7 @@
         <v>250</v>
       </c>
       <c r="C18" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4073,10 +4067,10 @@
         <v>15</v>
       </c>
       <c r="B19" s="0" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="C19" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4084,10 +4078,10 @@
         <v>15</v>
       </c>
       <c r="B20" s="0" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="C20" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4098,7 +4092,7 @@
         <v>321</v>
       </c>
       <c r="C21" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4109,7 +4103,7 @@
         <v>313</v>
       </c>
       <c r="C22" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4120,7 +4114,7 @@
         <v>317</v>
       </c>
       <c r="C23" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4128,10 +4122,10 @@
         <v>15</v>
       </c>
       <c r="B24" s="0" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="C24" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4139,10 +4133,10 @@
         <v>15</v>
       </c>
       <c r="B25" s="0" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="C25" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4150,10 +4144,10 @@
         <v>15</v>
       </c>
       <c r="B26" s="0" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="C26" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4161,10 +4155,10 @@
         <v>15</v>
       </c>
       <c r="B27" s="0" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="C27" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4172,10 +4166,10 @@
         <v>15</v>
       </c>
       <c r="B28" s="0" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="C28" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4183,10 +4177,10 @@
         <v>15</v>
       </c>
       <c r="B29" s="0" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="C29" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4194,10 +4188,10 @@
         <v>15</v>
       </c>
       <c r="B30" s="0" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="C30" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4205,10 +4199,10 @@
         <v>15</v>
       </c>
       <c r="B31" s="0" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="C31" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4216,10 +4210,10 @@
         <v>15</v>
       </c>
       <c r="B32" s="0" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="C32" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4227,10 +4221,10 @@
         <v>15</v>
       </c>
       <c r="B33" s="0" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="C33" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4238,10 +4232,10 @@
         <v>15</v>
       </c>
       <c r="B34" s="0" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="C34" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4249,10 +4243,10 @@
         <v>15</v>
       </c>
       <c r="B35" s="0" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="C35" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4260,10 +4254,10 @@
         <v>15</v>
       </c>
       <c r="B36" s="0" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="C36" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4271,10 +4265,10 @@
         <v>15</v>
       </c>
       <c r="B37" s="0" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="C37" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4282,10 +4276,10 @@
         <v>15</v>
       </c>
       <c r="B38" s="0" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="C38" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4293,10 +4287,10 @@
         <v>15</v>
       </c>
       <c r="B39" s="0" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="C39" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4304,10 +4298,10 @@
         <v>15</v>
       </c>
       <c r="B40" s="0" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="C40" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4315,10 +4309,10 @@
         <v>15</v>
       </c>
       <c r="B41" s="11" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="C41" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4326,10 +4320,10 @@
         <v>15</v>
       </c>
       <c r="B42" s="10" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="C42" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4337,10 +4331,10 @@
         <v>15</v>
       </c>
       <c r="B43" s="11" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="C43" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4348,10 +4342,10 @@
         <v>15</v>
       </c>
       <c r="B44" s="0" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="C44" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4359,10 +4353,10 @@
         <v>15</v>
       </c>
       <c r="B45" s="0" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="C45" s="0" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4370,10 +4364,10 @@
         <v>15</v>
       </c>
       <c r="B46" s="0" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="C46" s="0" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4381,10 +4375,10 @@
         <v>15</v>
       </c>
       <c r="B47" s="0" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="C47" s="0" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4392,10 +4386,10 @@
         <v>15</v>
       </c>
       <c r="B48" s="0" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="C48" s="0" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4403,10 +4397,10 @@
         <v>15</v>
       </c>
       <c r="B49" s="0" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="C49" s="0" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4414,10 +4408,10 @@
         <v>15</v>
       </c>
       <c r="B50" s="0" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="C50" s="0" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4425,10 +4419,10 @@
         <v>15</v>
       </c>
       <c r="B51" s="0" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="C51" s="0" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4436,10 +4430,10 @@
         <v>15</v>
       </c>
       <c r="B52" s="0" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="C52" s="0" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4447,10 +4441,10 @@
         <v>15</v>
       </c>
       <c r="B53" s="0" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
       <c r="C53" s="0" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4458,10 +4452,10 @@
         <v>15</v>
       </c>
       <c r="B54" s="0" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
       <c r="C54" s="0" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4469,10 +4463,10 @@
         <v>15</v>
       </c>
       <c r="B55" s="0" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
       <c r="C55" s="0" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4480,10 +4474,10 @@
         <v>15</v>
       </c>
       <c r="B56" s="0" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="C56" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4491,10 +4485,10 @@
         <v>15</v>
       </c>
       <c r="B57" s="0" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
       <c r="C57" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4502,10 +4496,10 @@
         <v>15</v>
       </c>
       <c r="B58" s="0" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
       <c r="C58" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4513,10 +4507,10 @@
         <v>15</v>
       </c>
       <c r="B59" s="0" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="C59" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4524,10 +4518,10 @@
         <v>15</v>
       </c>
       <c r="B60" s="0" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="C60" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4535,10 +4529,10 @@
         <v>15</v>
       </c>
       <c r="B61" s="0" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
       <c r="C61" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4546,10 +4540,10 @@
         <v>15</v>
       </c>
       <c r="B62" s="0" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
       <c r="C62" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4557,10 +4551,10 @@
         <v>15</v>
       </c>
       <c r="B63" s="0" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
       <c r="C63" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4568,10 +4562,10 @@
         <v>15</v>
       </c>
       <c r="B64" s="0" t="s">
-        <v>548</v>
+        <v>546</v>
       </c>
       <c r="C64" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4579,10 +4573,10 @@
         <v>15</v>
       </c>
       <c r="B65" s="0" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
       <c r="C65" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4590,10 +4584,10 @@
         <v>15</v>
       </c>
       <c r="B66" s="0" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="C66" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4601,10 +4595,10 @@
         <v>15</v>
       </c>
       <c r="B67" s="0" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
       <c r="C67" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4612,10 +4606,10 @@
         <v>15</v>
       </c>
       <c r="B68" s="0" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
       <c r="C68" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4623,10 +4617,10 @@
         <v>15</v>
       </c>
       <c r="B69" s="0" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
       <c r="C69" s="0" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="60" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4634,10 +4628,10 @@
         <v>15</v>
       </c>
       <c r="B70" s="21" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
       <c r="C70" s="10" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="60" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4645,10 +4639,10 @@
         <v>15</v>
       </c>
       <c r="B71" s="21" t="s">
+        <v>553</v>
+      </c>
+      <c r="C71" s="10" t="s">
         <v>555</v>
-      </c>
-      <c r="C71" s="10" t="s">
-        <v>557</v>
       </c>
     </row>
   </sheetData>
@@ -4669,20 +4663,20 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D25"/>
-  <sheetFormatPr defaultColWidth="9.15234375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.16015625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="22" t="s">
+        <v>556</v>
+      </c>
+      <c r="B1" s="22" t="s">
+        <v>557</v>
+      </c>
+      <c r="C1" s="22" t="s">
         <v>558</v>
       </c>
-      <c r="B1" s="22" t="s">
+      <c r="D1" s="22" t="s">
         <v>559</v>
-      </c>
-      <c r="C1" s="22" t="s">
-        <v>560</v>
-      </c>
-      <c r="D1" s="22" t="s">
-        <v>561</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4690,13 +4684,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="23" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="C2" s="23" t="n">
         <v>1</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4704,13 +4698,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="23" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="C3" s="23" t="n">
         <v>2</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4718,13 +4712,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="23" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="C4" s="23" t="n">
         <v>3</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4732,13 +4726,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="C5" s="23" t="n">
         <v>4</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4746,13 +4740,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="C6" s="23" t="n">
         <v>5</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4760,13 +4754,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="C7" s="23" t="n">
         <v>6</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4774,13 +4768,13 @@
         <v>7</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="C8" s="23" t="n">
         <v>7</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4788,13 +4782,13 @@
         <v>8</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="C9" s="23" t="n">
         <v>8</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4802,13 +4796,13 @@
         <v>9</v>
       </c>
       <c r="B10" s="23" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="C10" s="23" t="n">
         <v>9</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4816,13 +4810,13 @@
         <v>10</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="C11" s="23" t="n">
         <v>10</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4830,13 +4824,13 @@
         <v>11</v>
       </c>
       <c r="B12" s="23" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="C12" s="23" t="n">
         <v>11</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4844,13 +4838,13 @@
         <v>12</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="C13" s="23" t="n">
         <v>12</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4858,7 +4852,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="23" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="C14" s="23"/>
       <c r="D14" s="23"/>
@@ -4868,7 +4862,7 @@
         <v>14</v>
       </c>
       <c r="B15" s="23" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="C15" s="23"/>
       <c r="D15" s="23"/>
@@ -4878,7 +4872,7 @@
         <v>15</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="C16" s="23"/>
       <c r="D16" s="23"/>
@@ -4888,7 +4882,7 @@
         <v>16</v>
       </c>
       <c r="B17" s="23" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="C17" s="23"/>
       <c r="D17" s="23"/>
@@ -4898,7 +4892,7 @@
         <v>17</v>
       </c>
       <c r="B18" s="23" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="C18" s="23"/>
       <c r="D18" s="23"/>
@@ -4908,7 +4902,7 @@
         <v>18</v>
       </c>
       <c r="B19" s="23" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="C19" s="23"/>
       <c r="D19" s="23"/>
@@ -4918,7 +4912,7 @@
         <v>19</v>
       </c>
       <c r="B20" s="23" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="C20" s="23"/>
       <c r="D20" s="23"/>
@@ -4928,7 +4922,7 @@
         <v>20</v>
       </c>
       <c r="B21" s="23" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="C21" s="23"/>
       <c r="D21" s="23"/>
@@ -4938,7 +4932,7 @@
         <v>21</v>
       </c>
       <c r="B22" s="23" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="C22" s="23"/>
       <c r="D22" s="23"/>
@@ -4948,7 +4942,7 @@
         <v>22</v>
       </c>
       <c r="B23" s="23" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="C23" s="23"/>
       <c r="D23" s="23"/>
@@ -4958,7 +4952,7 @@
         <v>23</v>
       </c>
       <c r="B24" s="23" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="C24" s="23"/>
       <c r="D24" s="23"/>
@@ -4968,7 +4962,7 @@
         <v>24</v>
       </c>
       <c r="B25" s="23" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="C25" s="23"/>
       <c r="D25" s="23"/>
@@ -4990,7 +4984,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E107"/>
-  <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.5859375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="7" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="34.43"/>
@@ -6726,7 +6720,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B43"/>
-  <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.5859375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
@@ -7126,7 +7120,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B60"/>
-  <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.5859375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="8" width="17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.43"/>
@@ -7628,8 +7622,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C91"/>
-  <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:C1048576"/>
+  <sheetFormatPr defaultColWidth="10.5859375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="8" width="10.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="8" width="69.43"/>
@@ -8245,18 +8239,22 @@
       <c r="A56" s="12" t="s">
         <v>248</v>
       </c>
-      <c r="B56" s="12"/>
-      <c r="C56" s="13" t="s">
+      <c r="B56" s="12" t="s">
         <v>339</v>
+      </c>
+      <c r="C56" s="12" t="s">
+        <v>340</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="12" t="s">
         <v>248</v>
       </c>
-      <c r="B57" s="12"/>
-      <c r="C57" s="13" t="s">
-        <v>340</v>
+      <c r="B57" s="12" t="s">
+        <v>341</v>
+      </c>
+      <c r="C57" s="12" t="s">
+        <v>342</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8264,10 +8262,10 @@
         <v>248</v>
       </c>
       <c r="B58" s="12" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="C58" s="12" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8275,10 +8273,10 @@
         <v>248</v>
       </c>
       <c r="B59" s="12" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="C59" s="12" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8286,7 +8284,7 @@
         <v>248</v>
       </c>
       <c r="B60" s="12" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="C60" s="12" t="s">
         <v>346</v>
@@ -8297,10 +8295,10 @@
         <v>248</v>
       </c>
       <c r="B61" s="12" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="C61" s="12" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8308,10 +8306,10 @@
         <v>248</v>
       </c>
       <c r="B62" s="12" t="s">
+        <v>350</v>
+      </c>
+      <c r="C62" s="12" t="s">
         <v>349</v>
-      </c>
-      <c r="C62" s="12" t="s">
-        <v>348</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8319,10 +8317,10 @@
         <v>248</v>
       </c>
       <c r="B63" s="12" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="C63" s="12" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8330,10 +8328,10 @@
         <v>248</v>
       </c>
       <c r="B64" s="12" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C64" s="12" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8341,7 +8339,7 @@
         <v>248</v>
       </c>
       <c r="B65" s="12" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="C65" s="12" t="s">
         <v>354</v>
@@ -8352,10 +8350,10 @@
         <v>248</v>
       </c>
       <c r="B66" s="12" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="C66" s="12" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8363,10 +8361,10 @@
         <v>248</v>
       </c>
       <c r="B67" s="12" t="s">
+        <v>358</v>
+      </c>
+      <c r="C67" s="12" t="s">
         <v>357</v>
-      </c>
-      <c r="C67" s="12" t="s">
-        <v>356</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8374,10 +8372,10 @@
         <v>248</v>
       </c>
       <c r="B68" s="12" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="C68" s="12" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8385,10 +8383,10 @@
         <v>248</v>
       </c>
       <c r="B69" s="12" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="C69" s="12" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8396,7 +8394,7 @@
         <v>248</v>
       </c>
       <c r="B70" s="12" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="C70" s="12" t="s">
         <v>362</v>
@@ -8404,32 +8402,32 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="12" t="s">
-        <v>248</v>
+        <v>364</v>
       </c>
       <c r="B71" s="12" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C71" s="12" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="12" t="s">
-        <v>248</v>
+        <v>364</v>
       </c>
       <c r="B72" s="12" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="C72" s="12" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="12" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B73" s="12" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="C73" s="12" t="s">
         <v>368</v>
@@ -8437,153 +8435,153 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="12" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B74" s="12" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="C74" s="12" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="12" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B75" s="12" t="s">
+        <v>372</v>
+      </c>
+      <c r="C75" s="12" t="s">
         <v>371</v>
-      </c>
-      <c r="C75" s="12" t="s">
-        <v>370</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="12" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B76" s="12" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C76" s="12" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="12" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B77" s="12" t="s">
+        <v>375</v>
+      </c>
+      <c r="C77" s="12" t="s">
         <v>374</v>
-      </c>
-      <c r="C77" s="12" t="s">
-        <v>373</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="12" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B78" s="12" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C78" s="12" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="12" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B79" s="12" t="s">
         <v>377</v>
       </c>
       <c r="C79" s="12" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="12" t="s">
-        <v>366</v>
+        <v>378</v>
       </c>
       <c r="B80" s="12" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C80" s="12" t="s">
-        <v>376</v>
+        <v>380</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="12" t="s">
-        <v>366</v>
+        <v>378</v>
       </c>
       <c r="B81" s="12" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="C81" s="12" t="s">
-        <v>376</v>
+        <v>382</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="12" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="B82" s="12" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="C82" s="12" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="12" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="B83" s="12" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="C83" s="12" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="12" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="B84" s="12" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="C84" s="12" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="12" t="s">
-        <v>380</v>
+        <v>389</v>
       </c>
       <c r="B85" s="12" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="C85" s="12" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="12" t="s">
-        <v>380</v>
+        <v>389</v>
       </c>
       <c r="B86" s="12" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="C86" s="12" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="12" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="B87" s="12" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="C87" s="12" t="s">
         <v>393</v>
@@ -8591,48 +8589,28 @@
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="12" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="B88" s="12" t="s">
         <v>394</v>
       </c>
       <c r="C88" s="12" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="12" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="B89" s="12" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="C89" s="12" t="s">
-        <v>395</v>
-      </c>
-    </row>
-    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="12" t="s">
-        <v>391</v>
-      </c>
-      <c r="B90" s="12" t="s">
-        <v>396</v>
-      </c>
-      <c r="C90" s="12" t="s">
         <v>397</v>
       </c>
     </row>
-    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="12" t="s">
-        <v>391</v>
-      </c>
-      <c r="B91" s="12" t="s">
-        <v>398</v>
-      </c>
-      <c r="C91" s="12" t="s">
-        <v>399</v>
-      </c>
-    </row>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <autoFilter ref="A1:C1"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -8652,7 +8630,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C20"/>
-  <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.5859375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="11" width="18"/>
@@ -8668,7 +8646,7 @@
         <v>247</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8679,7 +8657,7 @@
         <v>266</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8690,7 +8668,7 @@
         <v>269</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8701,7 +8679,7 @@
         <v>269</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8712,7 +8690,7 @@
         <v>280</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8723,7 +8701,7 @@
         <v>300</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8734,7 +8712,7 @@
         <v>302</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8745,7 +8723,7 @@
         <v>304</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8756,7 +8734,7 @@
         <v>307</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8767,7 +8745,7 @@
         <v>307</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8778,7 +8756,7 @@
         <v>309</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8789,7 +8767,7 @@
         <v>311</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8800,7 +8778,7 @@
         <v>329</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8811,7 +8789,7 @@
         <v>331</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8822,7 +8800,7 @@
         <v>333</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8833,7 +8811,7 @@
         <v>333</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8844,40 +8822,40 @@
         <v>336</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
     </row>
   </sheetData>
@@ -8897,7 +8875,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I10"/>
-  <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.5859375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="11" width="21.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="36.7"/>
@@ -8909,79 +8887,79 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="13" t="s">
+        <v>415</v>
+      </c>
+      <c r="B1" s="14" t="s">
+        <v>416</v>
+      </c>
+      <c r="C1" s="14" t="s">
         <v>417</v>
       </c>
-      <c r="B1" s="15" t="s">
+      <c r="D1" s="15" t="s">
         <v>418</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="E1" s="15" t="s">
         <v>419</v>
       </c>
-      <c r="D1" s="16" t="s">
+      <c r="F1" s="15" t="s">
         <v>420</v>
-      </c>
-      <c r="E1" s="16" t="s">
-        <v>421</v>
-      </c>
-      <c r="F1" s="16" t="s">
-        <v>422</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
+        <v>421</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>422</v>
+      </c>
+      <c r="C2" s="11" t="s">
         <v>423</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="D2" s="11" t="s">
         <v>424</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="E2" s="11" t="s">
         <v>425</v>
       </c>
-      <c r="D2" s="11" t="s">
+      <c r="F2" s="11" t="s">
         <v>426</v>
-      </c>
-      <c r="E2" s="11" t="s">
-        <v>427</v>
-      </c>
-      <c r="F2" s="11" t="s">
-        <v>428</v>
       </c>
       <c r="I2" s="11"/>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="11" t="s">
+        <v>427</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>428</v>
+      </c>
+      <c r="C3" s="11" t="s">
         <v>429</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="D3" s="11" t="s">
         <v>430</v>
       </c>
-      <c r="C3" s="11" t="s">
+      <c r="E3" s="11" t="s">
         <v>431</v>
-      </c>
-      <c r="D3" s="11" t="s">
-        <v>432</v>
-      </c>
-      <c r="E3" s="11" t="s">
-        <v>433</v>
       </c>
       <c r="F3" s="11"/>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="C4" s="11" t="s">
+        <v>423</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>424</v>
+      </c>
+      <c r="E4" s="11" t="s">
         <v>425</v>
-      </c>
-      <c r="D4" s="11" t="s">
-        <v>426</v>
-      </c>
-      <c r="E4" s="11" t="s">
-        <v>427</v>
       </c>
       <c r="F4" s="11" t="s">
         <v>245</v>
@@ -8989,19 +8967,19 @@
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="B5" s="11" t="s">
+        <v>428</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>429</v>
+      </c>
+      <c r="D5" s="11" t="s">
         <v>430</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="E5" s="11" t="s">
         <v>431</v>
-      </c>
-      <c r="D5" s="11" t="s">
-        <v>432</v>
-      </c>
-      <c r="E5" s="11" t="s">
-        <v>433</v>
       </c>
       <c r="F5" s="11"/>
     </row>
@@ -9026,7 +9004,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E80"/>
-  <sheetFormatPr defaultColWidth="8.58203125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5859375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="19.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="22.57"/>
@@ -9036,28 +9014,28 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>437</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>438</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>439</v>
       </c>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="13"/>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
+      <c r="A2" s="16"/>
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
       <c r="D2" s="11"/>
       <c r="E2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="13"/>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
+      <c r="A3" s="16"/>
+      <c r="B3" s="16"/>
+      <c r="C3" s="16"/>
       <c r="D3" s="11"/>
       <c r="E3" s="11"/>
     </row>
@@ -9490,8 +9468,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AC69"/>
-  <sheetFormatPr defaultColWidth="9.15234375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:AC1048576"/>
+  <sheetFormatPr defaultColWidth="9.16015625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19"/>
@@ -9500,106 +9478,106 @@
   <sheetData>
     <row r="1" customFormat="false" ht="60" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
+        <v>438</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>439</v>
+      </c>
+      <c r="C1" s="9" t="s">
         <v>440</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="D1" s="9" t="s">
         <v>441</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="E1" s="9" t="s">
         <v>442</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="F1" s="9" t="s">
         <v>443</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="G1" s="9" t="s">
         <v>444</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="H1" s="9" t="s">
         <v>445</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="I1" s="9" t="s">
         <v>446</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="J1" s="9" t="s">
         <v>447</v>
       </c>
-      <c r="I1" s="9" t="s">
+      <c r="K1" s="9" t="s">
         <v>448</v>
       </c>
-      <c r="J1" s="9" t="s">
+      <c r="L1" s="9" t="s">
         <v>449</v>
       </c>
-      <c r="K1" s="9" t="s">
+      <c r="M1" s="9" t="s">
         <v>450</v>
       </c>
-      <c r="L1" s="9" t="s">
+      <c r="N1" s="9" t="s">
         <v>451</v>
       </c>
-      <c r="M1" s="9" t="s">
+      <c r="O1" s="9" t="s">
         <v>452</v>
       </c>
-      <c r="N1" s="9" t="s">
+      <c r="P1" s="9" t="s">
         <v>453</v>
       </c>
-      <c r="O1" s="9" t="s">
+      <c r="Q1" s="9" t="s">
         <v>454</v>
       </c>
-      <c r="P1" s="9" t="s">
+      <c r="R1" s="9" t="s">
         <v>455</v>
       </c>
-      <c r="Q1" s="9" t="s">
+      <c r="S1" s="9" t="s">
         <v>456</v>
       </c>
-      <c r="R1" s="9" t="s">
+      <c r="T1" s="9" t="s">
         <v>457</v>
       </c>
-      <c r="S1" s="9" t="s">
+      <c r="U1" s="9" t="s">
         <v>458</v>
       </c>
-      <c r="T1" s="9" t="s">
+      <c r="V1" s="9" t="s">
         <v>459</v>
       </c>
-      <c r="U1" s="9" t="s">
+      <c r="W1" s="9" t="s">
         <v>460</v>
       </c>
-      <c r="V1" s="9" t="s">
+      <c r="X1" s="9" t="s">
         <v>461</v>
       </c>
-      <c r="W1" s="9" t="s">
+      <c r="Y1" s="9" t="s">
         <v>462</v>
       </c>
-      <c r="X1" s="9" t="s">
+      <c r="Z1" s="9" t="s">
         <v>463</v>
       </c>
-      <c r="Y1" s="9" t="s">
+      <c r="AA1" s="9" t="s">
         <v>464</v>
       </c>
-      <c r="Z1" s="9" t="s">
+      <c r="AB1" s="9" t="s">
         <v>465</v>
-      </c>
-      <c r="AA1" s="9" t="s">
-        <v>466</v>
-      </c>
-      <c r="AB1" s="9" t="s">
-        <v>467</v>
       </c>
       <c r="AC1" s="9"/>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="B2" s="18" t="n">
         <v>1</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="F2" s="18" t="n">
         <v>0.33</v>
@@ -9674,19 +9652,19 @@
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="B3" s="18" t="n">
         <v>1</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="F3" s="18" t="n">
         <v>0.33</v>
@@ -9767,13 +9745,13 @@
         <v>2</v>
       </c>
       <c r="C4" s="10" t="s">
+        <v>469</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>470</v>
+      </c>
+      <c r="E4" s="10" t="s">
         <v>471</v>
-      </c>
-      <c r="D4" s="10" t="s">
-        <v>472</v>
-      </c>
-      <c r="E4" s="10" t="s">
-        <v>473</v>
       </c>
       <c r="F4" s="18" t="n">
         <v>0.35</v>
@@ -9854,13 +9832,13 @@
         <v>2</v>
       </c>
       <c r="C5" s="10" t="s">
+        <v>469</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>470</v>
+      </c>
+      <c r="E5" s="10" t="s">
         <v>471</v>
-      </c>
-      <c r="D5" s="10" t="s">
-        <v>472</v>
-      </c>
-      <c r="E5" s="10" t="s">
-        <v>473</v>
       </c>
       <c r="F5" s="18" t="n">
         <v>0.35</v>
@@ -9941,13 +9919,13 @@
         <v>3</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="F6" s="18" t="n">
         <v>0.4</v>
@@ -10028,13 +10006,13 @@
         <v>3</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="F7" s="18" t="n">
         <v>0.4</v>
@@ -10115,13 +10093,13 @@
         <v>4</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="F8" s="18" t="n">
         <v>0.46</v>
@@ -10202,13 +10180,13 @@
         <v>4</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="F9" s="18" t="n">
         <v>0.46</v>
@@ -10289,13 +10267,13 @@
         <v>6</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="F10" s="18" t="n">
         <v>0.35</v>
@@ -10376,13 +10354,13 @@
         <v>6</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="F11" s="18" t="n">
         <v>0.35</v>
@@ -10463,13 +10441,13 @@
         <v>7</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="F12" s="18" t="n">
         <v>0.4</v>
@@ -10550,13 +10528,13 @@
         <v>7</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="F13" s="18" t="n">
         <v>0.4</v>
@@ -10637,13 +10615,13 @@
         <v>8</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="F14" s="18" t="n">
         <v>0.46</v>
@@ -10724,13 +10702,13 @@
         <v>8</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="F15" s="18" t="n">
         <v>0.46</v>
@@ -10811,13 +10789,13 @@
         <v>10</v>
       </c>
       <c r="C16" s="10" t="s">
+        <v>477</v>
+      </c>
+      <c r="D16" s="10" t="s">
+        <v>478</v>
+      </c>
+      <c r="E16" s="10" t="s">
         <v>479</v>
-      </c>
-      <c r="D16" s="10" t="s">
-        <v>480</v>
-      </c>
-      <c r="E16" s="10" t="s">
-        <v>481</v>
       </c>
       <c r="F16" s="18" t="n">
         <v>0.36</v>
@@ -10898,13 +10876,13 @@
         <v>10</v>
       </c>
       <c r="C17" s="10" t="s">
+        <v>477</v>
+      </c>
+      <c r="D17" s="10" t="s">
+        <v>478</v>
+      </c>
+      <c r="E17" s="10" t="s">
         <v>479</v>
-      </c>
-      <c r="D17" s="10" t="s">
-        <v>480</v>
-      </c>
-      <c r="E17" s="10" t="s">
-        <v>481</v>
       </c>
       <c r="F17" s="18" t="n">
         <v>0.36</v>
@@ -10985,13 +10963,13 @@
         <v>11</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="F18" s="18" t="n">
         <v>0.41</v>
@@ -11072,13 +11050,13 @@
         <v>11</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="F19" s="18" t="n">
         <v>0.41</v>
@@ -11159,13 +11137,13 @@
         <v>12</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D20" s="10" t="s">
         <v>266</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="F20" s="18" t="n">
         <v>0.4</v>
@@ -11246,13 +11224,13 @@
         <v>12</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D21" s="10" t="s">
         <v>266</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="F21" s="18" t="n">
         <v>0.4</v>
@@ -11333,13 +11311,13 @@
         <v>13</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D22" s="10" t="s">
         <v>272</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="F22" s="18" t="n">
         <v>0.48</v>
@@ -11420,13 +11398,13 @@
         <v>13</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D23" s="10" t="s">
         <v>272</v>
       </c>
       <c r="E23" s="10" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="F23" s="18" t="n">
         <v>0.48</v>
@@ -11507,13 +11485,13 @@
         <v>14</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D24" s="10" t="s">
         <v>278</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="F24" s="18" t="n">
         <v>0.56</v>
@@ -11594,13 +11572,13 @@
         <v>14</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D25" s="10" t="s">
         <v>278</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="F25" s="18" t="n">
         <v>0.56</v>
@@ -11681,13 +11659,13 @@
         <v>15</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D26" s="10" t="s">
         <v>282</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="F26" s="18" t="n">
         <v>0.58</v>
@@ -11768,13 +11746,13 @@
         <v>15</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D27" s="10" t="s">
         <v>282</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="F27" s="18" t="n">
         <v>0.58</v>
@@ -11855,13 +11833,13 @@
         <v>16</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D28" s="10" t="s">
         <v>261</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="F28" s="18" t="n">
         <v>0.6</v>
@@ -11942,13 +11920,13 @@
         <v>16</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D29" s="10" t="s">
         <v>261</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="F29" s="18" t="n">
         <v>0.6</v>
@@ -12029,13 +12007,13 @@
         <v>17</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D30" s="10" t="s">
         <v>250</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="F30" s="18" t="n">
         <v>0.51</v>
@@ -12116,13 +12094,13 @@
         <v>17</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D31" s="10" t="s">
         <v>250</v>
       </c>
       <c r="E31" s="10" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="F31" s="18" t="n">
         <v>0.51</v>
@@ -12197,19 +12175,19 @@
     </row>
     <row r="32" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="10" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="B32" s="18" t="n">
         <v>18</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D32" s="10" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="F32" s="18" t="n">
         <v>0.35</v>
@@ -12284,19 +12262,19 @@
     </row>
     <row r="33" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="B33" s="18" t="n">
         <v>18</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D33" s="10" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="E33" s="10" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="F33" s="18" t="n">
         <v>0.35</v>
@@ -12371,19 +12349,19 @@
     </row>
     <row r="34" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="10" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="B34" s="18" t="n">
         <v>19</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D34" s="10" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="E34" s="10" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="F34" s="18" t="n">
         <v>0.42</v>
@@ -12458,19 +12436,19 @@
     </row>
     <row r="35" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="B35" s="18" t="n">
         <v>19</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D35" s="10" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="E35" s="10" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="F35" s="18" t="n">
         <v>0.42</v>
@@ -12551,13 +12529,13 @@
         <v>20</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="D36" s="10" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="E36" s="10" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="F36" s="18" t="n">
         <v>0.35</v>
@@ -12638,13 +12616,13 @@
         <v>20</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="D37" s="10" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="E37" s="10" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="F37" s="18" t="n">
         <v>0.35</v>
@@ -12725,13 +12703,13 @@
         <v>21</v>
       </c>
       <c r="C38" s="10" t="s">
+        <v>488</v>
+      </c>
+      <c r="D38" s="10" t="s">
+        <v>470</v>
+      </c>
+      <c r="E38" s="10" t="s">
         <v>490</v>
-      </c>
-      <c r="D38" s="10" t="s">
-        <v>472</v>
-      </c>
-      <c r="E38" s="10" t="s">
-        <v>492</v>
       </c>
       <c r="F38" s="18" t="n">
         <v>0.35</v>
@@ -12812,13 +12790,13 @@
         <v>21</v>
       </c>
       <c r="C39" s="10" t="s">
+        <v>488</v>
+      </c>
+      <c r="D39" s="10" t="s">
+        <v>470</v>
+      </c>
+      <c r="E39" s="10" t="s">
         <v>490</v>
-      </c>
-      <c r="D39" s="10" t="s">
-        <v>472</v>
-      </c>
-      <c r="E39" s="10" t="s">
-        <v>492</v>
       </c>
       <c r="F39" s="18" t="n">
         <v>0.35</v>
@@ -12899,13 +12877,13 @@
         <v>22</v>
       </c>
       <c r="C40" s="10" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="D40" s="10" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="E40" s="10" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="F40" s="18" t="n">
         <v>0.4</v>
@@ -12986,13 +12964,13 @@
         <v>22</v>
       </c>
       <c r="C41" s="10" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="D41" s="10" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="E41" s="10" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="F41" s="18" t="n">
         <v>0.4</v>
@@ -13067,19 +13045,19 @@
     </row>
     <row r="42" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="10" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="B42" s="18" t="n">
         <v>23</v>
       </c>
       <c r="C42" s="10" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="D42" s="10" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="E42" s="10" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="F42" s="18" t="n">
         <v>0.29</v>
@@ -13154,19 +13132,19 @@
     </row>
     <row r="43" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="10" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="B43" s="18" t="n">
         <v>24</v>
       </c>
       <c r="C43" s="10" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="D43" s="10" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="E43" s="10" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
       <c r="F43" s="18" t="n">
         <v>0.39</v>
@@ -13247,13 +13225,13 @@
         <v>26</v>
       </c>
       <c r="C44" s="10" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="D44" s="10" t="s">
         <v>261</v>
       </c>
       <c r="E44" s="10" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="F44" s="18" t="n">
         <v>0.6</v>
@@ -13334,13 +13312,13 @@
         <v>26</v>
       </c>
       <c r="C45" s="10" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="D45" s="10" t="s">
         <v>261</v>
       </c>
       <c r="E45" s="10" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="F45" s="18" t="n">
         <v>0.6</v>
@@ -13415,19 +13393,19 @@
     </row>
     <row r="46" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="10" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="B46" s="18" t="n">
         <v>27</v>
       </c>
       <c r="C46" s="10" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="D46" s="10" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="E46" s="10" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="F46" s="18" t="n">
         <v>0.42</v>
@@ -13502,19 +13480,19 @@
     </row>
     <row r="47" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="10" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="B47" s="18" t="n">
         <v>27</v>
       </c>
       <c r="C47" s="10" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="D47" s="10" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="E47" s="10" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="F47" s="18" t="n">
         <v>0.42</v>
@@ -13587,174 +13565,66 @@
       </c>
       <c r="AC47" s="18"/>
     </row>
-    <row r="48" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="13" t="s">
-        <v>339</v>
-      </c>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="10"/>
       <c r="B48" s="10"/>
-      <c r="C48" s="18" t="s">
-        <v>479</v>
-      </c>
-      <c r="D48" s="10" t="s">
-        <v>250</v>
-      </c>
-      <c r="E48" s="10" t="s">
-        <v>487</v>
-      </c>
-      <c r="F48" s="18" t="n">
-        <v>0.51</v>
-      </c>
-      <c r="G48" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="H48" s="18" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="I48" s="18" t="n">
-        <v>4</v>
-      </c>
-      <c r="J48" s="18" t="n">
-        <v>4</v>
-      </c>
-      <c r="K48" s="18" t="n">
-        <v>7.6</v>
-      </c>
-      <c r="L48" s="18" t="n">
-        <v>43.07</v>
-      </c>
-      <c r="M48" s="18" t="n">
-        <v>9.7</v>
-      </c>
-      <c r="N48" s="18" t="n">
-        <v>61.86</v>
-      </c>
-      <c r="O48" s="18" t="n">
-        <v>4.1</v>
-      </c>
-      <c r="P48" s="18" t="n">
-        <v>27.41</v>
-      </c>
-      <c r="Q48" s="18" t="n">
-        <v>8</v>
-      </c>
-      <c r="R48" s="18" t="n">
-        <v>48</v>
-      </c>
-      <c r="S48" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="T48" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="U48" s="18" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="V48" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="W48" s="18" t="n">
-        <v>27</v>
-      </c>
-      <c r="X48" s="18" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="Y48" s="18" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="Z48" s="18" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="AA48" s="18" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="AB48" s="18" t="n">
-        <v>0</v>
-      </c>
+      <c r="C48" s="18"/>
+      <c r="D48" s="10"/>
+      <c r="E48" s="10"/>
+      <c r="F48" s="10"/>
+      <c r="G48" s="18"/>
+      <c r="H48" s="18"/>
+      <c r="I48" s="18"/>
+      <c r="J48" s="18"/>
+      <c r="K48" s="18"/>
+      <c r="L48" s="18"/>
+      <c r="M48" s="18"/>
+      <c r="N48" s="18"/>
+      <c r="O48" s="18"/>
+      <c r="P48" s="18"/>
+      <c r="Q48" s="18"/>
+      <c r="R48" s="18"/>
+      <c r="S48" s="18"/>
+      <c r="T48" s="18"/>
+      <c r="U48" s="18"/>
+      <c r="V48" s="18"/>
+      <c r="W48" s="18"/>
+      <c r="X48" s="18"/>
+      <c r="Y48" s="18"/>
+      <c r="Z48" s="18"/>
+      <c r="AA48" s="18"/>
+      <c r="AB48" s="18"/>
       <c r="AC48" s="18"/>
     </row>
-    <row r="49" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="13" t="s">
-        <v>340</v>
-      </c>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="10"/>
       <c r="B49" s="10"/>
-      <c r="C49" s="18" t="s">
-        <v>496</v>
-      </c>
-      <c r="D49" s="10" t="s">
-        <v>261</v>
-      </c>
-      <c r="E49" s="10" t="s">
-        <v>486</v>
-      </c>
-      <c r="F49" s="18" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="G49" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="H49" s="18" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="I49" s="18" t="n">
-        <v>2</v>
-      </c>
-      <c r="J49" s="18" t="n">
-        <v>2</v>
-      </c>
-      <c r="K49" s="18" t="n">
-        <v>7.6</v>
-      </c>
-      <c r="L49" s="18" t="n">
-        <v>25.06</v>
-      </c>
-      <c r="M49" s="18" t="n">
-        <v>9.7</v>
-      </c>
-      <c r="N49" s="18" t="n">
-        <v>36.02</v>
-      </c>
-      <c r="O49" s="18" t="n">
-        <v>4.1</v>
-      </c>
-      <c r="P49" s="18" t="n">
-        <v>21.93</v>
-      </c>
-      <c r="Q49" s="18" t="n">
-        <v>8</v>
-      </c>
-      <c r="R49" s="18" t="n">
-        <v>48</v>
-      </c>
-      <c r="S49" s="18" t="n">
-        <v>19</v>
-      </c>
-      <c r="T49" s="18" t="n">
-        <v>5.301309524</v>
-      </c>
-      <c r="U49" s="18" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="V49" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="W49" s="18" t="n">
-        <v>27</v>
-      </c>
-      <c r="X49" s="18" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="Y49" s="18" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="Z49" s="18" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="AA49" s="18" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="AB49" s="18" t="n">
-        <v>0</v>
-      </c>
+      <c r="C49" s="18"/>
+      <c r="D49" s="10"/>
+      <c r="E49" s="10"/>
+      <c r="F49" s="10"/>
+      <c r="G49" s="18"/>
+      <c r="H49" s="18"/>
+      <c r="I49" s="18"/>
+      <c r="J49" s="18"/>
+      <c r="K49" s="18"/>
+      <c r="L49" s="18"/>
+      <c r="M49" s="18"/>
+      <c r="N49" s="18"/>
+      <c r="O49" s="18"/>
+      <c r="P49" s="18"/>
+      <c r="Q49" s="18"/>
+      <c r="R49" s="18"/>
+      <c r="S49" s="18"/>
+      <c r="T49" s="18"/>
+      <c r="U49" s="18"/>
+      <c r="V49" s="18"/>
+      <c r="W49" s="18"/>
+      <c r="X49" s="18"/>
+      <c r="Y49" s="18"/>
+      <c r="Z49" s="18"/>
+      <c r="AA49" s="18"/>
+      <c r="AB49" s="18"/>
       <c r="AC49" s="18"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14315,68 +14185,8 @@
       <c r="AB67" s="18"/>
       <c r="AC67" s="18"/>
     </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="10"/>
-      <c r="B68" s="10"/>
-      <c r="C68" s="18"/>
-      <c r="D68" s="10"/>
-      <c r="E68" s="10"/>
-      <c r="F68" s="10"/>
-      <c r="G68" s="18"/>
-      <c r="H68" s="18"/>
-      <c r="I68" s="18"/>
-      <c r="J68" s="18"/>
-      <c r="K68" s="18"/>
-      <c r="L68" s="18"/>
-      <c r="M68" s="18"/>
-      <c r="N68" s="18"/>
-      <c r="O68" s="18"/>
-      <c r="P68" s="18"/>
-      <c r="Q68" s="18"/>
-      <c r="R68" s="18"/>
-      <c r="S68" s="18"/>
-      <c r="T68" s="18"/>
-      <c r="U68" s="18"/>
-      <c r="V68" s="18"/>
-      <c r="W68" s="18"/>
-      <c r="X68" s="18"/>
-      <c r="Y68" s="18"/>
-      <c r="Z68" s="18"/>
-      <c r="AA68" s="18"/>
-      <c r="AB68" s="18"/>
-      <c r="AC68" s="18"/>
-    </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="10"/>
-      <c r="B69" s="10"/>
-      <c r="C69" s="18"/>
-      <c r="D69" s="10"/>
-      <c r="E69" s="10"/>
-      <c r="F69" s="10"/>
-      <c r="G69" s="18"/>
-      <c r="H69" s="18"/>
-      <c r="I69" s="18"/>
-      <c r="J69" s="18"/>
-      <c r="K69" s="18"/>
-      <c r="L69" s="18"/>
-      <c r="M69" s="18"/>
-      <c r="N69" s="18"/>
-      <c r="O69" s="18"/>
-      <c r="P69" s="18"/>
-      <c r="Q69" s="18"/>
-      <c r="R69" s="18"/>
-      <c r="S69" s="18"/>
-      <c r="T69" s="18"/>
-      <c r="U69" s="18"/>
-      <c r="V69" s="18"/>
-      <c r="W69" s="18"/>
-      <c r="X69" s="18"/>
-      <c r="Y69" s="18"/>
-      <c r="Z69" s="18"/>
-      <c r="AA69" s="18"/>
-      <c r="AB69" s="18"/>
-      <c r="AC69" s="18"/>
-    </row>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
refactor(tests+thermal): clean up unused mappings and constants, streamline thermal type filtering logic (delete dropna filter on key) (#28)
</commit_message>
<xml_diff>
--- a/tests/antares/resources/MAIN_PARAMS_2025.xlsx
+++ b/tests/antares/resources/MAIN_PARAMS_2025.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1529" uniqueCount="566">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1517" uniqueCount="564">
   <si>
     <t xml:space="preserve">dossier PEMMDB</t>
   </si>
@@ -1052,12 +1052,6 @@
   </si>
   <si>
     <t xml:space="preserve">Lignite old 2 CHP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gas pcomp CCS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gas pcomp H2</t>
   </si>
   <si>
     <t xml:space="preserve">Nuclear/-</t>
@@ -1971,10 +1965,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1984,6 +1974,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2118,9 +2112,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
-      <xdr:colOff>109440</xdr:colOff>
+      <xdr:colOff>109080</xdr:colOff>
       <xdr:row>10</xdr:row>
-      <xdr:rowOff>127440</xdr:rowOff>
+      <xdr:rowOff>127080</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -2129,8 +2123,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7523640" y="952560"/>
-          <a:ext cx="7632720" cy="1080000"/>
+          <a:off x="7528680" y="952560"/>
+          <a:ext cx="7637400" cy="1079640"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2230,9 +2224,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
-      <xdr:colOff>311040</xdr:colOff>
+      <xdr:colOff>310680</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>176040</xdr:rowOff>
+      <xdr:rowOff>175680</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -2241,8 +2235,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="11264040" y="429480"/>
-          <a:ext cx="8258400" cy="1080000"/>
+          <a:off x="11264760" y="429480"/>
+          <a:ext cx="8263440" cy="1079640"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2333,9 +2327,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>243000</xdr:colOff>
+      <xdr:colOff>242640</xdr:colOff>
       <xdr:row>26</xdr:row>
-      <xdr:rowOff>49320</xdr:rowOff>
+      <xdr:rowOff>48960</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -2344,8 +2338,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13868640" y="560160"/>
-          <a:ext cx="6840360" cy="4400280"/>
+          <a:off x="13867920" y="560160"/>
+          <a:ext cx="6843240" cy="4399920"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2778,9 +2772,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>550800</xdr:colOff>
+      <xdr:colOff>550440</xdr:colOff>
       <xdr:row>25</xdr:row>
-      <xdr:rowOff>111960</xdr:rowOff>
+      <xdr:rowOff>111600</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -2789,8 +2783,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13863600" y="771480"/>
-          <a:ext cx="7153200" cy="4061160"/>
+          <a:off x="13862880" y="771480"/>
+          <a:ext cx="7156080" cy="4060800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3232,9 +3226,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>318600</xdr:colOff>
+      <xdr:colOff>318240</xdr:colOff>
       <xdr:row>17</xdr:row>
-      <xdr:rowOff>128160</xdr:rowOff>
+      <xdr:rowOff>127800</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -3244,7 +3238,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="6582240" y="409320"/>
-          <a:ext cx="10342080" cy="2957400"/>
+          <a:ext cx="10347480" cy="2957040"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3558,7 +3552,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B25"/>
-  <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.5859375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="65.43"/>
@@ -3632,7 +3626,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D27"/>
-  <sheetFormatPr defaultColWidth="10.8671875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="8" width="10.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.57"/>
@@ -3648,152 +3642,152 @@
         <v>247</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="20" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="20" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="20" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="20" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="20" t="s">
+        <v>378</v>
+      </c>
+      <c r="B6" s="0" t="s">
         <v>380</v>
       </c>
-      <c r="B6" s="0" t="s">
-        <v>382</v>
-      </c>
       <c r="C6" s="0" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="20" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="C7" s="0" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="20" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="20" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="20" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="C10" s="0" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="B11" s="0" t="s">
+        <v>515</v>
+      </c>
+      <c r="C11" s="0" t="s">
+        <v>516</v>
+      </c>
+      <c r="D11" s="0" t="s">
         <v>517</v>
-      </c>
-      <c r="C11" s="0" t="s">
-        <v>518</v>
-      </c>
-      <c r="D11" s="0" t="s">
-        <v>519</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="20" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="B12" s="0" t="s">
+        <v>518</v>
+      </c>
+      <c r="C12" s="0" t="s">
+        <v>519</v>
+      </c>
+      <c r="D12" s="0" t="s">
         <v>520</v>
-      </c>
-      <c r="C12" s="0" t="s">
-        <v>521</v>
-      </c>
-      <c r="D12" s="0" t="s">
-        <v>522</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3863,7 +3857,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C71"/>
-  <sheetFormatPr defaultColWidth="10.8671875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="31"/>
@@ -3886,10 +3880,10 @@
         <v>15</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3897,10 +3891,10 @@
         <v>15</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3908,10 +3902,10 @@
         <v>15</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3919,10 +3913,10 @@
         <v>15</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3930,10 +3924,10 @@
         <v>15</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="C6" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3944,7 +3938,7 @@
         <v>331</v>
       </c>
       <c r="C7" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3955,7 +3949,7 @@
         <v>336</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3966,7 +3960,7 @@
         <v>326</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3974,10 +3968,10 @@
         <v>15</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
       <c r="C10" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3988,7 +3982,7 @@
         <v>288</v>
       </c>
       <c r="C11" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3999,7 +3993,7 @@
         <v>294</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4010,7 +4004,7 @@
         <v>278</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4021,7 +4015,7 @@
         <v>282</v>
       </c>
       <c r="C14" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4032,7 +4026,7 @@
         <v>266</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4043,7 +4037,7 @@
         <v>272</v>
       </c>
       <c r="C16" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4054,7 +4048,7 @@
         <v>261</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4065,7 +4059,7 @@
         <v>250</v>
       </c>
       <c r="C18" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4073,10 +4067,10 @@
         <v>15</v>
       </c>
       <c r="B19" s="0" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="C19" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4084,10 +4078,10 @@
         <v>15</v>
       </c>
       <c r="B20" s="0" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="C20" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4098,7 +4092,7 @@
         <v>321</v>
       </c>
       <c r="C21" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4109,7 +4103,7 @@
         <v>313</v>
       </c>
       <c r="C22" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4120,7 +4114,7 @@
         <v>317</v>
       </c>
       <c r="C23" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4128,10 +4122,10 @@
         <v>15</v>
       </c>
       <c r="B24" s="0" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="C24" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4139,10 +4133,10 @@
         <v>15</v>
       </c>
       <c r="B25" s="0" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="C25" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4150,10 +4144,10 @@
         <v>15</v>
       </c>
       <c r="B26" s="0" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="C26" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4161,10 +4155,10 @@
         <v>15</v>
       </c>
       <c r="B27" s="0" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="C27" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4172,10 +4166,10 @@
         <v>15</v>
       </c>
       <c r="B28" s="0" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="C28" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4183,10 +4177,10 @@
         <v>15</v>
       </c>
       <c r="B29" s="0" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="C29" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4194,10 +4188,10 @@
         <v>15</v>
       </c>
       <c r="B30" s="0" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="C30" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4205,10 +4199,10 @@
         <v>15</v>
       </c>
       <c r="B31" s="0" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="C31" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4216,10 +4210,10 @@
         <v>15</v>
       </c>
       <c r="B32" s="0" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="C32" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4227,10 +4221,10 @@
         <v>15</v>
       </c>
       <c r="B33" s="0" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="C33" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4238,10 +4232,10 @@
         <v>15</v>
       </c>
       <c r="B34" s="0" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="C34" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4249,10 +4243,10 @@
         <v>15</v>
       </c>
       <c r="B35" s="0" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="C35" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4260,10 +4254,10 @@
         <v>15</v>
       </c>
       <c r="B36" s="0" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="C36" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4271,10 +4265,10 @@
         <v>15</v>
       </c>
       <c r="B37" s="0" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="C37" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4282,10 +4276,10 @@
         <v>15</v>
       </c>
       <c r="B38" s="0" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="C38" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4293,10 +4287,10 @@
         <v>15</v>
       </c>
       <c r="B39" s="0" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="C39" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4304,10 +4298,10 @@
         <v>15</v>
       </c>
       <c r="B40" s="0" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="C40" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4315,10 +4309,10 @@
         <v>15</v>
       </c>
       <c r="B41" s="11" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="C41" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4326,10 +4320,10 @@
         <v>15</v>
       </c>
       <c r="B42" s="10" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="C42" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4337,10 +4331,10 @@
         <v>15</v>
       </c>
       <c r="B43" s="11" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="C43" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4348,10 +4342,10 @@
         <v>15</v>
       </c>
       <c r="B44" s="0" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="C44" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4359,10 +4353,10 @@
         <v>15</v>
       </c>
       <c r="B45" s="0" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="C45" s="0" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4370,10 +4364,10 @@
         <v>15</v>
       </c>
       <c r="B46" s="0" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="C46" s="0" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4381,10 +4375,10 @@
         <v>15</v>
       </c>
       <c r="B47" s="0" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="C47" s="0" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4392,10 +4386,10 @@
         <v>15</v>
       </c>
       <c r="B48" s="0" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="C48" s="0" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4403,10 +4397,10 @@
         <v>15</v>
       </c>
       <c r="B49" s="0" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="C49" s="0" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4414,10 +4408,10 @@
         <v>15</v>
       </c>
       <c r="B50" s="0" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="C50" s="0" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4425,10 +4419,10 @@
         <v>15</v>
       </c>
       <c r="B51" s="0" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="C51" s="0" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4436,10 +4430,10 @@
         <v>15</v>
       </c>
       <c r="B52" s="0" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="C52" s="0" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4447,10 +4441,10 @@
         <v>15</v>
       </c>
       <c r="B53" s="0" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
       <c r="C53" s="0" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4458,10 +4452,10 @@
         <v>15</v>
       </c>
       <c r="B54" s="0" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
       <c r="C54" s="0" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4469,10 +4463,10 @@
         <v>15</v>
       </c>
       <c r="B55" s="0" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
       <c r="C55" s="0" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4480,10 +4474,10 @@
         <v>15</v>
       </c>
       <c r="B56" s="0" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="C56" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4491,10 +4485,10 @@
         <v>15</v>
       </c>
       <c r="B57" s="0" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
       <c r="C57" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4502,10 +4496,10 @@
         <v>15</v>
       </c>
       <c r="B58" s="0" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
       <c r="C58" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4513,10 +4507,10 @@
         <v>15</v>
       </c>
       <c r="B59" s="0" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="C59" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4524,10 +4518,10 @@
         <v>15</v>
       </c>
       <c r="B60" s="0" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="C60" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4535,10 +4529,10 @@
         <v>15</v>
       </c>
       <c r="B61" s="0" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
       <c r="C61" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4546,10 +4540,10 @@
         <v>15</v>
       </c>
       <c r="B62" s="0" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
       <c r="C62" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4557,10 +4551,10 @@
         <v>15</v>
       </c>
       <c r="B63" s="0" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
       <c r="C63" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4568,10 +4562,10 @@
         <v>15</v>
       </c>
       <c r="B64" s="0" t="s">
-        <v>548</v>
+        <v>546</v>
       </c>
       <c r="C64" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4579,10 +4573,10 @@
         <v>15</v>
       </c>
       <c r="B65" s="0" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
       <c r="C65" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4590,10 +4584,10 @@
         <v>15</v>
       </c>
       <c r="B66" s="0" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="C66" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4601,10 +4595,10 @@
         <v>15</v>
       </c>
       <c r="B67" s="0" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
       <c r="C67" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4612,10 +4606,10 @@
         <v>15</v>
       </c>
       <c r="B68" s="0" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
       <c r="C68" s="0" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4623,10 +4617,10 @@
         <v>15</v>
       </c>
       <c r="B69" s="0" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
       <c r="C69" s="0" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="60" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4634,10 +4628,10 @@
         <v>15</v>
       </c>
       <c r="B70" s="21" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
       <c r="C70" s="10" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="60" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4645,10 +4639,10 @@
         <v>15</v>
       </c>
       <c r="B71" s="21" t="s">
+        <v>553</v>
+      </c>
+      <c r="C71" s="10" t="s">
         <v>555</v>
-      </c>
-      <c r="C71" s="10" t="s">
-        <v>557</v>
       </c>
     </row>
   </sheetData>
@@ -4669,20 +4663,20 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D25"/>
-  <sheetFormatPr defaultColWidth="9.15234375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.16015625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="22" t="s">
+        <v>556</v>
+      </c>
+      <c r="B1" s="22" t="s">
+        <v>557</v>
+      </c>
+      <c r="C1" s="22" t="s">
         <v>558</v>
       </c>
-      <c r="B1" s="22" t="s">
+      <c r="D1" s="22" t="s">
         <v>559</v>
-      </c>
-      <c r="C1" s="22" t="s">
-        <v>560</v>
-      </c>
-      <c r="D1" s="22" t="s">
-        <v>561</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4690,13 +4684,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="23" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="C2" s="23" t="n">
         <v>1</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4704,13 +4698,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="23" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="C3" s="23" t="n">
         <v>2</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4718,13 +4712,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="23" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="C4" s="23" t="n">
         <v>3</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4732,13 +4726,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="C5" s="23" t="n">
         <v>4</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4746,13 +4740,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="C6" s="23" t="n">
         <v>5</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4760,13 +4754,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="C7" s="23" t="n">
         <v>6</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4774,13 +4768,13 @@
         <v>7</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="C8" s="23" t="n">
         <v>7</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4788,13 +4782,13 @@
         <v>8</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="C9" s="23" t="n">
         <v>8</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4802,13 +4796,13 @@
         <v>9</v>
       </c>
       <c r="B10" s="23" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="C10" s="23" t="n">
         <v>9</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4816,13 +4810,13 @@
         <v>10</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="C11" s="23" t="n">
         <v>10</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4830,13 +4824,13 @@
         <v>11</v>
       </c>
       <c r="B12" s="23" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="C12" s="23" t="n">
         <v>11</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4844,13 +4838,13 @@
         <v>12</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="C13" s="23" t="n">
         <v>12</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4858,7 +4852,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="23" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="C14" s="23"/>
       <c r="D14" s="23"/>
@@ -4868,7 +4862,7 @@
         <v>14</v>
       </c>
       <c r="B15" s="23" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="C15" s="23"/>
       <c r="D15" s="23"/>
@@ -4878,7 +4872,7 @@
         <v>15</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="C16" s="23"/>
       <c r="D16" s="23"/>
@@ -4888,7 +4882,7 @@
         <v>16</v>
       </c>
       <c r="B17" s="23" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="C17" s="23"/>
       <c r="D17" s="23"/>
@@ -4898,7 +4892,7 @@
         <v>17</v>
       </c>
       <c r="B18" s="23" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="C18" s="23"/>
       <c r="D18" s="23"/>
@@ -4908,7 +4902,7 @@
         <v>18</v>
       </c>
       <c r="B19" s="23" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="C19" s="23"/>
       <c r="D19" s="23"/>
@@ -4918,7 +4912,7 @@
         <v>19</v>
       </c>
       <c r="B20" s="23" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="C20" s="23"/>
       <c r="D20" s="23"/>
@@ -4928,7 +4922,7 @@
         <v>20</v>
       </c>
       <c r="B21" s="23" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="C21" s="23"/>
       <c r="D21" s="23"/>
@@ -4938,7 +4932,7 @@
         <v>21</v>
       </c>
       <c r="B22" s="23" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="C22" s="23"/>
       <c r="D22" s="23"/>
@@ -4948,7 +4942,7 @@
         <v>22</v>
       </c>
       <c r="B23" s="23" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="C23" s="23"/>
       <c r="D23" s="23"/>
@@ -4958,7 +4952,7 @@
         <v>23</v>
       </c>
       <c r="B24" s="23" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="C24" s="23"/>
       <c r="D24" s="23"/>
@@ -4968,7 +4962,7 @@
         <v>24</v>
       </c>
       <c r="B25" s="23" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="C25" s="23"/>
       <c r="D25" s="23"/>
@@ -4990,7 +4984,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E107"/>
-  <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.5859375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="7" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="34.43"/>
@@ -6726,7 +6720,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B43"/>
-  <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.5859375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
@@ -7126,7 +7120,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B60"/>
-  <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.5859375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="8" width="17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.43"/>
@@ -7628,8 +7622,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C91"/>
-  <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:C1048576"/>
+  <sheetFormatPr defaultColWidth="10.5859375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="8" width="10.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="8" width="69.43"/>
@@ -8245,18 +8239,22 @@
       <c r="A56" s="12" t="s">
         <v>248</v>
       </c>
-      <c r="B56" s="12"/>
-      <c r="C56" s="13" t="s">
+      <c r="B56" s="12" t="s">
         <v>339</v>
+      </c>
+      <c r="C56" s="12" t="s">
+        <v>340</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="12" t="s">
         <v>248</v>
       </c>
-      <c r="B57" s="12"/>
-      <c r="C57" s="13" t="s">
-        <v>340</v>
+      <c r="B57" s="12" t="s">
+        <v>341</v>
+      </c>
+      <c r="C57" s="12" t="s">
+        <v>342</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8264,10 +8262,10 @@
         <v>248</v>
       </c>
       <c r="B58" s="12" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="C58" s="12" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8275,10 +8273,10 @@
         <v>248</v>
       </c>
       <c r="B59" s="12" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="C59" s="12" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8286,7 +8284,7 @@
         <v>248</v>
       </c>
       <c r="B60" s="12" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="C60" s="12" t="s">
         <v>346</v>
@@ -8297,10 +8295,10 @@
         <v>248</v>
       </c>
       <c r="B61" s="12" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="C61" s="12" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8308,10 +8306,10 @@
         <v>248</v>
       </c>
       <c r="B62" s="12" t="s">
+        <v>350</v>
+      </c>
+      <c r="C62" s="12" t="s">
         <v>349</v>
-      </c>
-      <c r="C62" s="12" t="s">
-        <v>348</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8319,10 +8317,10 @@
         <v>248</v>
       </c>
       <c r="B63" s="12" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="C63" s="12" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8330,10 +8328,10 @@
         <v>248</v>
       </c>
       <c r="B64" s="12" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C64" s="12" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8341,7 +8339,7 @@
         <v>248</v>
       </c>
       <c r="B65" s="12" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="C65" s="12" t="s">
         <v>354</v>
@@ -8352,10 +8350,10 @@
         <v>248</v>
       </c>
       <c r="B66" s="12" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="C66" s="12" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8363,10 +8361,10 @@
         <v>248</v>
       </c>
       <c r="B67" s="12" t="s">
+        <v>358</v>
+      </c>
+      <c r="C67" s="12" t="s">
         <v>357</v>
-      </c>
-      <c r="C67" s="12" t="s">
-        <v>356</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8374,10 +8372,10 @@
         <v>248</v>
       </c>
       <c r="B68" s="12" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="C68" s="12" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8385,10 +8383,10 @@
         <v>248</v>
       </c>
       <c r="B69" s="12" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="C69" s="12" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8396,7 +8394,7 @@
         <v>248</v>
       </c>
       <c r="B70" s="12" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="C70" s="12" t="s">
         <v>362</v>
@@ -8404,32 +8402,32 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="12" t="s">
-        <v>248</v>
+        <v>364</v>
       </c>
       <c r="B71" s="12" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C71" s="12" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="12" t="s">
-        <v>248</v>
+        <v>364</v>
       </c>
       <c r="B72" s="12" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="C72" s="12" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="12" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B73" s="12" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="C73" s="12" t="s">
         <v>368</v>
@@ -8437,153 +8435,153 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="12" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B74" s="12" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="C74" s="12" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="12" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B75" s="12" t="s">
+        <v>372</v>
+      </c>
+      <c r="C75" s="12" t="s">
         <v>371</v>
-      </c>
-      <c r="C75" s="12" t="s">
-        <v>370</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="12" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B76" s="12" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C76" s="12" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="12" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B77" s="12" t="s">
+        <v>375</v>
+      </c>
+      <c r="C77" s="12" t="s">
         <v>374</v>
-      </c>
-      <c r="C77" s="12" t="s">
-        <v>373</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="12" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B78" s="12" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C78" s="12" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="12" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="B79" s="12" t="s">
         <v>377</v>
       </c>
       <c r="C79" s="12" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="12" t="s">
-        <v>366</v>
+        <v>378</v>
       </c>
       <c r="B80" s="12" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C80" s="12" t="s">
-        <v>376</v>
+        <v>380</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="12" t="s">
-        <v>366</v>
+        <v>378</v>
       </c>
       <c r="B81" s="12" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="C81" s="12" t="s">
-        <v>376</v>
+        <v>382</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="12" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="B82" s="12" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="C82" s="12" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="12" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="B83" s="12" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="C83" s="12" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="12" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="B84" s="12" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="C84" s="12" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="12" t="s">
-        <v>380</v>
+        <v>389</v>
       </c>
       <c r="B85" s="12" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="C85" s="12" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="12" t="s">
-        <v>380</v>
+        <v>389</v>
       </c>
       <c r="B86" s="12" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="C86" s="12" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="12" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="B87" s="12" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="C87" s="12" t="s">
         <v>393</v>
@@ -8591,48 +8589,28 @@
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="12" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="B88" s="12" t="s">
         <v>394</v>
       </c>
       <c r="C88" s="12" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="12" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="B89" s="12" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="C89" s="12" t="s">
-        <v>395</v>
-      </c>
-    </row>
-    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="12" t="s">
-        <v>391</v>
-      </c>
-      <c r="B90" s="12" t="s">
-        <v>396</v>
-      </c>
-      <c r="C90" s="12" t="s">
         <v>397</v>
       </c>
     </row>
-    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="12" t="s">
-        <v>391</v>
-      </c>
-      <c r="B91" s="12" t="s">
-        <v>398</v>
-      </c>
-      <c r="C91" s="12" t="s">
-        <v>399</v>
-      </c>
-    </row>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <autoFilter ref="A1:C1"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -8652,7 +8630,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C20"/>
-  <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.5859375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="11" width="18"/>
@@ -8668,7 +8646,7 @@
         <v>247</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8679,7 +8657,7 @@
         <v>266</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8690,7 +8668,7 @@
         <v>269</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8701,7 +8679,7 @@
         <v>269</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8712,7 +8690,7 @@
         <v>280</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8723,7 +8701,7 @@
         <v>300</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8734,7 +8712,7 @@
         <v>302</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8745,7 +8723,7 @@
         <v>304</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8756,7 +8734,7 @@
         <v>307</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8767,7 +8745,7 @@
         <v>307</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8778,7 +8756,7 @@
         <v>309</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8789,7 +8767,7 @@
         <v>311</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8800,7 +8778,7 @@
         <v>329</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8811,7 +8789,7 @@
         <v>331</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8822,7 +8800,7 @@
         <v>333</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8833,7 +8811,7 @@
         <v>333</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8844,40 +8822,40 @@
         <v>336</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
     </row>
   </sheetData>
@@ -8897,7 +8875,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I10"/>
-  <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.5859375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="11" width="21.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="36.7"/>
@@ -8909,79 +8887,79 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="13" t="s">
+        <v>415</v>
+      </c>
+      <c r="B1" s="14" t="s">
+        <v>416</v>
+      </c>
+      <c r="C1" s="14" t="s">
         <v>417</v>
       </c>
-      <c r="B1" s="15" t="s">
+      <c r="D1" s="15" t="s">
         <v>418</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="E1" s="15" t="s">
         <v>419</v>
       </c>
-      <c r="D1" s="16" t="s">
+      <c r="F1" s="15" t="s">
         <v>420</v>
-      </c>
-      <c r="E1" s="16" t="s">
-        <v>421</v>
-      </c>
-      <c r="F1" s="16" t="s">
-        <v>422</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
+        <v>421</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>422</v>
+      </c>
+      <c r="C2" s="11" t="s">
         <v>423</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="D2" s="11" t="s">
         <v>424</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="E2" s="11" t="s">
         <v>425</v>
       </c>
-      <c r="D2" s="11" t="s">
+      <c r="F2" s="11" t="s">
         <v>426</v>
-      </c>
-      <c r="E2" s="11" t="s">
-        <v>427</v>
-      </c>
-      <c r="F2" s="11" t="s">
-        <v>428</v>
       </c>
       <c r="I2" s="11"/>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="11" t="s">
+        <v>427</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>428</v>
+      </c>
+      <c r="C3" s="11" t="s">
         <v>429</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="D3" s="11" t="s">
         <v>430</v>
       </c>
-      <c r="C3" s="11" t="s">
+      <c r="E3" s="11" t="s">
         <v>431</v>
-      </c>
-      <c r="D3" s="11" t="s">
-        <v>432</v>
-      </c>
-      <c r="E3" s="11" t="s">
-        <v>433</v>
       </c>
       <c r="F3" s="11"/>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="C4" s="11" t="s">
+        <v>423</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>424</v>
+      </c>
+      <c r="E4" s="11" t="s">
         <v>425</v>
-      </c>
-      <c r="D4" s="11" t="s">
-        <v>426</v>
-      </c>
-      <c r="E4" s="11" t="s">
-        <v>427</v>
       </c>
       <c r="F4" s="11" t="s">
         <v>245</v>
@@ -8989,19 +8967,19 @@
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="B5" s="11" t="s">
+        <v>428</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>429</v>
+      </c>
+      <c r="D5" s="11" t="s">
         <v>430</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="E5" s="11" t="s">
         <v>431</v>
-      </c>
-      <c r="D5" s="11" t="s">
-        <v>432</v>
-      </c>
-      <c r="E5" s="11" t="s">
-        <v>433</v>
       </c>
       <c r="F5" s="11"/>
     </row>
@@ -9026,7 +9004,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E80"/>
-  <sheetFormatPr defaultColWidth="8.58203125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5859375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="19.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="22.57"/>
@@ -9036,28 +9014,28 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>437</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>438</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>439</v>
       </c>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="13"/>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
+      <c r="A2" s="16"/>
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
       <c r="D2" s="11"/>
       <c r="E2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="13"/>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
+      <c r="A3" s="16"/>
+      <c r="B3" s="16"/>
+      <c r="C3" s="16"/>
       <c r="D3" s="11"/>
       <c r="E3" s="11"/>
     </row>
@@ -9490,8 +9468,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AC69"/>
-  <sheetFormatPr defaultColWidth="9.15234375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:AC1048576"/>
+  <sheetFormatPr defaultColWidth="9.16015625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19"/>
@@ -9500,106 +9478,106 @@
   <sheetData>
     <row r="1" customFormat="false" ht="60" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
+        <v>438</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>439</v>
+      </c>
+      <c r="C1" s="9" t="s">
         <v>440</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="D1" s="9" t="s">
         <v>441</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="E1" s="9" t="s">
         <v>442</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="F1" s="9" t="s">
         <v>443</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="G1" s="9" t="s">
         <v>444</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="H1" s="9" t="s">
         <v>445</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="I1" s="9" t="s">
         <v>446</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="J1" s="9" t="s">
         <v>447</v>
       </c>
-      <c r="I1" s="9" t="s">
+      <c r="K1" s="9" t="s">
         <v>448</v>
       </c>
-      <c r="J1" s="9" t="s">
+      <c r="L1" s="9" t="s">
         <v>449</v>
       </c>
-      <c r="K1" s="9" t="s">
+      <c r="M1" s="9" t="s">
         <v>450</v>
       </c>
-      <c r="L1" s="9" t="s">
+      <c r="N1" s="9" t="s">
         <v>451</v>
       </c>
-      <c r="M1" s="9" t="s">
+      <c r="O1" s="9" t="s">
         <v>452</v>
       </c>
-      <c r="N1" s="9" t="s">
+      <c r="P1" s="9" t="s">
         <v>453</v>
       </c>
-      <c r="O1" s="9" t="s">
+      <c r="Q1" s="9" t="s">
         <v>454</v>
       </c>
-      <c r="P1" s="9" t="s">
+      <c r="R1" s="9" t="s">
         <v>455</v>
       </c>
-      <c r="Q1" s="9" t="s">
+      <c r="S1" s="9" t="s">
         <v>456</v>
       </c>
-      <c r="R1" s="9" t="s">
+      <c r="T1" s="9" t="s">
         <v>457</v>
       </c>
-      <c r="S1" s="9" t="s">
+      <c r="U1" s="9" t="s">
         <v>458</v>
       </c>
-      <c r="T1" s="9" t="s">
+      <c r="V1" s="9" t="s">
         <v>459</v>
       </c>
-      <c r="U1" s="9" t="s">
+      <c r="W1" s="9" t="s">
         <v>460</v>
       </c>
-      <c r="V1" s="9" t="s">
+      <c r="X1" s="9" t="s">
         <v>461</v>
       </c>
-      <c r="W1" s="9" t="s">
+      <c r="Y1" s="9" t="s">
         <v>462</v>
       </c>
-      <c r="X1" s="9" t="s">
+      <c r="Z1" s="9" t="s">
         <v>463</v>
       </c>
-      <c r="Y1" s="9" t="s">
+      <c r="AA1" s="9" t="s">
         <v>464</v>
       </c>
-      <c r="Z1" s="9" t="s">
+      <c r="AB1" s="9" t="s">
         <v>465</v>
-      </c>
-      <c r="AA1" s="9" t="s">
-        <v>466</v>
-      </c>
-      <c r="AB1" s="9" t="s">
-        <v>467</v>
       </c>
       <c r="AC1" s="9"/>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="B2" s="18" t="n">
         <v>1</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="F2" s="18" t="n">
         <v>0.33</v>
@@ -9674,19 +9652,19 @@
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="B3" s="18" t="n">
         <v>1</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="F3" s="18" t="n">
         <v>0.33</v>
@@ -9767,13 +9745,13 @@
         <v>2</v>
       </c>
       <c r="C4" s="10" t="s">
+        <v>469</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>470</v>
+      </c>
+      <c r="E4" s="10" t="s">
         <v>471</v>
-      </c>
-      <c r="D4" s="10" t="s">
-        <v>472</v>
-      </c>
-      <c r="E4" s="10" t="s">
-        <v>473</v>
       </c>
       <c r="F4" s="18" t="n">
         <v>0.35</v>
@@ -9854,13 +9832,13 @@
         <v>2</v>
       </c>
       <c r="C5" s="10" t="s">
+        <v>469</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>470</v>
+      </c>
+      <c r="E5" s="10" t="s">
         <v>471</v>
-      </c>
-      <c r="D5" s="10" t="s">
-        <v>472</v>
-      </c>
-      <c r="E5" s="10" t="s">
-        <v>473</v>
       </c>
       <c r="F5" s="18" t="n">
         <v>0.35</v>
@@ -9941,13 +9919,13 @@
         <v>3</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="F6" s="18" t="n">
         <v>0.4</v>
@@ -10028,13 +10006,13 @@
         <v>3</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="F7" s="18" t="n">
         <v>0.4</v>
@@ -10115,13 +10093,13 @@
         <v>4</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="F8" s="18" t="n">
         <v>0.46</v>
@@ -10202,13 +10180,13 @@
         <v>4</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="F9" s="18" t="n">
         <v>0.46</v>
@@ -10289,13 +10267,13 @@
         <v>6</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="F10" s="18" t="n">
         <v>0.35</v>
@@ -10376,13 +10354,13 @@
         <v>6</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="F11" s="18" t="n">
         <v>0.35</v>
@@ -10463,13 +10441,13 @@
         <v>7</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="F12" s="18" t="n">
         <v>0.4</v>
@@ -10550,13 +10528,13 @@
         <v>7</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="F13" s="18" t="n">
         <v>0.4</v>
@@ -10637,13 +10615,13 @@
         <v>8</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="F14" s="18" t="n">
         <v>0.46</v>
@@ -10724,13 +10702,13 @@
         <v>8</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="F15" s="18" t="n">
         <v>0.46</v>
@@ -10811,13 +10789,13 @@
         <v>10</v>
       </c>
       <c r="C16" s="10" t="s">
+        <v>477</v>
+      </c>
+      <c r="D16" s="10" t="s">
+        <v>478</v>
+      </c>
+      <c r="E16" s="10" t="s">
         <v>479</v>
-      </c>
-      <c r="D16" s="10" t="s">
-        <v>480</v>
-      </c>
-      <c r="E16" s="10" t="s">
-        <v>481</v>
       </c>
       <c r="F16" s="18" t="n">
         <v>0.36</v>
@@ -10898,13 +10876,13 @@
         <v>10</v>
       </c>
       <c r="C17" s="10" t="s">
+        <v>477</v>
+      </c>
+      <c r="D17" s="10" t="s">
+        <v>478</v>
+      </c>
+      <c r="E17" s="10" t="s">
         <v>479</v>
-      </c>
-      <c r="D17" s="10" t="s">
-        <v>480</v>
-      </c>
-      <c r="E17" s="10" t="s">
-        <v>481</v>
       </c>
       <c r="F17" s="18" t="n">
         <v>0.36</v>
@@ -10985,13 +10963,13 @@
         <v>11</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="F18" s="18" t="n">
         <v>0.41</v>
@@ -11072,13 +11050,13 @@
         <v>11</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="F19" s="18" t="n">
         <v>0.41</v>
@@ -11159,13 +11137,13 @@
         <v>12</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D20" s="10" t="s">
         <v>266</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="F20" s="18" t="n">
         <v>0.4</v>
@@ -11246,13 +11224,13 @@
         <v>12</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D21" s="10" t="s">
         <v>266</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="F21" s="18" t="n">
         <v>0.4</v>
@@ -11333,13 +11311,13 @@
         <v>13</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D22" s="10" t="s">
         <v>272</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="F22" s="18" t="n">
         <v>0.48</v>
@@ -11420,13 +11398,13 @@
         <v>13</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D23" s="10" t="s">
         <v>272</v>
       </c>
       <c r="E23" s="10" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="F23" s="18" t="n">
         <v>0.48</v>
@@ -11507,13 +11485,13 @@
         <v>14</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D24" s="10" t="s">
         <v>278</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="F24" s="18" t="n">
         <v>0.56</v>
@@ -11594,13 +11572,13 @@
         <v>14</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D25" s="10" t="s">
         <v>278</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="F25" s="18" t="n">
         <v>0.56</v>
@@ -11681,13 +11659,13 @@
         <v>15</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D26" s="10" t="s">
         <v>282</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="F26" s="18" t="n">
         <v>0.58</v>
@@ -11768,13 +11746,13 @@
         <v>15</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D27" s="10" t="s">
         <v>282</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="F27" s="18" t="n">
         <v>0.58</v>
@@ -11855,13 +11833,13 @@
         <v>16</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D28" s="10" t="s">
         <v>261</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="F28" s="18" t="n">
         <v>0.6</v>
@@ -11942,13 +11920,13 @@
         <v>16</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D29" s="10" t="s">
         <v>261</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="F29" s="18" t="n">
         <v>0.6</v>
@@ -12029,13 +12007,13 @@
         <v>17</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D30" s="10" t="s">
         <v>250</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="F30" s="18" t="n">
         <v>0.51</v>
@@ -12116,13 +12094,13 @@
         <v>17</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D31" s="10" t="s">
         <v>250</v>
       </c>
       <c r="E31" s="10" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="F31" s="18" t="n">
         <v>0.51</v>
@@ -12197,19 +12175,19 @@
     </row>
     <row r="32" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="10" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="B32" s="18" t="n">
         <v>18</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D32" s="10" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="F32" s="18" t="n">
         <v>0.35</v>
@@ -12284,19 +12262,19 @@
     </row>
     <row r="33" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="B33" s="18" t="n">
         <v>18</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D33" s="10" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="E33" s="10" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="F33" s="18" t="n">
         <v>0.35</v>
@@ -12371,19 +12349,19 @@
     </row>
     <row r="34" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="10" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="B34" s="18" t="n">
         <v>19</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D34" s="10" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="E34" s="10" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="F34" s="18" t="n">
         <v>0.42</v>
@@ -12458,19 +12436,19 @@
     </row>
     <row r="35" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="B35" s="18" t="n">
         <v>19</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="D35" s="10" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="E35" s="10" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="F35" s="18" t="n">
         <v>0.42</v>
@@ -12551,13 +12529,13 @@
         <v>20</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="D36" s="10" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="E36" s="10" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="F36" s="18" t="n">
         <v>0.35</v>
@@ -12638,13 +12616,13 @@
         <v>20</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="D37" s="10" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="E37" s="10" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="F37" s="18" t="n">
         <v>0.35</v>
@@ -12725,13 +12703,13 @@
         <v>21</v>
       </c>
       <c r="C38" s="10" t="s">
+        <v>488</v>
+      </c>
+      <c r="D38" s="10" t="s">
+        <v>470</v>
+      </c>
+      <c r="E38" s="10" t="s">
         <v>490</v>
-      </c>
-      <c r="D38" s="10" t="s">
-        <v>472</v>
-      </c>
-      <c r="E38" s="10" t="s">
-        <v>492</v>
       </c>
       <c r="F38" s="18" t="n">
         <v>0.35</v>
@@ -12812,13 +12790,13 @@
         <v>21</v>
       </c>
       <c r="C39" s="10" t="s">
+        <v>488</v>
+      </c>
+      <c r="D39" s="10" t="s">
+        <v>470</v>
+      </c>
+      <c r="E39" s="10" t="s">
         <v>490</v>
-      </c>
-      <c r="D39" s="10" t="s">
-        <v>472</v>
-      </c>
-      <c r="E39" s="10" t="s">
-        <v>492</v>
       </c>
       <c r="F39" s="18" t="n">
         <v>0.35</v>
@@ -12899,13 +12877,13 @@
         <v>22</v>
       </c>
       <c r="C40" s="10" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="D40" s="10" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="E40" s="10" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="F40" s="18" t="n">
         <v>0.4</v>
@@ -12986,13 +12964,13 @@
         <v>22</v>
       </c>
       <c r="C41" s="10" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="D41" s="10" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="E41" s="10" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="F41" s="18" t="n">
         <v>0.4</v>
@@ -13067,19 +13045,19 @@
     </row>
     <row r="42" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="10" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="B42" s="18" t="n">
         <v>23</v>
       </c>
       <c r="C42" s="10" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="D42" s="10" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="E42" s="10" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="F42" s="18" t="n">
         <v>0.29</v>
@@ -13154,19 +13132,19 @@
     </row>
     <row r="43" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="10" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="B43" s="18" t="n">
         <v>24</v>
       </c>
       <c r="C43" s="10" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="D43" s="10" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="E43" s="10" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
       <c r="F43" s="18" t="n">
         <v>0.39</v>
@@ -13247,13 +13225,13 @@
         <v>26</v>
       </c>
       <c r="C44" s="10" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="D44" s="10" t="s">
         <v>261</v>
       </c>
       <c r="E44" s="10" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="F44" s="18" t="n">
         <v>0.6</v>
@@ -13334,13 +13312,13 @@
         <v>26</v>
       </c>
       <c r="C45" s="10" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="D45" s="10" t="s">
         <v>261</v>
       </c>
       <c r="E45" s="10" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="F45" s="18" t="n">
         <v>0.6</v>
@@ -13415,19 +13393,19 @@
     </row>
     <row r="46" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="10" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="B46" s="18" t="n">
         <v>27</v>
       </c>
       <c r="C46" s="10" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="D46" s="10" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="E46" s="10" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="F46" s="18" t="n">
         <v>0.42</v>
@@ -13502,19 +13480,19 @@
     </row>
     <row r="47" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="10" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="B47" s="18" t="n">
         <v>27</v>
       </c>
       <c r="C47" s="10" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="D47" s="10" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="E47" s="10" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="F47" s="18" t="n">
         <v>0.42</v>
@@ -13587,174 +13565,66 @@
       </c>
       <c r="AC47" s="18"/>
     </row>
-    <row r="48" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="13" t="s">
-        <v>339</v>
-      </c>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="10"/>
       <c r="B48" s="10"/>
-      <c r="C48" s="18" t="s">
-        <v>479</v>
-      </c>
-      <c r="D48" s="10" t="s">
-        <v>250</v>
-      </c>
-      <c r="E48" s="10" t="s">
-        <v>487</v>
-      </c>
-      <c r="F48" s="18" t="n">
-        <v>0.51</v>
-      </c>
-      <c r="G48" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="H48" s="18" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="I48" s="18" t="n">
-        <v>4</v>
-      </c>
-      <c r="J48" s="18" t="n">
-        <v>4</v>
-      </c>
-      <c r="K48" s="18" t="n">
-        <v>7.6</v>
-      </c>
-      <c r="L48" s="18" t="n">
-        <v>43.07</v>
-      </c>
-      <c r="M48" s="18" t="n">
-        <v>9.7</v>
-      </c>
-      <c r="N48" s="18" t="n">
-        <v>61.86</v>
-      </c>
-      <c r="O48" s="18" t="n">
-        <v>4.1</v>
-      </c>
-      <c r="P48" s="18" t="n">
-        <v>27.41</v>
-      </c>
-      <c r="Q48" s="18" t="n">
-        <v>8</v>
-      </c>
-      <c r="R48" s="18" t="n">
-        <v>48</v>
-      </c>
-      <c r="S48" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="T48" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="U48" s="18" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="V48" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="W48" s="18" t="n">
-        <v>27</v>
-      </c>
-      <c r="X48" s="18" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="Y48" s="18" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="Z48" s="18" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="AA48" s="18" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="AB48" s="18" t="n">
-        <v>0</v>
-      </c>
+      <c r="C48" s="18"/>
+      <c r="D48" s="10"/>
+      <c r="E48" s="10"/>
+      <c r="F48" s="10"/>
+      <c r="G48" s="18"/>
+      <c r="H48" s="18"/>
+      <c r="I48" s="18"/>
+      <c r="J48" s="18"/>
+      <c r="K48" s="18"/>
+      <c r="L48" s="18"/>
+      <c r="M48" s="18"/>
+      <c r="N48" s="18"/>
+      <c r="O48" s="18"/>
+      <c r="P48" s="18"/>
+      <c r="Q48" s="18"/>
+      <c r="R48" s="18"/>
+      <c r="S48" s="18"/>
+      <c r="T48" s="18"/>
+      <c r="U48" s="18"/>
+      <c r="V48" s="18"/>
+      <c r="W48" s="18"/>
+      <c r="X48" s="18"/>
+      <c r="Y48" s="18"/>
+      <c r="Z48" s="18"/>
+      <c r="AA48" s="18"/>
+      <c r="AB48" s="18"/>
       <c r="AC48" s="18"/>
     </row>
-    <row r="49" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="13" t="s">
-        <v>340</v>
-      </c>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="10"/>
       <c r="B49" s="10"/>
-      <c r="C49" s="18" t="s">
-        <v>496</v>
-      </c>
-      <c r="D49" s="10" t="s">
-        <v>261</v>
-      </c>
-      <c r="E49" s="10" t="s">
-        <v>486</v>
-      </c>
-      <c r="F49" s="18" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="G49" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="H49" s="18" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="I49" s="18" t="n">
-        <v>2</v>
-      </c>
-      <c r="J49" s="18" t="n">
-        <v>2</v>
-      </c>
-      <c r="K49" s="18" t="n">
-        <v>7.6</v>
-      </c>
-      <c r="L49" s="18" t="n">
-        <v>25.06</v>
-      </c>
-      <c r="M49" s="18" t="n">
-        <v>9.7</v>
-      </c>
-      <c r="N49" s="18" t="n">
-        <v>36.02</v>
-      </c>
-      <c r="O49" s="18" t="n">
-        <v>4.1</v>
-      </c>
-      <c r="P49" s="18" t="n">
-        <v>21.93</v>
-      </c>
-      <c r="Q49" s="18" t="n">
-        <v>8</v>
-      </c>
-      <c r="R49" s="18" t="n">
-        <v>48</v>
-      </c>
-      <c r="S49" s="18" t="n">
-        <v>19</v>
-      </c>
-      <c r="T49" s="18" t="n">
-        <v>5.301309524</v>
-      </c>
-      <c r="U49" s="18" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="V49" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="W49" s="18" t="n">
-        <v>27</v>
-      </c>
-      <c r="X49" s="18" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="Y49" s="18" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="Z49" s="18" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="AA49" s="18" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="AB49" s="18" t="n">
-        <v>0</v>
-      </c>
+      <c r="C49" s="18"/>
+      <c r="D49" s="10"/>
+      <c r="E49" s="10"/>
+      <c r="F49" s="10"/>
+      <c r="G49" s="18"/>
+      <c r="H49" s="18"/>
+      <c r="I49" s="18"/>
+      <c r="J49" s="18"/>
+      <c r="K49" s="18"/>
+      <c r="L49" s="18"/>
+      <c r="M49" s="18"/>
+      <c r="N49" s="18"/>
+      <c r="O49" s="18"/>
+      <c r="P49" s="18"/>
+      <c r="Q49" s="18"/>
+      <c r="R49" s="18"/>
+      <c r="S49" s="18"/>
+      <c r="T49" s="18"/>
+      <c r="U49" s="18"/>
+      <c r="V49" s="18"/>
+      <c r="W49" s="18"/>
+      <c r="X49" s="18"/>
+      <c r="Y49" s="18"/>
+      <c r="Z49" s="18"/>
+      <c r="AA49" s="18"/>
+      <c r="AB49" s="18"/>
       <c r="AC49" s="18"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14315,68 +14185,8 @@
       <c r="AB67" s="18"/>
       <c r="AC67" s="18"/>
     </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="10"/>
-      <c r="B68" s="10"/>
-      <c r="C68" s="18"/>
-      <c r="D68" s="10"/>
-      <c r="E68" s="10"/>
-      <c r="F68" s="10"/>
-      <c r="G68" s="18"/>
-      <c r="H68" s="18"/>
-      <c r="I68" s="18"/>
-      <c r="J68" s="18"/>
-      <c r="K68" s="18"/>
-      <c r="L68" s="18"/>
-      <c r="M68" s="18"/>
-      <c r="N68" s="18"/>
-      <c r="O68" s="18"/>
-      <c r="P68" s="18"/>
-      <c r="Q68" s="18"/>
-      <c r="R68" s="18"/>
-      <c r="S68" s="18"/>
-      <c r="T68" s="18"/>
-      <c r="U68" s="18"/>
-      <c r="V68" s="18"/>
-      <c r="W68" s="18"/>
-      <c r="X68" s="18"/>
-      <c r="Y68" s="18"/>
-      <c r="Z68" s="18"/>
-      <c r="AA68" s="18"/>
-      <c r="AB68" s="18"/>
-      <c r="AC68" s="18"/>
-    </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="10"/>
-      <c r="B69" s="10"/>
-      <c r="C69" s="18"/>
-      <c r="D69" s="10"/>
-      <c r="E69" s="10"/>
-      <c r="F69" s="10"/>
-      <c r="G69" s="18"/>
-      <c r="H69" s="18"/>
-      <c r="I69" s="18"/>
-      <c r="J69" s="18"/>
-      <c r="K69" s="18"/>
-      <c r="L69" s="18"/>
-      <c r="M69" s="18"/>
-      <c r="N69" s="18"/>
-      <c r="O69" s="18"/>
-      <c r="P69" s="18"/>
-      <c r="Q69" s="18"/>
-      <c r="R69" s="18"/>
-      <c r="S69" s="18"/>
-      <c r="T69" s="18"/>
-      <c r="U69" s="18"/>
-      <c r="V69" s="18"/>
-      <c r="W69" s="18"/>
-      <c r="X69" s="18"/>
-      <c r="Y69" s="18"/>
-      <c r="Z69" s="18"/>
-      <c r="AA69" s="18"/>
-      <c r="AB69" s="18"/>
-      <c r="AC69" s="18"/>
-    </row>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
chore: update `MAIN_PARAMS_2025.xlsx` resource file
</commit_message>
<xml_diff>
--- a/tests/antares/resources/MAIN_PARAMS_2025.xlsx
+++ b/tests/antares/resources/MAIN_PARAMS_2025.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="PAYS" sheetId="1" state="visible" r:id="rId2"/>
@@ -382,6 +382,12 @@
     <t xml:space="preserve">LT</t>
   </si>
   <si>
+    <t xml:space="preserve">LT00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LTH1_OFF</t>
+  </si>
+  <si>
     <t xml:space="preserve">Luxembourg</t>
   </si>
   <si>
@@ -538,31 +544,43 @@
     <t xml:space="preserve">Norvège médian</t>
   </si>
   <si>
+    <t xml:space="preserve">NOM1</t>
+  </si>
+  <si>
     <t xml:space="preserve">NOm</t>
   </si>
   <si>
     <t xml:space="preserve">Norvège nord</t>
   </si>
   <si>
+    <t xml:space="preserve">NON1</t>
+  </si>
+  <si>
     <t xml:space="preserve">NOn</t>
   </si>
   <si>
+    <t xml:space="preserve">NONC_OFF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOND_OFF</t>
+  </si>
+  <si>
     <t xml:space="preserve">Norvège sud</t>
   </si>
   <si>
-    <t xml:space="preserve">NOs1</t>
+    <t xml:space="preserve">NOS1</t>
   </si>
   <si>
     <t xml:space="preserve">NOs</t>
   </si>
   <si>
-    <t xml:space="preserve">NOs2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOs3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOsF_OFF</t>
+    <t xml:space="preserve">NOS2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOS3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOSF_OFF</t>
   </si>
   <si>
     <t xml:space="preserve">NOWB_OFF</t>
@@ -722,24 +740,6 @@
   </si>
   <si>
     <t xml:space="preserve">TYNDP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LT00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOM1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NON1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOS1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOS2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOS3</t>
   </si>
   <si>
     <t xml:space="preserve">PLE0</t>
@@ -1364,23 +1364,16 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF000000"/>
       <name val="Times New Roman"/>
       <family val="0"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFCAEEFB"/>
-        <bgColor rgb="FFCCFFFF"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -1478,19 +1471,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1518,7 +1511,7 @@
     <cellStyle name="Standard_Data provided by OT3" xfId="21"/>
     <cellStyle name="Style 45" xfId="22"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="3">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1531,13 +1524,6 @@
         <patternFill patternType="solid">
           <fgColor rgb="FF3D3D3D"/>
           <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFCAEEFB"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1570,7 +1556,7 @@
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FFFBE3D6"/>
-      <rgbColor rgb="FFCAEEFB"/>
+      <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
@@ -1627,9 +1613,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
-      <xdr:colOff>109080</xdr:colOff>
+      <xdr:colOff>108720</xdr:colOff>
       <xdr:row>10</xdr:row>
-      <xdr:rowOff>127080</xdr:rowOff>
+      <xdr:rowOff>126720</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1638,8 +1624,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7518240" y="905040"/>
-          <a:ext cx="7627680" cy="1031760"/>
+          <a:off x="7523640" y="905040"/>
+          <a:ext cx="7632000" cy="1031400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1739,9 +1725,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>541080</xdr:colOff>
+      <xdr:colOff>540720</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>167760</xdr:rowOff>
+      <xdr:rowOff>167400</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1750,8 +1736,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13574880" y="402480"/>
-          <a:ext cx="8050680" cy="1032120"/>
+          <a:off x="13578120" y="402480"/>
+          <a:ext cx="8055360" cy="1031760"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1837,7 +1823,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E107"/>
-  <sheetFormatPr defaultColWidth="10.57421875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="34.43"/>
@@ -1862,7 +1848,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
@@ -1879,7 +1865,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
         <v>8</v>
       </c>
@@ -1896,7 +1882,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
         <v>11</v>
       </c>
@@ -1913,7 +1899,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
         <v>14</v>
       </c>
@@ -1930,13 +1916,14 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>15</v>
       </c>
+      <c r="C6" s="4"/>
       <c r="D6" s="3" t="s">
         <v>17</v>
       </c>
@@ -1944,13 +1931,14 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>15</v>
       </c>
+      <c r="C7" s="4"/>
       <c r="D7" s="3" t="s">
         <v>19</v>
       </c>
@@ -1958,7 +1946,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
         <v>20</v>
       </c>
@@ -1975,7 +1963,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
         <v>23</v>
       </c>
@@ -1992,7 +1980,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
         <v>26</v>
       </c>
@@ -2009,7 +1997,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
         <v>29</v>
       </c>
@@ -2026,7 +2014,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
         <v>32</v>
       </c>
@@ -2043,13 +2031,14 @@
         <v>33</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
         <v>32</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>33</v>
       </c>
+      <c r="C13" s="4"/>
       <c r="D13" s="3" t="s">
         <v>35</v>
       </c>
@@ -2057,35 +2046,37 @@
         <v>36</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="C14" s="4"/>
+      <c r="D14" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="E14" s="3" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="C15" s="4"/>
+      <c r="D15" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="E15" s="4" t="s">
+      <c r="E15" s="3" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
         <v>37</v>
       </c>
@@ -2095,202 +2086,216 @@
       <c r="C16" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D16" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="E16" s="3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="C17" s="4"/>
+      <c r="D17" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="E17" s="4" t="s">
+      <c r="E17" s="3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="C18" s="4"/>
+      <c r="D18" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="E18" s="4" t="s">
+      <c r="E18" s="3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="C19" s="4"/>
+      <c r="D19" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="E19" s="4" t="s">
+      <c r="E19" s="3" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="C20" s="4"/>
+      <c r="D20" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="E20" s="4" t="s">
+      <c r="E20" s="3" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="C21" s="4"/>
+      <c r="D21" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="E21" s="4" t="s">
+      <c r="E21" s="3" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="C22" s="4"/>
+      <c r="D22" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="E22" s="4" t="s">
+      <c r="E22" s="3" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D23" s="4" t="s">
+      <c r="C23" s="4"/>
+      <c r="D23" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="E23" s="4" t="s">
+      <c r="E23" s="3" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D24" s="4" t="s">
+      <c r="C24" s="4"/>
+      <c r="D24" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="E24" s="4" t="s">
+      <c r="E24" s="3" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D25" s="4" t="s">
+      <c r="C25" s="4"/>
+      <c r="D25" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="E25" s="4" t="s">
+      <c r="E25" s="3" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D26" s="4" t="s">
+      <c r="C26" s="4"/>
+      <c r="D26" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="E26" s="4" t="s">
+      <c r="E26" s="3" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D27" s="4" t="s">
+      <c r="C27" s="4"/>
+      <c r="D27" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="E27" s="4" t="s">
+      <c r="E27" s="3" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D28" s="4" t="s">
+      <c r="C28" s="4"/>
+      <c r="D28" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="E28" s="4" t="s">
+      <c r="E28" s="3" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D29" s="4" t="s">
+      <c r="C29" s="4"/>
+      <c r="D29" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="E29" s="4" t="s">
+      <c r="E29" s="3" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>38</v>
       </c>
+      <c r="C30" s="4"/>
       <c r="D30" s="3" t="s">
         <v>60</v>
       </c>
@@ -2298,7 +2303,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
         <v>37</v>
       </c>
@@ -2315,7 +2320,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
         <v>64</v>
       </c>
@@ -2332,7 +2337,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
         <v>67</v>
       </c>
@@ -2349,7 +2354,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
         <v>70</v>
       </c>
@@ -2366,7 +2371,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
         <v>73</v>
       </c>
@@ -2383,7 +2388,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
         <v>73</v>
       </c>
@@ -2396,8 +2401,9 @@
       <c r="D36" s="3" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E36" s="4"/>
+    </row>
+    <row r="37" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="3" t="s">
         <v>78</v>
       </c>
@@ -2407,14 +2413,14 @@
       <c r="C37" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="D37" s="4" t="s">
+      <c r="D37" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="E37" s="4" t="s">
+      <c r="E37" s="3" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">
         <v>78</v>
       </c>
@@ -2424,14 +2430,14 @@
       <c r="C38" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="D38" s="4" t="s">
+      <c r="D38" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="E38" s="4" t="s">
+      <c r="E38" s="3" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="3" t="s">
         <v>83</v>
       </c>
@@ -2448,7 +2454,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
         <v>86</v>
       </c>
@@ -2465,7 +2471,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="3" t="s">
         <v>89</v>
       </c>
@@ -2482,7 +2488,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="s">
         <v>92</v>
       </c>
@@ -2499,7 +2505,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="3" t="s">
         <v>92</v>
       </c>
@@ -2516,7 +2522,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="3" t="s">
         <v>92</v>
       </c>
@@ -2533,7 +2539,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="3" t="s">
         <v>92</v>
       </c>
@@ -2550,7 +2556,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="3" t="s">
         <v>92</v>
       </c>
@@ -2567,7 +2573,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="3" t="s">
         <v>92</v>
       </c>
@@ -2584,7 +2590,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="3" t="s">
         <v>92</v>
       </c>
@@ -2601,7 +2607,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="3" t="s">
         <v>115</v>
       </c>
@@ -2611,895 +2617,929 @@
       <c r="C49" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="D49" s="4" t="s">
+      <c r="D49" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="E49" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="E49" s="4" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="50" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="3" t="s">
         <v>115</v>
       </c>
       <c r="B50" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="D50" s="4" t="s">
+      <c r="C50" s="4"/>
+      <c r="D50" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="E50" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="E50" s="4" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="51" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="3" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D51" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E51" s="4"/>
+    </row>
+    <row r="52" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="3" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="3" t="s">
-        <v>117</v>
-      </c>
       <c r="B52" s="3" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D52" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="E52" s="4"/>
+    </row>
+    <row r="53" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="B53" s="3" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="B53" s="3" t="s">
-        <v>118</v>
-      </c>
       <c r="C53" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="D53" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="E53" s="4" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>119</v>
+      </c>
+      <c r="D53" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="E53" s="3" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="3" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="D54" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="E54" s="4" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>119</v>
+      </c>
+      <c r="D54" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="E54" s="3" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="3" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="3" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>130</v>
+      </c>
+      <c r="E56" s="4"/>
+    </row>
+    <row r="57" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="3" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="3" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D58" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E58" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="E58" s="3" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="59" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="3" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="D60" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="E60" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D60" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="E60" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D61" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="E61" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C61" s="4"/>
+      <c r="D61" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="E61" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D62" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="E62" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>142</v>
+      </c>
+      <c r="C62" s="4"/>
+      <c r="D62" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="E62" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D63" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="E63" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>142</v>
+      </c>
+      <c r="C63" s="4"/>
+      <c r="D63" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="E63" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D64" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="E64" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>142</v>
+      </c>
+      <c r="C64" s="4"/>
+      <c r="D64" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="E64" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D65" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="E65" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>142</v>
+      </c>
+      <c r="C65" s="4"/>
+      <c r="D65" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="E65" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D66" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="E66" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="67" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>142</v>
+      </c>
+      <c r="C66" s="4"/>
+      <c r="D66" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="E66" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D67" s="4" t="s">
-        <v>148</v>
-      </c>
-      <c r="E67" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="68" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>142</v>
+      </c>
+      <c r="C67" s="4"/>
+      <c r="D67" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="E67" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D68" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="E68" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="69" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>142</v>
+      </c>
+      <c r="C68" s="4"/>
+      <c r="D68" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="E68" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D69" s="4" t="s">
-        <v>150</v>
-      </c>
-      <c r="E69" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="70" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>142</v>
+      </c>
+      <c r="C69" s="4"/>
+      <c r="D69" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="E69" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D70" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="E70" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="71" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>142</v>
+      </c>
+      <c r="C70" s="4"/>
+      <c r="D70" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="E70" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D71" s="4" t="s">
-        <v>152</v>
-      </c>
-      <c r="E71" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="72" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>142</v>
+      </c>
+      <c r="C71" s="4"/>
+      <c r="D71" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E71" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D72" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="E72" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="73" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>142</v>
+      </c>
+      <c r="C72" s="4"/>
+      <c r="D72" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="E72" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D73" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="E73" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="74" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>142</v>
+      </c>
+      <c r="C73" s="4"/>
+      <c r="D73" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="E73" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D74" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="E74" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="75" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>142</v>
+      </c>
+      <c r="C74" s="4"/>
+      <c r="D74" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="E74" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D75" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="E75" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="76" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>142</v>
+      </c>
+      <c r="C75" s="4"/>
+      <c r="D75" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="E75" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D76" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="E76" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="77" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>142</v>
+      </c>
+      <c r="C76" s="4"/>
+      <c r="D76" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="E76" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D77" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="E77" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="78" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>142</v>
+      </c>
+      <c r="C77" s="4"/>
+      <c r="D77" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="E77" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B78" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D78" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="E78" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="79" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>142</v>
+      </c>
+      <c r="C78" s="4"/>
+      <c r="D78" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="E78" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D79" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="E79" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="80" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>142</v>
+      </c>
+      <c r="C79" s="4"/>
+      <c r="D79" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="E79" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B80" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D80" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="E80" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="81" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>142</v>
+      </c>
+      <c r="C80" s="4"/>
+      <c r="D80" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="E80" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B81" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D81" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="E81" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="82" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>142</v>
+      </c>
+      <c r="C81" s="4"/>
+      <c r="D81" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="E81" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B82" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D82" s="4" t="s">
-        <v>163</v>
-      </c>
-      <c r="E82" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="83" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>142</v>
+      </c>
+      <c r="C82" s="4"/>
+      <c r="D82" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="E82" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B83" s="3" t="s">
-        <v>140</v>
-      </c>
+        <v>142</v>
+      </c>
+      <c r="C83" s="4"/>
       <c r="D83" s="3" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="E83" s="3" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="84" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="3" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B84" s="3" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C84" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="D84" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="E84" s="3" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="D84" s="4" t="s">
+      <c r="B85" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="E84" s="4" t="s">
+      <c r="C85" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="D85" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E85" s="3" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="B86" s="3" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="85" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="B85" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="C85" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="D85" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="E85" s="4" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="86" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="B86" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="D86" s="4" t="s">
+      <c r="C86" s="4"/>
+      <c r="D86" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="E86" s="3" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="B87" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="E86" s="4" t="s">
+      <c r="C87" s="4"/>
+      <c r="D87" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="E87" s="3" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="B88" s="3" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="87" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="B87" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="D87" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="E87" s="4" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="88" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="B88" s="3" t="s">
-        <v>167</v>
-      </c>
       <c r="C88" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="D88" s="4" t="s">
-        <v>173</v>
-      </c>
-      <c r="E88" s="4" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="89" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>178</v>
+      </c>
+      <c r="D88" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="E88" s="3" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="89" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="3" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B89" s="3" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C89" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="D89" s="4" t="s">
-        <v>175</v>
-      </c>
-      <c r="E89" s="4" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="90" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>178</v>
+      </c>
+      <c r="D89" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="E89" s="3" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="3" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B90" s="3" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C90" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="D90" s="4" t="s">
-        <v>176</v>
-      </c>
-      <c r="E90" s="4" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="91" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>178</v>
+      </c>
+      <c r="D90" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="E90" s="3" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="3" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B91" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="D91" s="4" t="s">
-        <v>177</v>
-      </c>
-      <c r="E91" s="4" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="92" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>169</v>
+      </c>
+      <c r="C91" s="4"/>
+      <c r="D91" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="E91" s="3" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="3" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B92" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="D92" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="E92" s="4" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="93" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>169</v>
+      </c>
+      <c r="C92" s="4"/>
+      <c r="D92" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="E92" s="3" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="93" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="3" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B93" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="D93" s="4" t="s">
-        <v>179</v>
-      </c>
-      <c r="E93" s="4" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="94" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>169</v>
+      </c>
+      <c r="C93" s="4"/>
+      <c r="D93" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="E93" s="3" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="94" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="3" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="B94" s="3" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="C94" s="3" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="D94" s="3" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="E94" s="3" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="95" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="95" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="3" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="B95" s="3" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="C95" s="3" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="D95" s="3" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="E95" s="3" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="96" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="96" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="3" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
       <c r="B96" s="3" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="C96" s="3" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
       <c r="D96" s="3" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="E96" s="3" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="97" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="97" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="3" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="B97" s="3" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="C97" s="3" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="D97" s="3" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="E97" s="3" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="98" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="98" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="3" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="B98" s="3" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="C98" s="3" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="D98" s="3" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="E98" s="3" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="99" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="99" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="3" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="B99" s="3" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="C99" s="3" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="D99" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="E99" s="3" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="100" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A100" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="E99" s="3" t="s">
+      <c r="B100" s="3" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="100" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A100" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="B100" s="3" t="s">
-        <v>193</v>
-      </c>
       <c r="C100" s="3" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="D100" s="3" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="E100" s="3" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="101" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="101" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="3" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="B101" s="3" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="C101" s="3" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="D101" s="3" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="E101" s="3" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="102" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="102" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="3" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="B102" s="3" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="C102" s="3" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="D102" s="3" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="E102" s="3" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="103" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="103" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="B103" s="3" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="C103" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="D103" s="3" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="E103" s="3" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="104" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="104" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="3" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="B104" s="3" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="C104" s="3" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="D104" s="3" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="105" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>220</v>
+      </c>
+      <c r="E104" s="4"/>
+    </row>
+    <row r="105" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="3" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="B105" s="3" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
       <c r="C105" s="3" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="D105" s="3" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="106" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>223</v>
+      </c>
+      <c r="E105" s="4"/>
+    </row>
+    <row r="106" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="3" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
       <c r="B106" s="3" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="C106" s="3" t="s">
-        <v>220</v>
+        <v>226</v>
       </c>
       <c r="D106" s="3" t="s">
-        <v>221</v>
+        <v>227</v>
       </c>
       <c r="E106" s="3" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="107" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="107" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="3" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
       <c r="B107" s="3" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="C107" s="3" t="s">
-        <v>224</v>
+        <v>230</v>
       </c>
       <c r="D107" s="3" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="E107" s="3" t="s">
-        <v>226</v>
+        <v>232</v>
       </c>
     </row>
   </sheetData>
@@ -3521,14 +3561,14 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B42"/>
-  <sheetFormatPr defaultColWidth="10.57421875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>227</v>
+        <v>233</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>228</v>
+        <v>234</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3536,7 +3576,7 @@
         <v>2020</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3545,7 +3585,7 @@
         <v>2021</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3554,7 +3594,7 @@
         <v>2022</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3563,7 +3603,7 @@
         <v>2023</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3572,7 +3612,7 @@
         <v>2024</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3581,7 +3621,7 @@
         <v>2025</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3590,7 +3630,7 @@
         <v>2026</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3599,7 +3639,7 @@
         <v>2027</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3608,7 +3648,7 @@
         <v>2028</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3617,7 +3657,7 @@
         <v>2029</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3626,7 +3666,7 @@
         <v>2030</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3635,7 +3675,7 @@
         <v>2031</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3644,7 +3684,7 @@
         <v>2032</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3653,7 +3693,7 @@
         <v>2033</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3662,7 +3702,7 @@
         <v>2034</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3671,7 +3711,7 @@
         <v>2035</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3680,7 +3720,7 @@
         <v>2036</v>
       </c>
       <c r="B18" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3689,7 +3729,7 @@
         <v>2037</v>
       </c>
       <c r="B19" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3698,7 +3738,7 @@
         <v>2038</v>
       </c>
       <c r="B20" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3707,7 +3747,7 @@
         <v>2039</v>
       </c>
       <c r="B21" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3716,7 +3756,7 @@
         <v>2040</v>
       </c>
       <c r="B22" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3725,7 +3765,7 @@
         <v>2041</v>
       </c>
       <c r="B23" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3734,7 +3774,7 @@
         <v>2042</v>
       </c>
       <c r="B24" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3743,7 +3783,7 @@
         <v>2043</v>
       </c>
       <c r="B25" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3752,7 +3792,7 @@
         <v>2044</v>
       </c>
       <c r="B26" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3761,7 +3801,7 @@
         <v>2045</v>
       </c>
       <c r="B27" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3770,7 +3810,7 @@
         <v>2046</v>
       </c>
       <c r="B28" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3779,7 +3819,7 @@
         <v>2047</v>
       </c>
       <c r="B29" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3788,7 +3828,7 @@
         <v>2048</v>
       </c>
       <c r="B30" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3797,7 +3837,7 @@
         <v>2049</v>
       </c>
       <c r="B31" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3806,7 +3846,7 @@
         <v>2050</v>
       </c>
       <c r="B32" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3815,7 +3855,7 @@
         <v>2051</v>
       </c>
       <c r="B33" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3824,7 +3864,7 @@
         <v>2052</v>
       </c>
       <c r="B34" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3833,7 +3873,7 @@
         <v>2053</v>
       </c>
       <c r="B35" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3842,7 +3882,7 @@
         <v>2054</v>
       </c>
       <c r="B36" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3851,7 +3891,7 @@
         <v>2055</v>
       </c>
       <c r="B37" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3860,7 +3900,7 @@
         <v>2056</v>
       </c>
       <c r="B38" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3869,7 +3909,7 @@
         <v>2057</v>
       </c>
       <c r="B39" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3878,7 +3918,7 @@
         <v>2058</v>
       </c>
       <c r="B40" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3887,7 +3927,7 @@
         <v>2059</v>
       </c>
       <c r="B41" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3896,7 +3936,7 @@
         <v>2060</v>
       </c>
       <c r="B42" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
   </sheetData>
@@ -3917,7 +3957,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B60"/>
-  <sheetFormatPr defaultColWidth="10.57421875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.43"/>
@@ -4189,7 +4229,7 @@
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
-        <v>231</v>
+        <v>117</v>
       </c>
       <c r="B34" s="3" t="s">
         <v>116</v>
@@ -4197,106 +4237,106 @@
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="6" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="6" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="3" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="B39" s="3" t="s">
         <v>135</v>
-      </c>
-      <c r="B39" s="3" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="3" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="s">
-        <v>232</v>
+        <v>171</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="3" t="s">
-        <v>233</v>
+        <v>174</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="6" t="s">
-        <v>234</v>
+        <v>179</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="6" t="s">
-        <v>235</v>
+        <v>181</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="6" t="s">
-        <v>236</v>
+        <v>182</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="6" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4304,7 +4344,7 @@
         <v>237</v>
       </c>
       <c r="B48" s="6" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4312,95 +4352,95 @@
         <v>238</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="3" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="3" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="3" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="3" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="3" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="3" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="3" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="3" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="3" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="3" t="s">
-        <v>221</v>
+        <v>227</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>222</v>
+        <v>228</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="3" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>226</v>
+        <v>232</v>
       </c>
     </row>
   </sheetData>
@@ -4420,7 +4460,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D90"/>
-  <sheetFormatPr defaultColWidth="10.57421875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="69.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30.29"/>
@@ -5636,7 +5676,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D67"/>
-  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.15234375" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.14"/>
@@ -6343,7 +6383,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D25"/>
-  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.15234375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">

</xml_diff>

<commit_message>
chore: update sheet PAYS : `MAIN_PARAMS_2025.xlsx` resource file (#34)
* chore: update `MAIN_PARAMS_2025.xlsx` resource file

* tests: update referential data mappings in `test_main_params.py`
</commit_message>
<xml_diff>
--- a/tests/antares/resources/MAIN_PARAMS_2025.xlsx
+++ b/tests/antares/resources/MAIN_PARAMS_2025.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="PAYS" sheetId="1" state="visible" r:id="rId2"/>
@@ -382,6 +382,12 @@
     <t xml:space="preserve">LT</t>
   </si>
   <si>
+    <t xml:space="preserve">LT00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LTH1_OFF</t>
+  </si>
+  <si>
     <t xml:space="preserve">Luxembourg</t>
   </si>
   <si>
@@ -538,31 +544,43 @@
     <t xml:space="preserve">Norvège médian</t>
   </si>
   <si>
+    <t xml:space="preserve">NOM1</t>
+  </si>
+  <si>
     <t xml:space="preserve">NOm</t>
   </si>
   <si>
     <t xml:space="preserve">Norvège nord</t>
   </si>
   <si>
+    <t xml:space="preserve">NON1</t>
+  </si>
+  <si>
     <t xml:space="preserve">NOn</t>
   </si>
   <si>
+    <t xml:space="preserve">NONC_OFF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOND_OFF</t>
+  </si>
+  <si>
     <t xml:space="preserve">Norvège sud</t>
   </si>
   <si>
-    <t xml:space="preserve">NOs1</t>
+    <t xml:space="preserve">NOS1</t>
   </si>
   <si>
     <t xml:space="preserve">NOs</t>
   </si>
   <si>
-    <t xml:space="preserve">NOs2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOs3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOsF_OFF</t>
+    <t xml:space="preserve">NOS2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOS3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOSF_OFF</t>
   </si>
   <si>
     <t xml:space="preserve">NOWB_OFF</t>
@@ -722,24 +740,6 @@
   </si>
   <si>
     <t xml:space="preserve">TYNDP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LT00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOM1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NON1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOS1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOS2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOS3</t>
   </si>
   <si>
     <t xml:space="preserve">PLE0</t>
@@ -1364,23 +1364,16 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF000000"/>
       <name val="Times New Roman"/>
       <family val="0"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFCAEEFB"/>
-        <bgColor rgb="FFCCFFFF"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -1478,19 +1471,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1518,7 +1511,7 @@
     <cellStyle name="Standard_Data provided by OT3" xfId="21"/>
     <cellStyle name="Style 45" xfId="22"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="3">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1531,13 +1524,6 @@
         <patternFill patternType="solid">
           <fgColor rgb="FF3D3D3D"/>
           <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFCAEEFB"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1570,7 +1556,7 @@
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FFFBE3D6"/>
-      <rgbColor rgb="FFCAEEFB"/>
+      <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
@@ -1627,9 +1613,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
-      <xdr:colOff>109080</xdr:colOff>
+      <xdr:colOff>108720</xdr:colOff>
       <xdr:row>10</xdr:row>
-      <xdr:rowOff>127080</xdr:rowOff>
+      <xdr:rowOff>126720</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1638,8 +1624,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7518240" y="905040"/>
-          <a:ext cx="7627680" cy="1031760"/>
+          <a:off x="7523640" y="905040"/>
+          <a:ext cx="7632000" cy="1031400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1739,9 +1725,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>541080</xdr:colOff>
+      <xdr:colOff>540720</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>167760</xdr:rowOff>
+      <xdr:rowOff>167400</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1750,8 +1736,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13574880" y="402480"/>
-          <a:ext cx="8050680" cy="1032120"/>
+          <a:off x="13578120" y="402480"/>
+          <a:ext cx="8055360" cy="1031760"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1837,7 +1823,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E107"/>
-  <sheetFormatPr defaultColWidth="10.57421875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="34.43"/>
@@ -1862,7 +1848,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
@@ -1879,7 +1865,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
         <v>8</v>
       </c>
@@ -1896,7 +1882,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
         <v>11</v>
       </c>
@@ -1913,7 +1899,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
         <v>14</v>
       </c>
@@ -1930,13 +1916,14 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>15</v>
       </c>
+      <c r="C6" s="4"/>
       <c r="D6" s="3" t="s">
         <v>17</v>
       </c>
@@ -1944,13 +1931,14 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>15</v>
       </c>
+      <c r="C7" s="4"/>
       <c r="D7" s="3" t="s">
         <v>19</v>
       </c>
@@ -1958,7 +1946,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
         <v>20</v>
       </c>
@@ -1975,7 +1963,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
         <v>23</v>
       </c>
@@ -1992,7 +1980,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
         <v>26</v>
       </c>
@@ -2009,7 +1997,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
         <v>29</v>
       </c>
@@ -2026,7 +2014,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
         <v>32</v>
       </c>
@@ -2043,13 +2031,14 @@
         <v>33</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
         <v>32</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>33</v>
       </c>
+      <c r="C13" s="4"/>
       <c r="D13" s="3" t="s">
         <v>35</v>
       </c>
@@ -2057,35 +2046,37 @@
         <v>36</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="C14" s="4"/>
+      <c r="D14" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="E14" s="3" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="C15" s="4"/>
+      <c r="D15" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="E15" s="4" t="s">
+      <c r="E15" s="3" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
         <v>37</v>
       </c>
@@ -2095,202 +2086,216 @@
       <c r="C16" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D16" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="E16" s="3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="C17" s="4"/>
+      <c r="D17" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="E17" s="4" t="s">
+      <c r="E17" s="3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="C18" s="4"/>
+      <c r="D18" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="E18" s="4" t="s">
+      <c r="E18" s="3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="C19" s="4"/>
+      <c r="D19" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="E19" s="4" t="s">
+      <c r="E19" s="3" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="C20" s="4"/>
+      <c r="D20" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="E20" s="4" t="s">
+      <c r="E20" s="3" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="C21" s="4"/>
+      <c r="D21" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="E21" s="4" t="s">
+      <c r="E21" s="3" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="C22" s="4"/>
+      <c r="D22" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="E22" s="4" t="s">
+      <c r="E22" s="3" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D23" s="4" t="s">
+      <c r="C23" s="4"/>
+      <c r="D23" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="E23" s="4" t="s">
+      <c r="E23" s="3" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D24" s="4" t="s">
+      <c r="C24" s="4"/>
+      <c r="D24" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="E24" s="4" t="s">
+      <c r="E24" s="3" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D25" s="4" t="s">
+      <c r="C25" s="4"/>
+      <c r="D25" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="E25" s="4" t="s">
+      <c r="E25" s="3" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D26" s="4" t="s">
+      <c r="C26" s="4"/>
+      <c r="D26" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="E26" s="4" t="s">
+      <c r="E26" s="3" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D27" s="4" t="s">
+      <c r="C27" s="4"/>
+      <c r="D27" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="E27" s="4" t="s">
+      <c r="E27" s="3" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D28" s="4" t="s">
+      <c r="C28" s="4"/>
+      <c r="D28" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="E28" s="4" t="s">
+      <c r="E28" s="3" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D29" s="4" t="s">
+      <c r="C29" s="4"/>
+      <c r="D29" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="E29" s="4" t="s">
+      <c r="E29" s="3" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>38</v>
       </c>
+      <c r="C30" s="4"/>
       <c r="D30" s="3" t="s">
         <v>60</v>
       </c>
@@ -2298,7 +2303,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
         <v>37</v>
       </c>
@@ -2315,7 +2320,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
         <v>64</v>
       </c>
@@ -2332,7 +2337,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
         <v>67</v>
       </c>
@@ -2349,7 +2354,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
         <v>70</v>
       </c>
@@ -2366,7 +2371,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
         <v>73</v>
       </c>
@@ -2383,7 +2388,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
         <v>73</v>
       </c>
@@ -2396,8 +2401,9 @@
       <c r="D36" s="3" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E36" s="4"/>
+    </row>
+    <row r="37" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="3" t="s">
         <v>78</v>
       </c>
@@ -2407,14 +2413,14 @@
       <c r="C37" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="D37" s="4" t="s">
+      <c r="D37" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="E37" s="4" t="s">
+      <c r="E37" s="3" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">
         <v>78</v>
       </c>
@@ -2424,14 +2430,14 @@
       <c r="C38" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="D38" s="4" t="s">
+      <c r="D38" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="E38" s="4" t="s">
+      <c r="E38" s="3" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="3" t="s">
         <v>83</v>
       </c>
@@ -2448,7 +2454,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
         <v>86</v>
       </c>
@@ -2465,7 +2471,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="3" t="s">
         <v>89</v>
       </c>
@@ -2482,7 +2488,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="s">
         <v>92</v>
       </c>
@@ -2499,7 +2505,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="3" t="s">
         <v>92</v>
       </c>
@@ -2516,7 +2522,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="3" t="s">
         <v>92</v>
       </c>
@@ -2533,7 +2539,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="3" t="s">
         <v>92</v>
       </c>
@@ -2550,7 +2556,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="3" t="s">
         <v>92</v>
       </c>
@@ -2567,7 +2573,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="3" t="s">
         <v>92</v>
       </c>
@@ -2584,7 +2590,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="3" t="s">
         <v>92</v>
       </c>
@@ -2601,7 +2607,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="3" t="s">
         <v>115</v>
       </c>
@@ -2611,895 +2617,929 @@
       <c r="C49" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="D49" s="4" t="s">
+      <c r="D49" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="E49" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="E49" s="4" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="50" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="3" t="s">
         <v>115</v>
       </c>
       <c r="B50" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="D50" s="4" t="s">
+      <c r="C50" s="4"/>
+      <c r="D50" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="E50" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="E50" s="4" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="51" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="3" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D51" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E51" s="4"/>
+    </row>
+    <row r="52" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="3" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="3" t="s">
-        <v>117</v>
-      </c>
       <c r="B52" s="3" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D52" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="E52" s="4"/>
+    </row>
+    <row r="53" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="B53" s="3" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="B53" s="3" t="s">
-        <v>118</v>
-      </c>
       <c r="C53" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="D53" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="E53" s="4" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>119</v>
+      </c>
+      <c r="D53" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="E53" s="3" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="3" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="D54" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="E54" s="4" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>119</v>
+      </c>
+      <c r="D54" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="E54" s="3" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="3" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E55" s="3" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="3" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>130</v>
+      </c>
+      <c r="E56" s="4"/>
+    </row>
+    <row r="57" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="3" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="3" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D58" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E58" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="E58" s="3" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="59" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="3" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="D60" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="E60" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D60" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="E60" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D61" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="E61" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C61" s="4"/>
+      <c r="D61" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="E61" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D62" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="E62" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>142</v>
+      </c>
+      <c r="C62" s="4"/>
+      <c r="D62" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="E62" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D63" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="E63" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="64" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>142</v>
+      </c>
+      <c r="C63" s="4"/>
+      <c r="D63" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="E63" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D64" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="E64" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>142</v>
+      </c>
+      <c r="C64" s="4"/>
+      <c r="D64" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="E64" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D65" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="E65" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="66" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>142</v>
+      </c>
+      <c r="C65" s="4"/>
+      <c r="D65" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="E65" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D66" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="E66" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="67" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>142</v>
+      </c>
+      <c r="C66" s="4"/>
+      <c r="D66" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="E66" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D67" s="4" t="s">
-        <v>148</v>
-      </c>
-      <c r="E67" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="68" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>142</v>
+      </c>
+      <c r="C67" s="4"/>
+      <c r="D67" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="E67" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D68" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="E68" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="69" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>142</v>
+      </c>
+      <c r="C68" s="4"/>
+      <c r="D68" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="E68" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D69" s="4" t="s">
-        <v>150</v>
-      </c>
-      <c r="E69" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="70" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>142</v>
+      </c>
+      <c r="C69" s="4"/>
+      <c r="D69" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="E69" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D70" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="E70" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="71" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>142</v>
+      </c>
+      <c r="C70" s="4"/>
+      <c r="D70" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="E70" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D71" s="4" t="s">
-        <v>152</v>
-      </c>
-      <c r="E71" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="72" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>142</v>
+      </c>
+      <c r="C71" s="4"/>
+      <c r="D71" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E71" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D72" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="E72" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="73" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>142</v>
+      </c>
+      <c r="C72" s="4"/>
+      <c r="D72" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="E72" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D73" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="E73" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="74" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>142</v>
+      </c>
+      <c r="C73" s="4"/>
+      <c r="D73" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="E73" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D74" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="E74" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="75" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>142</v>
+      </c>
+      <c r="C74" s="4"/>
+      <c r="D74" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="E74" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D75" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="E75" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="76" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>142</v>
+      </c>
+      <c r="C75" s="4"/>
+      <c r="D75" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="E75" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D76" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="E76" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="77" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>142</v>
+      </c>
+      <c r="C76" s="4"/>
+      <c r="D76" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="E76" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D77" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="E77" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="78" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>142</v>
+      </c>
+      <c r="C77" s="4"/>
+      <c r="D77" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="E77" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B78" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D78" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="E78" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="79" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>142</v>
+      </c>
+      <c r="C78" s="4"/>
+      <c r="D78" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="E78" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D79" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="E79" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="80" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>142</v>
+      </c>
+      <c r="C79" s="4"/>
+      <c r="D79" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="E79" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B80" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D80" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="E80" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="81" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>142</v>
+      </c>
+      <c r="C80" s="4"/>
+      <c r="D80" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="E80" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B81" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D81" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="E81" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="82" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>142</v>
+      </c>
+      <c r="C81" s="4"/>
+      <c r="D81" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="E81" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B82" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D82" s="4" t="s">
-        <v>163</v>
-      </c>
-      <c r="E82" s="4" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="83" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>142</v>
+      </c>
+      <c r="C82" s="4"/>
+      <c r="D82" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="E82" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B83" s="3" t="s">
-        <v>140</v>
-      </c>
+        <v>142</v>
+      </c>
+      <c r="C83" s="4"/>
       <c r="D83" s="3" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="E83" s="3" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="84" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="3" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B84" s="3" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C84" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="D84" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="E84" s="3" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="D84" s="4" t="s">
+      <c r="B85" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="E84" s="4" t="s">
+      <c r="C85" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="D85" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E85" s="3" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="B86" s="3" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="85" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="B85" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="C85" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="D85" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="E85" s="4" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="86" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="B86" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="D86" s="4" t="s">
+      <c r="C86" s="4"/>
+      <c r="D86" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="E86" s="3" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="B87" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="E86" s="4" t="s">
+      <c r="C87" s="4"/>
+      <c r="D87" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="E87" s="3" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="B88" s="3" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="87" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="B87" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="D87" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="E87" s="4" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="88" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="B88" s="3" t="s">
-        <v>167</v>
-      </c>
       <c r="C88" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="D88" s="4" t="s">
-        <v>173</v>
-      </c>
-      <c r="E88" s="4" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="89" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>178</v>
+      </c>
+      <c r="D88" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="E88" s="3" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="89" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="3" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B89" s="3" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C89" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="D89" s="4" t="s">
-        <v>175</v>
-      </c>
-      <c r="E89" s="4" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="90" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>178</v>
+      </c>
+      <c r="D89" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="E89" s="3" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="3" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B90" s="3" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C90" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="D90" s="4" t="s">
-        <v>176</v>
-      </c>
-      <c r="E90" s="4" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="91" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>178</v>
+      </c>
+      <c r="D90" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="E90" s="3" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="3" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B91" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="D91" s="4" t="s">
-        <v>177</v>
-      </c>
-      <c r="E91" s="4" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="92" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>169</v>
+      </c>
+      <c r="C91" s="4"/>
+      <c r="D91" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="E91" s="3" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="3" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B92" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="D92" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="E92" s="4" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="93" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>169</v>
+      </c>
+      <c r="C92" s="4"/>
+      <c r="D92" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="E92" s="3" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="93" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="3" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B93" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="D93" s="4" t="s">
-        <v>179</v>
-      </c>
-      <c r="E93" s="4" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="94" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>169</v>
+      </c>
+      <c r="C93" s="4"/>
+      <c r="D93" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="E93" s="3" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="94" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="3" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="B94" s="3" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="C94" s="3" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="D94" s="3" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="E94" s="3" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="95" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="95" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="3" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="B95" s="3" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="C95" s="3" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="D95" s="3" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="E95" s="3" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="96" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="96" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="3" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
       <c r="B96" s="3" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="C96" s="3" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
       <c r="D96" s="3" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="E96" s="3" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="97" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="97" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="3" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="B97" s="3" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="C97" s="3" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="D97" s="3" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="E97" s="3" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="98" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="98" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="3" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="B98" s="3" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="C98" s="3" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="D98" s="3" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="E98" s="3" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="99" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="99" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="3" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="B99" s="3" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="C99" s="3" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="D99" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="E99" s="3" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="100" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A100" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="E99" s="3" t="s">
+      <c r="B100" s="3" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="100" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A100" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="B100" s="3" t="s">
-        <v>193</v>
-      </c>
       <c r="C100" s="3" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="D100" s="3" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="E100" s="3" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="101" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="101" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="3" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="B101" s="3" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="C101" s="3" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="D101" s="3" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="E101" s="3" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="102" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="102" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="3" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="B102" s="3" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="C102" s="3" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="D102" s="3" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="E102" s="3" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="103" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="103" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="B103" s="3" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="C103" s="3" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="D103" s="3" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="E103" s="3" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="104" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="104" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="3" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="B104" s="3" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="C104" s="3" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="D104" s="3" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="105" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>220</v>
+      </c>
+      <c r="E104" s="4"/>
+    </row>
+    <row r="105" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="3" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="B105" s="3" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
       <c r="C105" s="3" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="D105" s="3" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="106" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>223</v>
+      </c>
+      <c r="E105" s="4"/>
+    </row>
+    <row r="106" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="3" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
       <c r="B106" s="3" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="C106" s="3" t="s">
-        <v>220</v>
+        <v>226</v>
       </c>
       <c r="D106" s="3" t="s">
-        <v>221</v>
+        <v>227</v>
       </c>
       <c r="E106" s="3" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="107" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="107" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="3" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
       <c r="B107" s="3" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="C107" s="3" t="s">
-        <v>224</v>
+        <v>230</v>
       </c>
       <c r="D107" s="3" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="E107" s="3" t="s">
-        <v>226</v>
+        <v>232</v>
       </c>
     </row>
   </sheetData>
@@ -3521,14 +3561,14 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B42"/>
-  <sheetFormatPr defaultColWidth="10.57421875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>227</v>
+        <v>233</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>228</v>
+        <v>234</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3536,7 +3576,7 @@
         <v>2020</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3545,7 +3585,7 @@
         <v>2021</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3554,7 +3594,7 @@
         <v>2022</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3563,7 +3603,7 @@
         <v>2023</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3572,7 +3612,7 @@
         <v>2024</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3581,7 +3621,7 @@
         <v>2025</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3590,7 +3630,7 @@
         <v>2026</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3599,7 +3639,7 @@
         <v>2027</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3608,7 +3648,7 @@
         <v>2028</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3617,7 +3657,7 @@
         <v>2029</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3626,7 +3666,7 @@
         <v>2030</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3635,7 +3675,7 @@
         <v>2031</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3644,7 +3684,7 @@
         <v>2032</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3653,7 +3693,7 @@
         <v>2033</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3662,7 +3702,7 @@
         <v>2034</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3671,7 +3711,7 @@
         <v>2035</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3680,7 +3720,7 @@
         <v>2036</v>
       </c>
       <c r="B18" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3689,7 +3729,7 @@
         <v>2037</v>
       </c>
       <c r="B19" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3698,7 +3738,7 @@
         <v>2038</v>
       </c>
       <c r="B20" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3707,7 +3747,7 @@
         <v>2039</v>
       </c>
       <c r="B21" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3716,7 +3756,7 @@
         <v>2040</v>
       </c>
       <c r="B22" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3725,7 +3765,7 @@
         <v>2041</v>
       </c>
       <c r="B23" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3734,7 +3774,7 @@
         <v>2042</v>
       </c>
       <c r="B24" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3743,7 +3783,7 @@
         <v>2043</v>
       </c>
       <c r="B25" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3752,7 +3792,7 @@
         <v>2044</v>
       </c>
       <c r="B26" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3761,7 +3801,7 @@
         <v>2045</v>
       </c>
       <c r="B27" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3770,7 +3810,7 @@
         <v>2046</v>
       </c>
       <c r="B28" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3779,7 +3819,7 @@
         <v>2047</v>
       </c>
       <c r="B29" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3788,7 +3828,7 @@
         <v>2048</v>
       </c>
       <c r="B30" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3797,7 +3837,7 @@
         <v>2049</v>
       </c>
       <c r="B31" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3806,7 +3846,7 @@
         <v>2050</v>
       </c>
       <c r="B32" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3815,7 +3855,7 @@
         <v>2051</v>
       </c>
       <c r="B33" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3824,7 +3864,7 @@
         <v>2052</v>
       </c>
       <c r="B34" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3833,7 +3873,7 @@
         <v>2053</v>
       </c>
       <c r="B35" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3842,7 +3882,7 @@
         <v>2054</v>
       </c>
       <c r="B36" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3851,7 +3891,7 @@
         <v>2055</v>
       </c>
       <c r="B37" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3860,7 +3900,7 @@
         <v>2056</v>
       </c>
       <c r="B38" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3869,7 +3909,7 @@
         <v>2057</v>
       </c>
       <c r="B39" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3878,7 +3918,7 @@
         <v>2058</v>
       </c>
       <c r="B40" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3887,7 +3927,7 @@
         <v>2059</v>
       </c>
       <c r="B41" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3896,7 +3936,7 @@
         <v>2060</v>
       </c>
       <c r="B42" s="0" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
     </row>
   </sheetData>
@@ -3917,7 +3957,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B60"/>
-  <sheetFormatPr defaultColWidth="10.57421875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.43"/>
@@ -4189,7 +4229,7 @@
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
-        <v>231</v>
+        <v>117</v>
       </c>
       <c r="B34" s="3" t="s">
         <v>116</v>
@@ -4197,106 +4237,106 @@
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="6" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="6" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="3" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="B39" s="3" t="s">
         <v>135</v>
-      </c>
-      <c r="B39" s="3" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="3" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="s">
-        <v>232</v>
+        <v>171</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="3" t="s">
-        <v>233</v>
+        <v>174</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="6" t="s">
-        <v>234</v>
+        <v>179</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="6" t="s">
-        <v>235</v>
+        <v>181</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="6" t="s">
-        <v>236</v>
+        <v>182</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="6" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4304,7 +4344,7 @@
         <v>237</v>
       </c>
       <c r="B48" s="6" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4312,95 +4352,95 @@
         <v>238</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="3" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="3" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="3" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="3" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="3" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="3" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="3" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="3" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="3" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="3" t="s">
-        <v>221</v>
+        <v>227</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>222</v>
+        <v>228</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="3" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>226</v>
+        <v>232</v>
       </c>
     </row>
   </sheetData>
@@ -4420,7 +4460,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D90"/>
-  <sheetFormatPr defaultColWidth="10.57421875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="69.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30.29"/>
@@ -5636,7 +5676,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D67"/>
-  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.15234375" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.14"/>
@@ -6343,7 +6383,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D25"/>
-  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.15234375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">

</xml_diff>

<commit_message>
tests: update `test_main_params.py` to include new mappings and adjust related resources
</commit_message>
<xml_diff>
--- a/tests/antares/resources/MAIN_PARAMS_2025.xlsx
+++ b/tests/antares/resources/MAIN_PARAMS_2025.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="PAYS" sheetId="1" state="visible" r:id="rId2"/>
@@ -16,7 +16,7 @@
     <sheet name="PEAK_PARAMS" sheetId="6" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">CLUSTER!$A$1:$D$89</definedName>
+    <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">CLUSTER!$A$1:$D$93</definedName>
     <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">PAYS!$A$1:$E$107</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1162" uniqueCount="426">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1178" uniqueCount="430">
   <si>
     <t xml:space="preserve">Nom_pays</t>
   </si>
@@ -1133,6 +1133,18 @@
   </si>
   <si>
     <t xml:space="preserve">Shale oil/old</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OtherNon-RES/Lignite/old 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OtherNon-RES/Hydrogen/CCGT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OtherNon-RES/Light oil/-</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OtherNon-RES/Hydrogen/OCGT</t>
   </si>
   <si>
     <t xml:space="preserve">RES</t>
@@ -1318,7 +1330,7 @@
     <numFmt numFmtId="165" formatCode="_-[$€-2]* #,##0.00_-;\-[$€-2]* #,##0.00_-;_-[$€-2]* \-??_-"/>
     <numFmt numFmtId="166" formatCode="0"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -1361,6 +1373,12 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="0"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1454,7 +1472,7 @@
       <alignment horizontal="right" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1484,6 +1502,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1613,9 +1635,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
-      <xdr:colOff>108720</xdr:colOff>
+      <xdr:colOff>108360</xdr:colOff>
       <xdr:row>10</xdr:row>
-      <xdr:rowOff>126720</xdr:rowOff>
+      <xdr:rowOff>126360</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1624,8 +1646,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7523640" y="905040"/>
-          <a:ext cx="7632000" cy="1031400"/>
+          <a:off x="7528680" y="905040"/>
+          <a:ext cx="7636680" cy="1031040"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1725,9 +1747,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>540720</xdr:colOff>
+      <xdr:colOff>540360</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>167400</xdr:rowOff>
+      <xdr:rowOff>167040</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1736,8 +1758,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13578120" y="402480"/>
-          <a:ext cx="8055360" cy="1031760"/>
+          <a:off x="13579920" y="402480"/>
+          <a:ext cx="8060400" cy="1031400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1823,7 +1845,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E107"/>
-  <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.5859375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="34.43"/>
@@ -3561,7 +3583,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B42"/>
-  <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.5859375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
@@ -3957,7 +3979,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B60"/>
-  <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.5859375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.43"/>
@@ -4459,8 +4481,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D90"/>
-  <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:D1048576"/>
+  <sheetFormatPr defaultColWidth="10.5859375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="69.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30.29"/>
@@ -5433,7 +5455,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="70" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="0" t="s">
         <v>243</v>
       </c>
@@ -5447,218 +5469,279 @@
         <v>363</v>
       </c>
     </row>
-    <row r="71" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="0" t="s">
+        <v>243</v>
+      </c>
+      <c r="B71" s="8" t="s">
         <v>368</v>
       </c>
-      <c r="B71" s="0" t="s">
+      <c r="C71" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="D71" s="0" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="0" t="s">
+        <v>243</v>
+      </c>
+      <c r="B72" s="8" t="s">
         <v>369</v>
       </c>
-      <c r="C71" s="0" t="s">
+      <c r="C72" s="8" t="s">
+        <v>253</v>
+      </c>
+      <c r="D72" s="0" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="0" t="s">
+        <v>243</v>
+      </c>
+      <c r="B73" s="8" t="s">
         <v>370</v>
       </c>
-    </row>
-    <row r="72" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="0" t="s">
-        <v>368</v>
-      </c>
-      <c r="B72" s="0" t="s">
+      <c r="C73" s="8" t="s">
+        <v>322</v>
+      </c>
+      <c r="D73" s="0" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="0" t="s">
+        <v>243</v>
+      </c>
+      <c r="B74" s="8" t="s">
         <v>371</v>
       </c>
-      <c r="C72" s="0" t="s">
-        <v>372</v>
-      </c>
-    </row>
-    <row r="73" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="0" t="s">
-        <v>368</v>
-      </c>
-      <c r="B73" s="0" t="s">
-        <v>373</v>
-      </c>
-      <c r="C73" s="0" t="s">
-        <v>372</v>
-      </c>
-    </row>
-    <row r="74" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="0" t="s">
-        <v>368</v>
-      </c>
-      <c r="B74" s="0" t="s">
-        <v>374</v>
-      </c>
-      <c r="C74" s="0" t="s">
-        <v>375</v>
+      <c r="C74" s="8" t="s">
+        <v>346</v>
+      </c>
+      <c r="D74" s="0" t="s">
+        <v>323</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="0" t="s">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="B75" s="0" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="C75" s="0" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="0" t="s">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="B76" s="0" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="C76" s="0" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="0" t="s">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="B77" s="0" t="s">
+        <v>377</v>
+      </c>
+      <c r="C77" s="0" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="0" t="s">
+        <v>372</v>
+      </c>
+      <c r="B78" s="0" t="s">
+        <v>378</v>
+      </c>
+      <c r="C78" s="0" t="s">
         <v>379</v>
       </c>
-      <c r="C77" s="0" t="s">
-        <v>378</v>
-      </c>
-    </row>
-    <row r="78" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="0" t="s">
-        <v>368</v>
-      </c>
-      <c r="B78" s="0" t="s">
+    </row>
+    <row r="79" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="0" t="s">
+        <v>372</v>
+      </c>
+      <c r="B79" s="0" t="s">
         <v>380</v>
       </c>
-      <c r="C78" s="0" t="s">
-        <v>378</v>
-      </c>
-    </row>
-    <row r="79" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="0" t="s">
-        <v>368</v>
-      </c>
-      <c r="B79" s="0" t="s">
+      <c r="C79" s="0" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="0" t="s">
+        <v>372</v>
+      </c>
+      <c r="B80" s="0" t="s">
         <v>381</v>
       </c>
-      <c r="C79" s="0" t="s">
-        <v>378</v>
-      </c>
-    </row>
-    <row r="80" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="0" t="s">
+      <c r="C80" s="0" t="s">
         <v>382</v>
       </c>
-      <c r="B80" s="0" t="s">
+    </row>
+    <row r="81" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="0" t="s">
+        <v>372</v>
+      </c>
+      <c r="B81" s="0" t="s">
         <v>383</v>
       </c>
-      <c r="C80" s="0" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="81" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="0" t="s">
+      <c r="C81" s="0" t="s">
         <v>382</v>
-      </c>
-      <c r="B81" s="0" t="s">
-        <v>385</v>
-      </c>
-      <c r="C81" s="0" t="s">
-        <v>386</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="0" t="s">
+        <v>372</v>
+      </c>
+      <c r="B82" s="0" t="s">
+        <v>384</v>
+      </c>
+      <c r="C82" s="0" t="s">
         <v>382</v>
-      </c>
-      <c r="B82" s="0" t="s">
-        <v>387</v>
-      </c>
-      <c r="C82" s="0" t="s">
-        <v>388</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="0" t="s">
+        <v>372</v>
+      </c>
+      <c r="B83" s="0" t="s">
+        <v>385</v>
+      </c>
+      <c r="C83" s="0" t="s">
         <v>382</v>
-      </c>
-      <c r="B83" s="0" t="s">
-        <v>389</v>
-      </c>
-      <c r="C83" s="0" t="s">
-        <v>390</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="0" t="s">
-        <v>382</v>
+        <v>386</v>
       </c>
       <c r="B84" s="0" t="s">
-        <v>391</v>
+        <v>387</v>
       </c>
       <c r="C84" s="0" t="s">
-        <v>392</v>
+        <v>388</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="0" t="s">
-        <v>393</v>
+        <v>386</v>
       </c>
       <c r="B85" s="0" t="s">
-        <v>394</v>
+        <v>389</v>
       </c>
       <c r="C85" s="0" t="s">
-        <v>395</v>
+        <v>390</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="0" t="s">
-        <v>393</v>
+        <v>386</v>
       </c>
       <c r="B86" s="0" t="s">
-        <v>396</v>
+        <v>391</v>
       </c>
       <c r="C86" s="0" t="s">
-        <v>396</v>
+        <v>392</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="0" t="s">
+        <v>386</v>
+      </c>
+      <c r="B87" s="0" t="s">
         <v>393</v>
       </c>
-      <c r="B87" s="0" t="s">
-        <v>397</v>
-      </c>
       <c r="C87" s="0" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="0" t="s">
-        <v>393</v>
+        <v>386</v>
       </c>
       <c r="B88" s="0" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
       <c r="C88" s="0" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="0" t="s">
-        <v>393</v>
+        <v>397</v>
       </c>
       <c r="B89" s="0" t="s">
+        <v>398</v>
+      </c>
+      <c r="C89" s="0" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="0" t="s">
+        <v>397</v>
+      </c>
+      <c r="B90" s="0" t="s">
         <v>400</v>
       </c>
-      <c r="C89" s="0" t="s">
+      <c r="C90" s="0" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="0" t="s">
+        <v>397</v>
+      </c>
+      <c r="B91" s="0" t="s">
         <v>401</v>
       </c>
-    </row>
-    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+      <c r="C91" s="0" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="0" t="s">
+        <v>397</v>
+      </c>
+      <c r="B92" s="0" t="s">
+        <v>402</v>
+      </c>
+      <c r="C92" s="0" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="93" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="0" t="s">
+        <v>397</v>
+      </c>
+      <c r="B93" s="0" t="s">
+        <v>404</v>
+      </c>
+      <c r="C93" s="0" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <autoFilter ref="A1:D89"/>
+  <autoFilter ref="A1:D93"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -5676,7 +5759,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D67"/>
-  <sheetFormatPr defaultColWidth="9.15234375" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.16015625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.14"/>
@@ -5684,13 +5767,13 @@
   <sheetData>
     <row r="1" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>402</v>
+        <v>406</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>403</v>
+        <v>407</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>404</v>
+        <v>408</v>
       </c>
       <c r="D1" s="2"/>
     </row>
@@ -5702,9 +5785,9 @@
         <v>342</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>405</v>
-      </c>
-      <c r="D2" s="8"/>
+        <v>409</v>
+      </c>
+      <c r="D2" s="9"/>
     </row>
     <row r="3" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
@@ -5714,657 +5797,657 @@
         <v>342</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>406</v>
-      </c>
-      <c r="D3" s="8"/>
+        <v>410</v>
+      </c>
+      <c r="D3" s="9"/>
     </row>
     <row r="4" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
         <v>304</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>407</v>
+        <v>411</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>408</v>
-      </c>
-      <c r="D4" s="8"/>
+        <v>412</v>
+      </c>
+      <c r="D4" s="9"/>
     </row>
     <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
         <v>307</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>407</v>
+        <v>411</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>408</v>
-      </c>
-      <c r="D5" s="8"/>
+        <v>412</v>
+      </c>
+      <c r="D5" s="9"/>
     </row>
     <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
         <v>309</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>407</v>
+        <v>411</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>409</v>
-      </c>
-      <c r="D6" s="8"/>
+        <v>413</v>
+      </c>
+      <c r="D6" s="9"/>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
         <v>311</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>407</v>
+        <v>411</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>409</v>
-      </c>
-      <c r="D7" s="8"/>
+        <v>413</v>
+      </c>
+      <c r="D7" s="9"/>
     </row>
     <row r="8" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
         <v>299</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>407</v>
+        <v>411</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>410</v>
-      </c>
-      <c r="D8" s="8"/>
+        <v>414</v>
+      </c>
+      <c r="D8" s="9"/>
     </row>
     <row r="9" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
         <v>302</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>407</v>
+        <v>411</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>410</v>
-      </c>
-      <c r="D9" s="8"/>
+        <v>414</v>
+      </c>
+      <c r="D9" s="9"/>
     </row>
     <row r="10" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
         <v>333</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>411</v>
+        <v>415</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>408</v>
-      </c>
-      <c r="D10" s="8"/>
+        <v>412</v>
+      </c>
+      <c r="D10" s="9"/>
     </row>
     <row r="11" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
         <v>335</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>411</v>
+        <v>415</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>408</v>
-      </c>
-      <c r="D11" s="8"/>
+        <v>412</v>
+      </c>
+      <c r="D11" s="9"/>
     </row>
     <row r="12" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
         <v>338</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>411</v>
+        <v>415</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>409</v>
-      </c>
-      <c r="D12" s="8"/>
+        <v>413</v>
+      </c>
+      <c r="D12" s="9"/>
     </row>
     <row r="13" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
         <v>340</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>411</v>
+        <v>415</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>409</v>
-      </c>
-      <c r="D13" s="8"/>
+        <v>413</v>
+      </c>
+      <c r="D13" s="9"/>
     </row>
     <row r="14" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
         <v>328</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>411</v>
+        <v>415</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>410</v>
-      </c>
-      <c r="D14" s="8"/>
+        <v>414</v>
+      </c>
+      <c r="D14" s="9"/>
     </row>
     <row r="15" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
         <v>331</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>411</v>
+        <v>415</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>410</v>
-      </c>
-      <c r="D15" s="8"/>
+        <v>414</v>
+      </c>
+      <c r="D15" s="9"/>
     </row>
     <row r="16" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
         <v>286</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>413</v>
-      </c>
-      <c r="D16" s="8"/>
+        <v>417</v>
+      </c>
+      <c r="D16" s="9"/>
     </row>
     <row r="17" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
         <v>290</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>413</v>
-      </c>
-      <c r="D17" s="8"/>
+        <v>417</v>
+      </c>
+      <c r="D17" s="9"/>
     </row>
     <row r="18" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
         <v>293</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>414</v>
-      </c>
-      <c r="D18" s="8"/>
+        <v>418</v>
+      </c>
+      <c r="D18" s="9"/>
     </row>
     <row r="19" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
         <v>296</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>414</v>
-      </c>
-      <c r="D19" s="8"/>
+        <v>418</v>
+      </c>
+      <c r="D19" s="9"/>
     </row>
     <row r="20" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
         <v>263</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>263</v>
       </c>
-      <c r="D20" s="8"/>
+      <c r="D20" s="9"/>
     </row>
     <row r="21" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
         <v>266</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>263</v>
       </c>
-      <c r="D21" s="8"/>
+      <c r="D21" s="9"/>
     </row>
     <row r="22" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
         <v>269</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="C22" s="3" t="s">
         <v>269</v>
       </c>
-      <c r="D22" s="8"/>
+      <c r="D22" s="9"/>
     </row>
     <row r="23" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
         <v>272</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>269</v>
       </c>
-      <c r="D23" s="8"/>
+      <c r="D23" s="9"/>
     </row>
     <row r="24" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
         <v>275</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>275</v>
       </c>
-      <c r="D24" s="8"/>
+      <c r="D24" s="9"/>
     </row>
     <row r="25" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
         <v>277</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>275</v>
       </c>
-      <c r="D25" s="8"/>
+      <c r="D25" s="9"/>
     </row>
     <row r="26" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
         <v>279</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>279</v>
       </c>
-      <c r="D26" s="8"/>
+      <c r="D26" s="9"/>
     </row>
     <row r="27" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
         <v>282</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="C27" s="3" t="s">
         <v>279</v>
       </c>
-      <c r="D27" s="8"/>
+      <c r="D27" s="9"/>
     </row>
     <row r="28" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
         <v>258</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="C28" s="3" t="s">
         <v>258</v>
       </c>
-      <c r="D28" s="8"/>
+      <c r="D28" s="9"/>
     </row>
     <row r="29" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
         <v>261</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="C29" s="3" t="s">
         <v>258</v>
       </c>
-      <c r="D29" s="8"/>
+      <c r="D29" s="9"/>
     </row>
     <row r="30" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
         <v>245</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="C30" s="3" t="s">
         <v>245</v>
       </c>
-      <c r="D30" s="8"/>
+      <c r="D30" s="9"/>
     </row>
     <row r="31" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
         <v>249</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="C31" s="3" t="s">
         <v>245</v>
       </c>
-      <c r="D31" s="8"/>
+      <c r="D31" s="9"/>
     </row>
     <row r="32" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
         <v>356</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="C32" s="3" t="s">
         <v>356</v>
       </c>
-      <c r="D32" s="8"/>
+      <c r="D32" s="9"/>
     </row>
     <row r="33" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
         <v>359</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="C33" s="3" t="s">
         <v>356</v>
       </c>
-      <c r="D33" s="8"/>
+      <c r="D33" s="9"/>
     </row>
     <row r="34" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
         <v>351</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="C34" s="3" t="s">
         <v>351</v>
       </c>
-      <c r="D34" s="8"/>
+      <c r="D34" s="9"/>
     </row>
     <row r="35" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
         <v>354</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="C35" s="3" t="s">
         <v>351</v>
       </c>
-      <c r="D35" s="8"/>
+      <c r="D35" s="9"/>
     </row>
     <row r="36" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
         <v>322</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>415</v>
+        <v>419</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>405</v>
-      </c>
-      <c r="D36" s="8"/>
+        <v>409</v>
+      </c>
+      <c r="D36" s="9"/>
     </row>
     <row r="37" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="3" t="s">
         <v>325</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>415</v>
+        <v>419</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>405</v>
-      </c>
-      <c r="D37" s="8"/>
+        <v>409</v>
+      </c>
+      <c r="D37" s="9"/>
     </row>
     <row r="38" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">
         <v>313</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>415</v>
+        <v>419</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>408</v>
-      </c>
-      <c r="D38" s="8"/>
+        <v>412</v>
+      </c>
+      <c r="D38" s="9"/>
     </row>
     <row r="39" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="3" t="s">
         <v>316</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>415</v>
+        <v>419</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>408</v>
-      </c>
-      <c r="D39" s="8"/>
+        <v>412</v>
+      </c>
+      <c r="D39" s="9"/>
     </row>
     <row r="40" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
         <v>318</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>415</v>
+        <v>419</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>409</v>
-      </c>
-      <c r="D40" s="8"/>
+        <v>413</v>
+      </c>
+      <c r="D40" s="9"/>
     </row>
     <row r="41" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="3" t="s">
         <v>320</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>415</v>
+        <v>419</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>409</v>
-      </c>
-      <c r="D41" s="8"/>
+        <v>413</v>
+      </c>
+      <c r="D41" s="9"/>
     </row>
     <row r="42" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="s">
         <v>365</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>415</v>
+        <v>419</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>416</v>
-      </c>
-      <c r="D42" s="8"/>
+        <v>420</v>
+      </c>
+      <c r="D42" s="9"/>
     </row>
     <row r="43" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="3" t="s">
         <v>362</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>415</v>
+        <v>419</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>410</v>
-      </c>
-      <c r="D43" s="8"/>
+        <v>414</v>
+      </c>
+      <c r="D43" s="9"/>
     </row>
     <row r="44" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="3" t="s">
         <v>253</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>417</v>
+        <v>421</v>
       </c>
       <c r="C44" s="3" t="s">
         <v>258</v>
       </c>
-      <c r="D44" s="8"/>
+      <c r="D44" s="9"/>
     </row>
     <row r="45" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="3" t="s">
         <v>255</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>417</v>
+        <v>421</v>
       </c>
       <c r="C45" s="3" t="s">
         <v>258</v>
       </c>
-      <c r="D45" s="8"/>
+      <c r="D45" s="9"/>
     </row>
     <row r="46" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="3" t="s">
         <v>346</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>417</v>
+        <v>421</v>
       </c>
       <c r="C46" s="3" t="s">
         <v>351</v>
       </c>
-      <c r="D46" s="8"/>
+      <c r="D46" s="9"/>
     </row>
     <row r="47" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="3" t="s">
         <v>348</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>417</v>
+        <v>421</v>
       </c>
       <c r="C47" s="3" t="s">
         <v>351</v>
       </c>
-      <c r="D47" s="8"/>
+      <c r="D47" s="9"/>
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="3"/>
-      <c r="B48" s="8"/>
+      <c r="B48" s="9"/>
       <c r="C48" s="3"/>
-      <c r="D48" s="8"/>
+      <c r="D48" s="9"/>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="3"/>
-      <c r="B49" s="8"/>
+      <c r="B49" s="9"/>
       <c r="C49" s="3"/>
-      <c r="D49" s="8"/>
+      <c r="D49" s="9"/>
     </row>
     <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="3"/>
-      <c r="B50" s="8"/>
+      <c r="B50" s="9"/>
       <c r="C50" s="3"/>
-      <c r="D50" s="8"/>
+      <c r="D50" s="9"/>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="3"/>
-      <c r="B51" s="8"/>
+      <c r="B51" s="9"/>
       <c r="C51" s="3"/>
-      <c r="D51" s="8"/>
+      <c r="D51" s="9"/>
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="3"/>
-      <c r="B52" s="8"/>
+      <c r="B52" s="9"/>
       <c r="C52" s="3"/>
-      <c r="D52" s="8"/>
+      <c r="D52" s="9"/>
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="3"/>
-      <c r="B53" s="8"/>
+      <c r="B53" s="9"/>
       <c r="C53" s="3"/>
-      <c r="D53" s="8"/>
+      <c r="D53" s="9"/>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="3"/>
-      <c r="B54" s="8"/>
+      <c r="B54" s="9"/>
       <c r="C54" s="3"/>
-      <c r="D54" s="8"/>
+      <c r="D54" s="9"/>
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="3"/>
-      <c r="B55" s="8"/>
+      <c r="B55" s="9"/>
       <c r="C55" s="3"/>
-      <c r="D55" s="8"/>
+      <c r="D55" s="9"/>
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="3"/>
-      <c r="B56" s="8"/>
+      <c r="B56" s="9"/>
       <c r="C56" s="3"/>
-      <c r="D56" s="8"/>
+      <c r="D56" s="9"/>
     </row>
     <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="3"/>
-      <c r="B57" s="8"/>
+      <c r="B57" s="9"/>
       <c r="C57" s="3"/>
-      <c r="D57" s="8"/>
+      <c r="D57" s="9"/>
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="3"/>
-      <c r="B58" s="8"/>
+      <c r="B58" s="9"/>
       <c r="C58" s="3"/>
-      <c r="D58" s="8"/>
+      <c r="D58" s="9"/>
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="3"/>
-      <c r="B59" s="8"/>
+      <c r="B59" s="9"/>
       <c r="C59" s="3"/>
-      <c r="D59" s="8"/>
+      <c r="D59" s="9"/>
     </row>
     <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="3"/>
-      <c r="B60" s="8"/>
+      <c r="B60" s="9"/>
       <c r="C60" s="3"/>
-      <c r="D60" s="8"/>
+      <c r="D60" s="9"/>
     </row>
     <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="3"/>
-      <c r="B61" s="8"/>
+      <c r="B61" s="9"/>
       <c r="C61" s="3"/>
-      <c r="D61" s="8"/>
+      <c r="D61" s="9"/>
     </row>
     <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="3"/>
-      <c r="B62" s="8"/>
+      <c r="B62" s="9"/>
       <c r="C62" s="3"/>
-      <c r="D62" s="8"/>
+      <c r="D62" s="9"/>
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="3"/>
-      <c r="B63" s="8"/>
+      <c r="B63" s="9"/>
       <c r="C63" s="3"/>
-      <c r="D63" s="8"/>
+      <c r="D63" s="9"/>
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="3"/>
-      <c r="B64" s="8"/>
+      <c r="B64" s="9"/>
       <c r="C64" s="3"/>
-      <c r="D64" s="8"/>
+      <c r="D64" s="9"/>
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="3"/>
-      <c r="B65" s="8"/>
+      <c r="B65" s="9"/>
       <c r="C65" s="3"/>
-      <c r="D65" s="8"/>
+      <c r="D65" s="9"/>
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="3"/>
-      <c r="B66" s="8"/>
+      <c r="B66" s="9"/>
       <c r="C66" s="3"/>
-      <c r="D66" s="8"/>
+      <c r="D66" s="9"/>
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="3"/>
-      <c r="B67" s="8"/>
+      <c r="B67" s="9"/>
       <c r="C67" s="3"/>
-      <c r="D67" s="8"/>
+      <c r="D67" s="9"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -6383,309 +6466,309 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D25"/>
-  <sheetFormatPr defaultColWidth="9.15234375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.16015625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="9" t="s">
-        <v>418</v>
-      </c>
-      <c r="B1" s="9" t="s">
-        <v>419</v>
-      </c>
-      <c r="C1" s="9" t="s">
-        <v>420</v>
-      </c>
-      <c r="D1" s="9" t="s">
-        <v>421</v>
+      <c r="A1" s="10" t="s">
+        <v>422</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>423</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>424</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>425</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="10" t="n">
+      <c r="A2" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="10" t="s">
-        <v>422</v>
-      </c>
-      <c r="C2" s="10" t="n">
+      <c r="B2" s="11" t="s">
+        <v>426</v>
+      </c>
+      <c r="C2" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="D2" s="10" t="s">
-        <v>423</v>
+      <c r="D2" s="11" t="s">
+        <v>427</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="10" t="n">
+      <c r="A3" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="10" t="s">
-        <v>422</v>
-      </c>
-      <c r="C3" s="10" t="n">
+      <c r="B3" s="11" t="s">
+        <v>426</v>
+      </c>
+      <c r="C3" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="D3" s="10" t="s">
-        <v>423</v>
+      <c r="D3" s="11" t="s">
+        <v>427</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="10" t="n">
+      <c r="A4" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="10" t="s">
-        <v>422</v>
-      </c>
-      <c r="C4" s="10" t="n">
+      <c r="B4" s="11" t="s">
+        <v>426</v>
+      </c>
+      <c r="C4" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="D4" s="10" t="s">
-        <v>423</v>
+      <c r="D4" s="11" t="s">
+        <v>427</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="10" t="n">
+      <c r="A5" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="10" t="s">
-        <v>422</v>
-      </c>
-      <c r="C5" s="10" t="n">
+      <c r="B5" s="11" t="s">
+        <v>426</v>
+      </c>
+      <c r="C5" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="D5" s="10" t="s">
-        <v>424</v>
+      <c r="D5" s="11" t="s">
+        <v>428</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="10" t="n">
+      <c r="A6" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="10" t="s">
-        <v>422</v>
-      </c>
-      <c r="C6" s="10" t="n">
+      <c r="B6" s="11" t="s">
+        <v>426</v>
+      </c>
+      <c r="C6" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="D6" s="10" t="s">
-        <v>424</v>
+      <c r="D6" s="11" t="s">
+        <v>428</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="10" t="n">
+      <c r="A7" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="10" t="s">
-        <v>422</v>
-      </c>
-      <c r="C7" s="10" t="n">
+      <c r="B7" s="11" t="s">
+        <v>426</v>
+      </c>
+      <c r="C7" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="D7" s="10" t="s">
-        <v>424</v>
+      <c r="D7" s="11" t="s">
+        <v>428</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="n">
+      <c r="A8" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="10" t="s">
-        <v>422</v>
-      </c>
-      <c r="C8" s="10" t="n">
+      <c r="B8" s="11" t="s">
+        <v>426</v>
+      </c>
+      <c r="C8" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="D8" s="10" t="s">
-        <v>424</v>
+      <c r="D8" s="11" t="s">
+        <v>428</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="10" t="n">
+      <c r="A9" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="10" t="s">
-        <v>422</v>
-      </c>
-      <c r="C9" s="10" t="n">
+      <c r="B9" s="11" t="s">
+        <v>426</v>
+      </c>
+      <c r="C9" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="D9" s="10" t="s">
-        <v>424</v>
+      <c r="D9" s="11" t="s">
+        <v>428</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10" t="n">
+      <c r="A10" s="11" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="10" t="s">
-        <v>425</v>
-      </c>
-      <c r="C10" s="10" t="n">
+      <c r="B10" s="11" t="s">
+        <v>429</v>
+      </c>
+      <c r="C10" s="11" t="n">
         <v>9</v>
       </c>
-      <c r="D10" s="10" t="s">
-        <v>424</v>
+      <c r="D10" s="11" t="s">
+        <v>428</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="10" t="n">
+      <c r="A11" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="10" t="s">
-        <v>425</v>
-      </c>
-      <c r="C11" s="10" t="n">
+      <c r="B11" s="11" t="s">
+        <v>429</v>
+      </c>
+      <c r="C11" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="D11" s="10" t="s">
-        <v>423</v>
+      <c r="D11" s="11" t="s">
+        <v>427</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="10" t="n">
+      <c r="A12" s="11" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="10" t="s">
-        <v>425</v>
-      </c>
-      <c r="C12" s="10" t="n">
+      <c r="B12" s="11" t="s">
+        <v>429</v>
+      </c>
+      <c r="C12" s="11" t="n">
         <v>11</v>
       </c>
-      <c r="D12" s="10" t="s">
-        <v>423</v>
+      <c r="D12" s="11" t="s">
+        <v>427</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="10" t="n">
+      <c r="A13" s="11" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="10" t="s">
-        <v>425</v>
-      </c>
-      <c r="C13" s="10" t="n">
+      <c r="B13" s="11" t="s">
+        <v>429</v>
+      </c>
+      <c r="C13" s="11" t="n">
         <v>12</v>
       </c>
-      <c r="D13" s="10" t="s">
-        <v>423</v>
+      <c r="D13" s="11" t="s">
+        <v>427</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="10" t="n">
+      <c r="A14" s="11" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="10" t="s">
-        <v>425</v>
-      </c>
-      <c r="C14" s="10"/>
-      <c r="D14" s="10"/>
+      <c r="B14" s="11" t="s">
+        <v>429</v>
+      </c>
+      <c r="C14" s="11"/>
+      <c r="D14" s="11"/>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="10" t="n">
+      <c r="A15" s="11" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="10" t="s">
-        <v>425</v>
-      </c>
-      <c r="C15" s="10"/>
-      <c r="D15" s="10"/>
+      <c r="B15" s="11" t="s">
+        <v>429</v>
+      </c>
+      <c r="C15" s="11"/>
+      <c r="D15" s="11"/>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="10" t="n">
+      <c r="A16" s="11" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="10" t="s">
-        <v>425</v>
-      </c>
-      <c r="C16" s="10"/>
-      <c r="D16" s="10"/>
+      <c r="B16" s="11" t="s">
+        <v>429</v>
+      </c>
+      <c r="C16" s="11"/>
+      <c r="D16" s="11"/>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="10" t="n">
+      <c r="A17" s="11" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="10" t="s">
-        <v>425</v>
-      </c>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
+      <c r="B17" s="11" t="s">
+        <v>429</v>
+      </c>
+      <c r="C17" s="11"/>
+      <c r="D17" s="11"/>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="10" t="n">
+      <c r="A18" s="11" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="10" t="s">
-        <v>425</v>
-      </c>
-      <c r="C18" s="10"/>
-      <c r="D18" s="10"/>
+      <c r="B18" s="11" t="s">
+        <v>429</v>
+      </c>
+      <c r="C18" s="11"/>
+      <c r="D18" s="11"/>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="10" t="n">
+      <c r="A19" s="11" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="10" t="s">
-        <v>425</v>
-      </c>
-      <c r="C19" s="10"/>
-      <c r="D19" s="10"/>
+      <c r="B19" s="11" t="s">
+        <v>429</v>
+      </c>
+      <c r="C19" s="11"/>
+      <c r="D19" s="11"/>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="10" t="n">
+      <c r="A20" s="11" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="10" t="s">
-        <v>425</v>
-      </c>
-      <c r="C20" s="10"/>
-      <c r="D20" s="10"/>
+      <c r="B20" s="11" t="s">
+        <v>429</v>
+      </c>
+      <c r="C20" s="11"/>
+      <c r="D20" s="11"/>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="10" t="n">
+      <c r="A21" s="11" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="10" t="s">
-        <v>425</v>
-      </c>
-      <c r="C21" s="10"/>
-      <c r="D21" s="10"/>
+      <c r="B21" s="11" t="s">
+        <v>429</v>
+      </c>
+      <c r="C21" s="11"/>
+      <c r="D21" s="11"/>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="10" t="n">
+      <c r="A22" s="11" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="10" t="s">
-        <v>422</v>
-      </c>
-      <c r="C22" s="10"/>
-      <c r="D22" s="10"/>
+      <c r="B22" s="11" t="s">
+        <v>426</v>
+      </c>
+      <c r="C22" s="11"/>
+      <c r="D22" s="11"/>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="10" t="n">
+      <c r="A23" s="11" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="10" t="s">
-        <v>422</v>
-      </c>
-      <c r="C23" s="10"/>
-      <c r="D23" s="10"/>
+      <c r="B23" s="11" t="s">
+        <v>426</v>
+      </c>
+      <c r="C23" s="11"/>
+      <c r="D23" s="11"/>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="10" t="n">
+      <c r="A24" s="11" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="10" t="s">
-        <v>422</v>
-      </c>
-      <c r="C24" s="10"/>
-      <c r="D24" s="10"/>
+      <c r="B24" s="11" t="s">
+        <v>426</v>
+      </c>
+      <c r="C24" s="11"/>
+      <c r="D24" s="11"/>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="10" t="n">
+      <c r="A25" s="11" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="10" t="s">
-        <v>422</v>
-      </c>
-      <c r="C25" s="10"/>
-      <c r="D25" s="10"/>
+      <c r="B25" s="11" t="s">
+        <v>426</v>
+      </c>
+      <c r="C25" s="11"/>
+      <c r="D25" s="11"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
tests: update `test_main_params.py` to include new mappings and adjust related resources (#36)
</commit_message>
<xml_diff>
--- a/tests/antares/resources/MAIN_PARAMS_2025.xlsx
+++ b/tests/antares/resources/MAIN_PARAMS_2025.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="PAYS" sheetId="1" state="visible" r:id="rId2"/>
@@ -16,7 +16,7 @@
     <sheet name="PEAK_PARAMS" sheetId="6" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">CLUSTER!$A$1:$D$89</definedName>
+    <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">CLUSTER!$A$1:$D$93</definedName>
     <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">PAYS!$A$1:$E$107</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1162" uniqueCount="426">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1178" uniqueCount="430">
   <si>
     <t xml:space="preserve">Nom_pays</t>
   </si>
@@ -1133,6 +1133,18 @@
   </si>
   <si>
     <t xml:space="preserve">Shale oil/old</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OtherNon-RES/Lignite/old 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OtherNon-RES/Hydrogen/CCGT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OtherNon-RES/Light oil/-</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OtherNon-RES/Hydrogen/OCGT</t>
   </si>
   <si>
     <t xml:space="preserve">RES</t>
@@ -1318,7 +1330,7 @@
     <numFmt numFmtId="165" formatCode="_-[$€-2]* #,##0.00_-;\-[$€-2]* #,##0.00_-;_-[$€-2]* \-??_-"/>
     <numFmt numFmtId="166" formatCode="0"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -1361,6 +1373,12 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="0"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1454,7 +1472,7 @@
       <alignment horizontal="right" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1484,6 +1502,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1613,9 +1635,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
-      <xdr:colOff>108720</xdr:colOff>
+      <xdr:colOff>108360</xdr:colOff>
       <xdr:row>10</xdr:row>
-      <xdr:rowOff>126720</xdr:rowOff>
+      <xdr:rowOff>126360</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1624,8 +1646,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7523640" y="905040"/>
-          <a:ext cx="7632000" cy="1031400"/>
+          <a:off x="7528680" y="905040"/>
+          <a:ext cx="7636680" cy="1031040"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1725,9 +1747,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>540720</xdr:colOff>
+      <xdr:colOff>540360</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>167400</xdr:rowOff>
+      <xdr:rowOff>167040</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1736,8 +1758,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13578120" y="402480"/>
-          <a:ext cx="8055360" cy="1031760"/>
+          <a:off x="13579920" y="402480"/>
+          <a:ext cx="8060400" cy="1031400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1823,7 +1845,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E107"/>
-  <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.5859375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="34.43"/>
@@ -3561,7 +3583,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B42"/>
-  <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.5859375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
@@ -3957,7 +3979,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B60"/>
-  <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.5859375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.43"/>
@@ -4459,8 +4481,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D90"/>
-  <sheetFormatPr defaultColWidth="10.58203125" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:D1048576"/>
+  <sheetFormatPr defaultColWidth="10.5859375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="69.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30.29"/>
@@ -5433,7 +5455,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="70" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="0" t="s">
         <v>243</v>
       </c>
@@ -5447,218 +5469,279 @@
         <v>363</v>
       </c>
     </row>
-    <row r="71" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="0" t="s">
+        <v>243</v>
+      </c>
+      <c r="B71" s="8" t="s">
         <v>368</v>
       </c>
-      <c r="B71" s="0" t="s">
+      <c r="C71" s="8" t="s">
+        <v>333</v>
+      </c>
+      <c r="D71" s="0" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="0" t="s">
+        <v>243</v>
+      </c>
+      <c r="B72" s="8" t="s">
         <v>369</v>
       </c>
-      <c r="C71" s="0" t="s">
+      <c r="C72" s="8" t="s">
+        <v>253</v>
+      </c>
+      <c r="D72" s="0" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="0" t="s">
+        <v>243</v>
+      </c>
+      <c r="B73" s="8" t="s">
         <v>370</v>
       </c>
-    </row>
-    <row r="72" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="0" t="s">
-        <v>368</v>
-      </c>
-      <c r="B72" s="0" t="s">
+      <c r="C73" s="8" t="s">
+        <v>322</v>
+      </c>
+      <c r="D73" s="0" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="0" t="s">
+        <v>243</v>
+      </c>
+      <c r="B74" s="8" t="s">
         <v>371</v>
       </c>
-      <c r="C72" s="0" t="s">
-        <v>372</v>
-      </c>
-    </row>
-    <row r="73" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="0" t="s">
-        <v>368</v>
-      </c>
-      <c r="B73" s="0" t="s">
-        <v>373</v>
-      </c>
-      <c r="C73" s="0" t="s">
-        <v>372</v>
-      </c>
-    </row>
-    <row r="74" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="0" t="s">
-        <v>368</v>
-      </c>
-      <c r="B74" s="0" t="s">
-        <v>374</v>
-      </c>
-      <c r="C74" s="0" t="s">
-        <v>375</v>
+      <c r="C74" s="8" t="s">
+        <v>346</v>
+      </c>
+      <c r="D74" s="0" t="s">
+        <v>323</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="0" t="s">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="B75" s="0" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="C75" s="0" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="0" t="s">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="B76" s="0" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="C76" s="0" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="0" t="s">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="B77" s="0" t="s">
+        <v>377</v>
+      </c>
+      <c r="C77" s="0" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="0" t="s">
+        <v>372</v>
+      </c>
+      <c r="B78" s="0" t="s">
+        <v>378</v>
+      </c>
+      <c r="C78" s="0" t="s">
         <v>379</v>
       </c>
-      <c r="C77" s="0" t="s">
-        <v>378</v>
-      </c>
-    </row>
-    <row r="78" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="0" t="s">
-        <v>368</v>
-      </c>
-      <c r="B78" s="0" t="s">
+    </row>
+    <row r="79" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="0" t="s">
+        <v>372</v>
+      </c>
+      <c r="B79" s="0" t="s">
         <v>380</v>
       </c>
-      <c r="C78" s="0" t="s">
-        <v>378</v>
-      </c>
-    </row>
-    <row r="79" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="0" t="s">
-        <v>368</v>
-      </c>
-      <c r="B79" s="0" t="s">
+      <c r="C79" s="0" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="0" t="s">
+        <v>372</v>
+      </c>
+      <c r="B80" s="0" t="s">
         <v>381</v>
       </c>
-      <c r="C79" s="0" t="s">
-        <v>378</v>
-      </c>
-    </row>
-    <row r="80" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="0" t="s">
+      <c r="C80" s="0" t="s">
         <v>382</v>
       </c>
-      <c r="B80" s="0" t="s">
+    </row>
+    <row r="81" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="0" t="s">
+        <v>372</v>
+      </c>
+      <c r="B81" s="0" t="s">
         <v>383</v>
       </c>
-      <c r="C80" s="0" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="81" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="0" t="s">
+      <c r="C81" s="0" t="s">
         <v>382</v>
-      </c>
-      <c r="B81" s="0" t="s">
-        <v>385</v>
-      </c>
-      <c r="C81" s="0" t="s">
-        <v>386</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="0" t="s">
+        <v>372</v>
+      </c>
+      <c r="B82" s="0" t="s">
+        <v>384</v>
+      </c>
+      <c r="C82" s="0" t="s">
         <v>382</v>
-      </c>
-      <c r="B82" s="0" t="s">
-        <v>387</v>
-      </c>
-      <c r="C82" s="0" t="s">
-        <v>388</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="0" t="s">
+        <v>372</v>
+      </c>
+      <c r="B83" s="0" t="s">
+        <v>385</v>
+      </c>
+      <c r="C83" s="0" t="s">
         <v>382</v>
-      </c>
-      <c r="B83" s="0" t="s">
-        <v>389</v>
-      </c>
-      <c r="C83" s="0" t="s">
-        <v>390</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="0" t="s">
-        <v>382</v>
+        <v>386</v>
       </c>
       <c r="B84" s="0" t="s">
-        <v>391</v>
+        <v>387</v>
       </c>
       <c r="C84" s="0" t="s">
-        <v>392</v>
+        <v>388</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="0" t="s">
-        <v>393</v>
+        <v>386</v>
       </c>
       <c r="B85" s="0" t="s">
-        <v>394</v>
+        <v>389</v>
       </c>
       <c r="C85" s="0" t="s">
-        <v>395</v>
+        <v>390</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="0" t="s">
-        <v>393</v>
+        <v>386</v>
       </c>
       <c r="B86" s="0" t="s">
-        <v>396</v>
+        <v>391</v>
       </c>
       <c r="C86" s="0" t="s">
-        <v>396</v>
+        <v>392</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="0" t="s">
+        <v>386</v>
+      </c>
+      <c r="B87" s="0" t="s">
         <v>393</v>
       </c>
-      <c r="B87" s="0" t="s">
-        <v>397</v>
-      </c>
       <c r="C87" s="0" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="0" t="s">
-        <v>393</v>
+        <v>386</v>
       </c>
       <c r="B88" s="0" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
       <c r="C88" s="0" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="0" t="s">
-        <v>393</v>
+        <v>397</v>
       </c>
       <c r="B89" s="0" t="s">
+        <v>398</v>
+      </c>
+      <c r="C89" s="0" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="0" t="s">
+        <v>397</v>
+      </c>
+      <c r="B90" s="0" t="s">
         <v>400</v>
       </c>
-      <c r="C89" s="0" t="s">
+      <c r="C90" s="0" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="0" t="s">
+        <v>397</v>
+      </c>
+      <c r="B91" s="0" t="s">
         <v>401</v>
       </c>
-    </row>
-    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+      <c r="C91" s="0" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="0" t="s">
+        <v>397</v>
+      </c>
+      <c r="B92" s="0" t="s">
+        <v>402</v>
+      </c>
+      <c r="C92" s="0" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="93" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="0" t="s">
+        <v>397</v>
+      </c>
+      <c r="B93" s="0" t="s">
+        <v>404</v>
+      </c>
+      <c r="C93" s="0" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <autoFilter ref="A1:D89"/>
+  <autoFilter ref="A1:D93"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -5676,7 +5759,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D67"/>
-  <sheetFormatPr defaultColWidth="9.15234375" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.16015625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.14"/>
@@ -5684,13 +5767,13 @@
   <sheetData>
     <row r="1" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>402</v>
+        <v>406</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>403</v>
+        <v>407</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>404</v>
+        <v>408</v>
       </c>
       <c r="D1" s="2"/>
     </row>
@@ -5702,9 +5785,9 @@
         <v>342</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>405</v>
-      </c>
-      <c r="D2" s="8"/>
+        <v>409</v>
+      </c>
+      <c r="D2" s="9"/>
     </row>
     <row r="3" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
@@ -5714,657 +5797,657 @@
         <v>342</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>406</v>
-      </c>
-      <c r="D3" s="8"/>
+        <v>410</v>
+      </c>
+      <c r="D3" s="9"/>
     </row>
     <row r="4" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
         <v>304</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>407</v>
+        <v>411</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>408</v>
-      </c>
-      <c r="D4" s="8"/>
+        <v>412</v>
+      </c>
+      <c r="D4" s="9"/>
     </row>
     <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
         <v>307</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>407</v>
+        <v>411</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>408</v>
-      </c>
-      <c r="D5" s="8"/>
+        <v>412</v>
+      </c>
+      <c r="D5" s="9"/>
     </row>
     <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
         <v>309</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>407</v>
+        <v>411</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>409</v>
-      </c>
-      <c r="D6" s="8"/>
+        <v>413</v>
+      </c>
+      <c r="D6" s="9"/>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
         <v>311</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>407</v>
+        <v>411</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>409</v>
-      </c>
-      <c r="D7" s="8"/>
+        <v>413</v>
+      </c>
+      <c r="D7" s="9"/>
     </row>
     <row r="8" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
         <v>299</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>407</v>
+        <v>411</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>410</v>
-      </c>
-      <c r="D8" s="8"/>
+        <v>414</v>
+      </c>
+      <c r="D8" s="9"/>
     </row>
     <row r="9" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
         <v>302</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>407</v>
+        <v>411</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>410</v>
-      </c>
-      <c r="D9" s="8"/>
+        <v>414</v>
+      </c>
+      <c r="D9" s="9"/>
     </row>
     <row r="10" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
         <v>333</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>411</v>
+        <v>415</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>408</v>
-      </c>
-      <c r="D10" s="8"/>
+        <v>412</v>
+      </c>
+      <c r="D10" s="9"/>
     </row>
     <row r="11" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
         <v>335</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>411</v>
+        <v>415</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>408</v>
-      </c>
-      <c r="D11" s="8"/>
+        <v>412</v>
+      </c>
+      <c r="D11" s="9"/>
     </row>
     <row r="12" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
         <v>338</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>411</v>
+        <v>415</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>409</v>
-      </c>
-      <c r="D12" s="8"/>
+        <v>413</v>
+      </c>
+      <c r="D12" s="9"/>
     </row>
     <row r="13" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
         <v>340</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>411</v>
+        <v>415</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>409</v>
-      </c>
-      <c r="D13" s="8"/>
+        <v>413</v>
+      </c>
+      <c r="D13" s="9"/>
     </row>
     <row r="14" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
         <v>328</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>411</v>
+        <v>415</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>410</v>
-      </c>
-      <c r="D14" s="8"/>
+        <v>414</v>
+      </c>
+      <c r="D14" s="9"/>
     </row>
     <row r="15" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
         <v>331</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>411</v>
+        <v>415</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>410</v>
-      </c>
-      <c r="D15" s="8"/>
+        <v>414</v>
+      </c>
+      <c r="D15" s="9"/>
     </row>
     <row r="16" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
         <v>286</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>413</v>
-      </c>
-      <c r="D16" s="8"/>
+        <v>417</v>
+      </c>
+      <c r="D16" s="9"/>
     </row>
     <row r="17" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
         <v>290</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>413</v>
-      </c>
-      <c r="D17" s="8"/>
+        <v>417</v>
+      </c>
+      <c r="D17" s="9"/>
     </row>
     <row r="18" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
         <v>293</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>414</v>
-      </c>
-      <c r="D18" s="8"/>
+        <v>418</v>
+      </c>
+      <c r="D18" s="9"/>
     </row>
     <row r="19" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
         <v>296</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>414</v>
-      </c>
-      <c r="D19" s="8"/>
+        <v>418</v>
+      </c>
+      <c r="D19" s="9"/>
     </row>
     <row r="20" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
         <v>263</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>263</v>
       </c>
-      <c r="D20" s="8"/>
+      <c r="D20" s="9"/>
     </row>
     <row r="21" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
         <v>266</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>263</v>
       </c>
-      <c r="D21" s="8"/>
+      <c r="D21" s="9"/>
     </row>
     <row r="22" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
         <v>269</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="C22" s="3" t="s">
         <v>269</v>
       </c>
-      <c r="D22" s="8"/>
+      <c r="D22" s="9"/>
     </row>
     <row r="23" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
         <v>272</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>269</v>
       </c>
-      <c r="D23" s="8"/>
+      <c r="D23" s="9"/>
     </row>
     <row r="24" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
         <v>275</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>275</v>
       </c>
-      <c r="D24" s="8"/>
+      <c r="D24" s="9"/>
     </row>
     <row r="25" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
         <v>277</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>275</v>
       </c>
-      <c r="D25" s="8"/>
+      <c r="D25" s="9"/>
     </row>
     <row r="26" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
         <v>279</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>279</v>
       </c>
-      <c r="D26" s="8"/>
+      <c r="D26" s="9"/>
     </row>
     <row r="27" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
         <v>282</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="C27" s="3" t="s">
         <v>279</v>
       </c>
-      <c r="D27" s="8"/>
+      <c r="D27" s="9"/>
     </row>
     <row r="28" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
         <v>258</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="C28" s="3" t="s">
         <v>258</v>
       </c>
-      <c r="D28" s="8"/>
+      <c r="D28" s="9"/>
     </row>
     <row r="29" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
         <v>261</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="C29" s="3" t="s">
         <v>258</v>
       </c>
-      <c r="D29" s="8"/>
+      <c r="D29" s="9"/>
     </row>
     <row r="30" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
         <v>245</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="C30" s="3" t="s">
         <v>245</v>
       </c>
-      <c r="D30" s="8"/>
+      <c r="D30" s="9"/>
     </row>
     <row r="31" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
         <v>249</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="C31" s="3" t="s">
         <v>245</v>
       </c>
-      <c r="D31" s="8"/>
+      <c r="D31" s="9"/>
     </row>
     <row r="32" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
         <v>356</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="C32" s="3" t="s">
         <v>356</v>
       </c>
-      <c r="D32" s="8"/>
+      <c r="D32" s="9"/>
     </row>
     <row r="33" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
         <v>359</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="C33" s="3" t="s">
         <v>356</v>
       </c>
-      <c r="D33" s="8"/>
+      <c r="D33" s="9"/>
     </row>
     <row r="34" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
         <v>351</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="C34" s="3" t="s">
         <v>351</v>
       </c>
-      <c r="D34" s="8"/>
+      <c r="D34" s="9"/>
     </row>
     <row r="35" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
         <v>354</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="C35" s="3" t="s">
         <v>351</v>
       </c>
-      <c r="D35" s="8"/>
+      <c r="D35" s="9"/>
     </row>
     <row r="36" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
         <v>322</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>415</v>
+        <v>419</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>405</v>
-      </c>
-      <c r="D36" s="8"/>
+        <v>409</v>
+      </c>
+      <c r="D36" s="9"/>
     </row>
     <row r="37" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="3" t="s">
         <v>325</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>415</v>
+        <v>419</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>405</v>
-      </c>
-      <c r="D37" s="8"/>
+        <v>409</v>
+      </c>
+      <c r="D37" s="9"/>
     </row>
     <row r="38" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">
         <v>313</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>415</v>
+        <v>419</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>408</v>
-      </c>
-      <c r="D38" s="8"/>
+        <v>412</v>
+      </c>
+      <c r="D38" s="9"/>
     </row>
     <row r="39" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="3" t="s">
         <v>316</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>415</v>
+        <v>419</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>408</v>
-      </c>
-      <c r="D39" s="8"/>
+        <v>412</v>
+      </c>
+      <c r="D39" s="9"/>
     </row>
     <row r="40" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
         <v>318</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>415</v>
+        <v>419</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>409</v>
-      </c>
-      <c r="D40" s="8"/>
+        <v>413</v>
+      </c>
+      <c r="D40" s="9"/>
     </row>
     <row r="41" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="3" t="s">
         <v>320</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>415</v>
+        <v>419</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>409</v>
-      </c>
-      <c r="D41" s="8"/>
+        <v>413</v>
+      </c>
+      <c r="D41" s="9"/>
     </row>
     <row r="42" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="s">
         <v>365</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>415</v>
+        <v>419</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>416</v>
-      </c>
-      <c r="D42" s="8"/>
+        <v>420</v>
+      </c>
+      <c r="D42" s="9"/>
     </row>
     <row r="43" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="3" t="s">
         <v>362</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>415</v>
+        <v>419</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>410</v>
-      </c>
-      <c r="D43" s="8"/>
+        <v>414</v>
+      </c>
+      <c r="D43" s="9"/>
     </row>
     <row r="44" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="3" t="s">
         <v>253</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>417</v>
+        <v>421</v>
       </c>
       <c r="C44" s="3" t="s">
         <v>258</v>
       </c>
-      <c r="D44" s="8"/>
+      <c r="D44" s="9"/>
     </row>
     <row r="45" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="3" t="s">
         <v>255</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>417</v>
+        <v>421</v>
       </c>
       <c r="C45" s="3" t="s">
         <v>258</v>
       </c>
-      <c r="D45" s="8"/>
+      <c r="D45" s="9"/>
     </row>
     <row r="46" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="3" t="s">
         <v>346</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>417</v>
+        <v>421</v>
       </c>
       <c r="C46" s="3" t="s">
         <v>351</v>
       </c>
-      <c r="D46" s="8"/>
+      <c r="D46" s="9"/>
     </row>
     <row r="47" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="3" t="s">
         <v>348</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>417</v>
+        <v>421</v>
       </c>
       <c r="C47" s="3" t="s">
         <v>351</v>
       </c>
-      <c r="D47" s="8"/>
+      <c r="D47" s="9"/>
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="3"/>
-      <c r="B48" s="8"/>
+      <c r="B48" s="9"/>
       <c r="C48" s="3"/>
-      <c r="D48" s="8"/>
+      <c r="D48" s="9"/>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="3"/>
-      <c r="B49" s="8"/>
+      <c r="B49" s="9"/>
       <c r="C49" s="3"/>
-      <c r="D49" s="8"/>
+      <c r="D49" s="9"/>
     </row>
     <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="3"/>
-      <c r="B50" s="8"/>
+      <c r="B50" s="9"/>
       <c r="C50" s="3"/>
-      <c r="D50" s="8"/>
+      <c r="D50" s="9"/>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="3"/>
-      <c r="B51" s="8"/>
+      <c r="B51" s="9"/>
       <c r="C51" s="3"/>
-      <c r="D51" s="8"/>
+      <c r="D51" s="9"/>
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="3"/>
-      <c r="B52" s="8"/>
+      <c r="B52" s="9"/>
       <c r="C52" s="3"/>
-      <c r="D52" s="8"/>
+      <c r="D52" s="9"/>
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="3"/>
-      <c r="B53" s="8"/>
+      <c r="B53" s="9"/>
       <c r="C53" s="3"/>
-      <c r="D53" s="8"/>
+      <c r="D53" s="9"/>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="3"/>
-      <c r="B54" s="8"/>
+      <c r="B54" s="9"/>
       <c r="C54" s="3"/>
-      <c r="D54" s="8"/>
+      <c r="D54" s="9"/>
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="3"/>
-      <c r="B55" s="8"/>
+      <c r="B55" s="9"/>
       <c r="C55" s="3"/>
-      <c r="D55" s="8"/>
+      <c r="D55" s="9"/>
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="3"/>
-      <c r="B56" s="8"/>
+      <c r="B56" s="9"/>
       <c r="C56" s="3"/>
-      <c r="D56" s="8"/>
+      <c r="D56" s="9"/>
     </row>
     <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="3"/>
-      <c r="B57" s="8"/>
+      <c r="B57" s="9"/>
       <c r="C57" s="3"/>
-      <c r="D57" s="8"/>
+      <c r="D57" s="9"/>
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="3"/>
-      <c r="B58" s="8"/>
+      <c r="B58" s="9"/>
       <c r="C58" s="3"/>
-      <c r="D58" s="8"/>
+      <c r="D58" s="9"/>
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="3"/>
-      <c r="B59" s="8"/>
+      <c r="B59" s="9"/>
       <c r="C59" s="3"/>
-      <c r="D59" s="8"/>
+      <c r="D59" s="9"/>
     </row>
     <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="3"/>
-      <c r="B60" s="8"/>
+      <c r="B60" s="9"/>
       <c r="C60" s="3"/>
-      <c r="D60" s="8"/>
+      <c r="D60" s="9"/>
     </row>
     <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="3"/>
-      <c r="B61" s="8"/>
+      <c r="B61" s="9"/>
       <c r="C61" s="3"/>
-      <c r="D61" s="8"/>
+      <c r="D61" s="9"/>
     </row>
     <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="3"/>
-      <c r="B62" s="8"/>
+      <c r="B62" s="9"/>
       <c r="C62" s="3"/>
-      <c r="D62" s="8"/>
+      <c r="D62" s="9"/>
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="3"/>
-      <c r="B63" s="8"/>
+      <c r="B63" s="9"/>
       <c r="C63" s="3"/>
-      <c r="D63" s="8"/>
+      <c r="D63" s="9"/>
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="3"/>
-      <c r="B64" s="8"/>
+      <c r="B64" s="9"/>
       <c r="C64" s="3"/>
-      <c r="D64" s="8"/>
+      <c r="D64" s="9"/>
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="3"/>
-      <c r="B65" s="8"/>
+      <c r="B65" s="9"/>
       <c r="C65" s="3"/>
-      <c r="D65" s="8"/>
+      <c r="D65" s="9"/>
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="3"/>
-      <c r="B66" s="8"/>
+      <c r="B66" s="9"/>
       <c r="C66" s="3"/>
-      <c r="D66" s="8"/>
+      <c r="D66" s="9"/>
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="3"/>
-      <c r="B67" s="8"/>
+      <c r="B67" s="9"/>
       <c r="C67" s="3"/>
-      <c r="D67" s="8"/>
+      <c r="D67" s="9"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -6383,309 +6466,309 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D25"/>
-  <sheetFormatPr defaultColWidth="9.15234375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.16015625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="9" t="s">
-        <v>418</v>
-      </c>
-      <c r="B1" s="9" t="s">
-        <v>419</v>
-      </c>
-      <c r="C1" s="9" t="s">
-        <v>420</v>
-      </c>
-      <c r="D1" s="9" t="s">
-        <v>421</v>
+      <c r="A1" s="10" t="s">
+        <v>422</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>423</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>424</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>425</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="10" t="n">
+      <c r="A2" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="10" t="s">
-        <v>422</v>
-      </c>
-      <c r="C2" s="10" t="n">
+      <c r="B2" s="11" t="s">
+        <v>426</v>
+      </c>
+      <c r="C2" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="D2" s="10" t="s">
-        <v>423</v>
+      <c r="D2" s="11" t="s">
+        <v>427</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="10" t="n">
+      <c r="A3" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="10" t="s">
-        <v>422</v>
-      </c>
-      <c r="C3" s="10" t="n">
+      <c r="B3" s="11" t="s">
+        <v>426</v>
+      </c>
+      <c r="C3" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="D3" s="10" t="s">
-        <v>423</v>
+      <c r="D3" s="11" t="s">
+        <v>427</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="10" t="n">
+      <c r="A4" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="10" t="s">
-        <v>422</v>
-      </c>
-      <c r="C4" s="10" t="n">
+      <c r="B4" s="11" t="s">
+        <v>426</v>
+      </c>
+      <c r="C4" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="D4" s="10" t="s">
-        <v>423</v>
+      <c r="D4" s="11" t="s">
+        <v>427</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="10" t="n">
+      <c r="A5" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="10" t="s">
-        <v>422</v>
-      </c>
-      <c r="C5" s="10" t="n">
+      <c r="B5" s="11" t="s">
+        <v>426</v>
+      </c>
+      <c r="C5" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="D5" s="10" t="s">
-        <v>424</v>
+      <c r="D5" s="11" t="s">
+        <v>428</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="10" t="n">
+      <c r="A6" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="10" t="s">
-        <v>422</v>
-      </c>
-      <c r="C6" s="10" t="n">
+      <c r="B6" s="11" t="s">
+        <v>426</v>
+      </c>
+      <c r="C6" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="D6" s="10" t="s">
-        <v>424</v>
+      <c r="D6" s="11" t="s">
+        <v>428</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="10" t="n">
+      <c r="A7" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="10" t="s">
-        <v>422</v>
-      </c>
-      <c r="C7" s="10" t="n">
+      <c r="B7" s="11" t="s">
+        <v>426</v>
+      </c>
+      <c r="C7" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="D7" s="10" t="s">
-        <v>424</v>
+      <c r="D7" s="11" t="s">
+        <v>428</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="n">
+      <c r="A8" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="10" t="s">
-        <v>422</v>
-      </c>
-      <c r="C8" s="10" t="n">
+      <c r="B8" s="11" t="s">
+        <v>426</v>
+      </c>
+      <c r="C8" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="D8" s="10" t="s">
-        <v>424</v>
+      <c r="D8" s="11" t="s">
+        <v>428</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="10" t="n">
+      <c r="A9" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="10" t="s">
-        <v>422</v>
-      </c>
-      <c r="C9" s="10" t="n">
+      <c r="B9" s="11" t="s">
+        <v>426</v>
+      </c>
+      <c r="C9" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="D9" s="10" t="s">
-        <v>424</v>
+      <c r="D9" s="11" t="s">
+        <v>428</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10" t="n">
+      <c r="A10" s="11" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="10" t="s">
-        <v>425</v>
-      </c>
-      <c r="C10" s="10" t="n">
+      <c r="B10" s="11" t="s">
+        <v>429</v>
+      </c>
+      <c r="C10" s="11" t="n">
         <v>9</v>
       </c>
-      <c r="D10" s="10" t="s">
-        <v>424</v>
+      <c r="D10" s="11" t="s">
+        <v>428</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="10" t="n">
+      <c r="A11" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="10" t="s">
-        <v>425</v>
-      </c>
-      <c r="C11" s="10" t="n">
+      <c r="B11" s="11" t="s">
+        <v>429</v>
+      </c>
+      <c r="C11" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="D11" s="10" t="s">
-        <v>423</v>
+      <c r="D11" s="11" t="s">
+        <v>427</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="10" t="n">
+      <c r="A12" s="11" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="10" t="s">
-        <v>425</v>
-      </c>
-      <c r="C12" s="10" t="n">
+      <c r="B12" s="11" t="s">
+        <v>429</v>
+      </c>
+      <c r="C12" s="11" t="n">
         <v>11</v>
       </c>
-      <c r="D12" s="10" t="s">
-        <v>423</v>
+      <c r="D12" s="11" t="s">
+        <v>427</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="10" t="n">
+      <c r="A13" s="11" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="10" t="s">
-        <v>425</v>
-      </c>
-      <c r="C13" s="10" t="n">
+      <c r="B13" s="11" t="s">
+        <v>429</v>
+      </c>
+      <c r="C13" s="11" t="n">
         <v>12</v>
       </c>
-      <c r="D13" s="10" t="s">
-        <v>423</v>
+      <c r="D13" s="11" t="s">
+        <v>427</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="10" t="n">
+      <c r="A14" s="11" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="10" t="s">
-        <v>425</v>
-      </c>
-      <c r="C14" s="10"/>
-      <c r="D14" s="10"/>
+      <c r="B14" s="11" t="s">
+        <v>429</v>
+      </c>
+      <c r="C14" s="11"/>
+      <c r="D14" s="11"/>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="10" t="n">
+      <c r="A15" s="11" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="10" t="s">
-        <v>425</v>
-      </c>
-      <c r="C15" s="10"/>
-      <c r="D15" s="10"/>
+      <c r="B15" s="11" t="s">
+        <v>429</v>
+      </c>
+      <c r="C15" s="11"/>
+      <c r="D15" s="11"/>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="10" t="n">
+      <c r="A16" s="11" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="10" t="s">
-        <v>425</v>
-      </c>
-      <c r="C16" s="10"/>
-      <c r="D16" s="10"/>
+      <c r="B16" s="11" t="s">
+        <v>429</v>
+      </c>
+      <c r="C16" s="11"/>
+      <c r="D16" s="11"/>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="10" t="n">
+      <c r="A17" s="11" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="10" t="s">
-        <v>425</v>
-      </c>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
+      <c r="B17" s="11" t="s">
+        <v>429</v>
+      </c>
+      <c r="C17" s="11"/>
+      <c r="D17" s="11"/>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="10" t="n">
+      <c r="A18" s="11" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="10" t="s">
-        <v>425</v>
-      </c>
-      <c r="C18" s="10"/>
-      <c r="D18" s="10"/>
+      <c r="B18" s="11" t="s">
+        <v>429</v>
+      </c>
+      <c r="C18" s="11"/>
+      <c r="D18" s="11"/>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="10" t="n">
+      <c r="A19" s="11" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="10" t="s">
-        <v>425</v>
-      </c>
-      <c r="C19" s="10"/>
-      <c r="D19" s="10"/>
+      <c r="B19" s="11" t="s">
+        <v>429</v>
+      </c>
+      <c r="C19" s="11"/>
+      <c r="D19" s="11"/>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="10" t="n">
+      <c r="A20" s="11" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="10" t="s">
-        <v>425</v>
-      </c>
-      <c r="C20" s="10"/>
-      <c r="D20" s="10"/>
+      <c r="B20" s="11" t="s">
+        <v>429</v>
+      </c>
+      <c r="C20" s="11"/>
+      <c r="D20" s="11"/>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="10" t="n">
+      <c r="A21" s="11" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="10" t="s">
-        <v>425</v>
-      </c>
-      <c r="C21" s="10"/>
-      <c r="D21" s="10"/>
+      <c r="B21" s="11" t="s">
+        <v>429</v>
+      </c>
+      <c r="C21" s="11"/>
+      <c r="D21" s="11"/>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="10" t="n">
+      <c r="A22" s="11" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="10" t="s">
-        <v>422</v>
-      </c>
-      <c r="C22" s="10"/>
-      <c r="D22" s="10"/>
+      <c r="B22" s="11" t="s">
+        <v>426</v>
+      </c>
+      <c r="C22" s="11"/>
+      <c r="D22" s="11"/>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="10" t="n">
+      <c r="A23" s="11" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="10" t="s">
-        <v>422</v>
-      </c>
-      <c r="C23" s="10"/>
-      <c r="D23" s="10"/>
+      <c r="B23" s="11" t="s">
+        <v>426</v>
+      </c>
+      <c r="C23" s="11"/>
+      <c r="D23" s="11"/>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="10" t="n">
+      <c r="A24" s="11" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="10" t="s">
-        <v>422</v>
-      </c>
-      <c r="C24" s="10"/>
-      <c r="D24" s="10"/>
+      <c r="B24" s="11" t="s">
+        <v>426</v>
+      </c>
+      <c r="C24" s="11"/>
+      <c r="D24" s="11"/>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="10" t="n">
+      <c r="A25" s="11" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="10" t="s">
-        <v>422</v>
-      </c>
-      <c r="C25" s="10"/>
-      <c r="D25" s="10"/>
+      <c r="B25" s="11" t="s">
+        <v>426</v>
+      </c>
+      <c r="C25" s="11"/>
+      <c r="D25" s="11"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
tests: update MAIN_PARAMS_2025.xlsx resource file, sheet "PEAK_PARAMS"
</commit_message>
<xml_diff>
--- a/tests/antares/resources/MAIN_PARAMS_2025.xlsx
+++ b/tests/antares/resources/MAIN_PARAMS_2025.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="PAYS" sheetId="1" state="visible" r:id="rId2"/>
@@ -1500,7 +1500,7 @@
       <family val="0"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1523,6 +1523,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF8000"/>
+        <bgColor rgb="FFFF6600"/>
       </patternFill>
     </fill>
   </fills>
@@ -1592,7 +1598,7 @@
       <alignment horizontal="right" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="17">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1641,7 +1647,23 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1657,7 +1679,7 @@
     <cellStyle name="Standard_Data provided by OT3" xfId="21"/>
     <cellStyle name="Style 45" xfId="22"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="4">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1679,6 +1701,16 @@
           <fgColor rgb="FFFBE3D6"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <charset val="1"/>
+        <family val="2"/>
+        <b val="1"/>
+        <color rgb="FF000000"/>
+        <sz val="11"/>
+      </font>
     </dxf>
   </dxfs>
   <colors>
@@ -1727,7 +1759,7 @@
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF92D050"/>
       <rgbColor rgb="FFFFCC00"/>
-      <rgbColor rgb="FFFF9900"/>
+      <rgbColor rgb="FFFF8000"/>
       <rgbColor rgb="FFFF6600"/>
       <rgbColor rgb="FF666699"/>
       <rgbColor rgb="FF969696"/>
@@ -1759,9 +1791,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
-      <xdr:colOff>108000</xdr:colOff>
+      <xdr:colOff>107640</xdr:colOff>
       <xdr:row>10</xdr:row>
-      <xdr:rowOff>126000</xdr:rowOff>
+      <xdr:rowOff>125640</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1770,8 +1802,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7533720" y="905040"/>
-          <a:ext cx="7641720" cy="1030680"/>
+          <a:off x="7538760" y="905040"/>
+          <a:ext cx="7646400" cy="1030320"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1871,9 +1903,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>540000</xdr:colOff>
+      <xdr:colOff>539640</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>166680</xdr:rowOff>
+      <xdr:rowOff>166320</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1882,8 +1914,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13581720" y="402480"/>
-          <a:ext cx="8065080" cy="1031040"/>
+          <a:off x="13583520" y="402480"/>
+          <a:ext cx="8069760" cy="1030680"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1969,7 +2001,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E107"/>
-  <sheetFormatPr defaultColWidth="10.59375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.6015625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="34.43"/>
@@ -3707,7 +3739,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B42"/>
-  <sheetFormatPr defaultColWidth="10.59375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.6015625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
@@ -4103,7 +4135,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B60"/>
-  <sheetFormatPr defaultColWidth="10.59375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.6015625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.43"/>
@@ -4606,7 +4638,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1048576"/>
-  <sheetFormatPr defaultColWidth="10.59375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.6015625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="69.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30.29"/>
@@ -5883,7 +5915,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AA67"/>
-  <sheetFormatPr defaultColWidth="9.1640625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.171875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.14"/>
@@ -9927,7 +9959,10 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D25"/>
-  <sheetFormatPr defaultColWidth="9.1640625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.171875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.35"/>
+  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
@@ -9943,295 +9978,393 @@
         <v>465</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="13" t="s">
         <v>466</v>
       </c>
-      <c r="C2" s="12" t="n">
+      <c r="C2" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="D2" s="14" t="s">
         <v>467</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="13" t="s">
         <v>466</v>
       </c>
-      <c r="C3" s="12" t="n">
+      <c r="C3" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="D3" s="12" t="s">
+      <c r="D3" s="14" t="s">
         <v>467</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="13" t="s">
         <v>466</v>
       </c>
-      <c r="C4" s="12" t="n">
+      <c r="C4" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="D4" s="12" t="s">
+      <c r="D4" s="14" t="s">
         <v>467</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="B5" s="13" t="s">
         <v>466</v>
       </c>
-      <c r="C5" s="12" t="n">
+      <c r="C5" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="D5" s="12" t="s">
+      <c r="D5" s="14" t="s">
         <v>468</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="B6" s="13" t="s">
         <v>466</v>
       </c>
-      <c r="C6" s="12" t="n">
+      <c r="C6" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="D6" s="12" t="s">
+      <c r="D6" s="14" t="s">
         <v>468</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="B7" s="13" t="s">
         <v>466</v>
       </c>
-      <c r="C7" s="12" t="n">
+      <c r="C7" s="14" t="n">
         <v>6</v>
       </c>
-      <c r="D7" s="12" t="s">
+      <c r="D7" s="14" t="s">
         <v>468</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="12" t="s">
+      <c r="B8" s="13" t="s">
         <v>466</v>
       </c>
-      <c r="C8" s="12" t="n">
+      <c r="C8" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="D8" s="12" t="s">
+      <c r="D8" s="14" t="s">
         <v>468</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="B9" s="13" t="s">
         <v>466</v>
       </c>
-      <c r="C9" s="12" t="n">
+      <c r="C9" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="D9" s="12" t="s">
+      <c r="D9" s="14" t="s">
         <v>468</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="12" t="n">
+      <c r="A10" s="15" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="12" t="s">
+      <c r="B10" s="16" t="s">
         <v>469</v>
       </c>
-      <c r="C10" s="12" t="n">
+      <c r="C10" s="14" t="n">
         <v>9</v>
       </c>
-      <c r="D10" s="12" t="s">
+      <c r="D10" s="14" t="s">
         <v>468</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="12" t="n">
+      <c r="A11" s="15" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="12" t="s">
+      <c r="B11" s="16" t="s">
         <v>469</v>
       </c>
-      <c r="C11" s="12" t="n">
+      <c r="C11" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="D11" s="12" t="s">
+      <c r="D11" s="14" t="s">
         <v>467</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="12" t="n">
+      <c r="A12" s="15" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="12" t="s">
+      <c r="B12" s="16" t="s">
         <v>469</v>
       </c>
-      <c r="C12" s="12" t="n">
+      <c r="C12" s="14" t="n">
         <v>11</v>
       </c>
-      <c r="D12" s="12" t="s">
+      <c r="D12" s="14" t="s">
         <v>467</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="12" t="n">
+      <c r="A13" s="15" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="12" t="s">
+      <c r="B13" s="16" t="s">
         <v>469</v>
       </c>
-      <c r="C13" s="12" t="n">
+      <c r="C13" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="D13" s="12" t="s">
+      <c r="D13" s="14" t="s">
         <v>467</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="12" t="n">
+      <c r="A14" s="15" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="12" t="s">
+      <c r="B14" s="16" t="s">
         <v>469</v>
       </c>
-      <c r="C14" s="12"/>
-      <c r="D14" s="12"/>
+      <c r="C14" s="14"/>
+      <c r="D14" s="14"/>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="12" t="n">
+      <c r="A15" s="15" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="12" t="s">
+      <c r="B15" s="16" t="s">
         <v>469</v>
       </c>
-      <c r="C15" s="12"/>
-      <c r="D15" s="12"/>
+      <c r="C15" s="14"/>
+      <c r="D15" s="14"/>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="12" t="n">
+      <c r="A16" s="15" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="12" t="s">
+      <c r="B16" s="16" t="s">
         <v>469</v>
       </c>
-      <c r="C16" s="12"/>
-      <c r="D16" s="12"/>
+      <c r="C16" s="14"/>
+      <c r="D16" s="14"/>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="12" t="n">
+      <c r="A17" s="15" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="12" t="s">
+      <c r="B17" s="16" t="s">
         <v>469</v>
       </c>
-      <c r="C17" s="12"/>
-      <c r="D17" s="12"/>
+      <c r="C17" s="14"/>
+      <c r="D17" s="14"/>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="12" t="n">
+      <c r="A18" s="15" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="12" t="s">
+      <c r="B18" s="16" t="s">
         <v>469</v>
       </c>
-      <c r="C18" s="12"/>
-      <c r="D18" s="12"/>
+      <c r="C18" s="14"/>
+      <c r="D18" s="14"/>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="12" t="n">
+      <c r="A19" s="15" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="12" t="s">
+      <c r="B19" s="16" t="s">
         <v>469</v>
       </c>
-      <c r="C19" s="12"/>
-      <c r="D19" s="12"/>
+      <c r="C19" s="14"/>
+      <c r="D19" s="14"/>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="12" t="n">
+      <c r="A20" s="15" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="12" t="s">
+      <c r="B20" s="16" t="s">
         <v>469</v>
       </c>
-      <c r="C20" s="12"/>
-      <c r="D20" s="12"/>
+      <c r="C20" s="14"/>
+      <c r="D20" s="14"/>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="12" t="n">
+      <c r="A21" s="15" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="12" t="s">
+      <c r="B21" s="16" t="s">
         <v>469</v>
       </c>
-      <c r="C21" s="12"/>
-      <c r="D21" s="12"/>
+      <c r="C21" s="14"/>
+      <c r="D21" s="14"/>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="12" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="12" t="s">
+      <c r="B22" s="13" t="s">
         <v>466</v>
       </c>
-      <c r="C22" s="12"/>
-      <c r="D22" s="12"/>
+      <c r="C22" s="14"/>
+      <c r="D22" s="14"/>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="12" t="s">
+      <c r="B23" s="13" t="s">
         <v>466</v>
       </c>
-      <c r="C23" s="12"/>
-      <c r="D23" s="12"/>
+      <c r="C23" s="14"/>
+      <c r="D23" s="14"/>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="12" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="12" t="s">
+      <c r="B24" s="13" t="s">
         <v>466</v>
       </c>
-      <c r="C24" s="12"/>
-      <c r="D24" s="12"/>
+      <c r="C24" s="14"/>
+      <c r="D24" s="14"/>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="12" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="12" t="s">
+      <c r="B25" s="13" t="s">
         <v>466</v>
       </c>
-      <c r="C25" s="12"/>
-      <c r="D25" s="12"/>
+      <c r="C25" s="14"/>
+      <c r="D25" s="14"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="B2:B25">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
+      <formula>hc</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B2:B25">
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3:B25">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max" val="0"/>
+        <color rgb="FFFF0000"/>
+        <color rgb="FFFFFF00"/>
+        <color rgb="FF00A933"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max" val="0"/>
+        <color rgb="FFFF0000"/>
+        <color rgb="FFFFFF00"/>
+        <color rgb="FF00A933"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3:B9">
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="min" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max" val="0"/>
+        <color rgb="FFFF0000"/>
+        <color rgb="FFFFFF00"/>
+        <color rgb="FF00A933"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="min" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max" val="0"/>
+        <color rgb="FFFF0000"/>
+        <color rgb="FFFFFF00"/>
+        <color rgb="FF00A933"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3:B9">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max" val="0"/>
+        <color rgb="FFFF0000"/>
+        <color rgb="FFFFFF00"/>
+        <color rgb="FF00A933"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="min" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max" val="0"/>
+        <color rgb="FFFF0000"/>
+        <color rgb="FFFFFF00"/>
+        <color rgb="FF00A933"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B2:B9">
+    <cfRule type="colorScale" priority="10">
+      <colorScale>
+        <cfvo type="min" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max" val="0"/>
+        <color rgb="FFFF0000"/>
+        <color rgb="FFFFFF00"/>
+        <color rgb="FF00A933"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="11">
+      <colorScale>
+        <cfvo type="min" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max" val="0"/>
+        <color rgb="FFFF0000"/>
+        <color rgb="FFFFFF00"/>
+        <color rgb="FF00A933"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
feat: - Add init batteries part - new sheet referential - input file
</commit_message>
<xml_diff>
--- a/tests/antares/resources/MAIN_PARAMS_2025.xlsx
+++ b/tests/antares/resources/MAIN_PARAMS_2025.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="PAYS" sheetId="1" state="visible" r:id="rId2"/>
@@ -14,6 +14,7 @@
     <sheet name="CLUSTER" sheetId="4" state="visible" r:id="rId5"/>
     <sheet name="Common Data" sheetId="5" state="visible" r:id="rId6"/>
     <sheet name="PEAK_PARAMS" sheetId="6" state="visible" r:id="rId7"/>
+    <sheet name="BATTERIES" sheetId="7" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">CLUSTER!$A$1:$D$93</definedName>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1216" uniqueCount="469">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1244" uniqueCount="489">
   <si>
     <t xml:space="preserve">Nom_pays</t>
   </si>
@@ -1435,6 +1436,66 @@
   </si>
   <si>
     <t xml:space="preserve">HP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SCENARIO_AGREGATION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PEMMDB_PLANT_TYPE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OP_STAT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GROUP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REFERENCE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">duration 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Battery utility scale;Battery residential</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Available on market </t>
+  </si>
+  <si>
+    <t xml:space="preserve">battery</t>
+  </si>
+  <si>
+    <t xml:space="preserve">battery_</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HOUR_STO </t>
+  </si>
+  <si>
+    <t xml:space="preserve">duration 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Battery residential</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Out of market - for PV/battery dispatch optimization</t>
+  </si>
+  <si>
+    <t xml:space="preserve">battery_out</t>
+  </si>
+  <si>
+    <t xml:space="preserve">battery_residential</t>
+  </si>
+  <si>
+    <t xml:space="preserve">class 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Battery utility scale ; Battery residential</t>
+  </si>
+  <si>
+    <t xml:space="preserve">class 2</t>
   </si>
 </sst>
 </file>
@@ -1446,7 +1507,7 @@
     <numFmt numFmtId="165" formatCode="_-[$€-2]* #,##0.00_-;\-[$€-2]* #,##0.00_-;_-[$€-2]* \-??_-"/>
     <numFmt numFmtId="166" formatCode="0"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -1495,8 +1556,14 @@
       <name val="Times New Roman"/>
       <family val="0"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="0"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1512,13 +1579,31 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFBE3D6"/>
-        <bgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE7E6E6"/>
+        <bgColor rgb="FFDEEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDEEBF7"/>
+        <bgColor rgb="FFE7E6E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor rgb="FFFBE3D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -1588,7 +1673,7 @@
       <alignment horizontal="right" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1641,6 +1726,18 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="9">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1680,7 +1777,7 @@
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
-      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFE7E6E6"/>
       <rgbColor rgb="FFFF0000"/>
       <rgbColor rgb="FF00FF00"/>
       <rgbColor rgb="FF0000FF"/>
@@ -1697,8 +1794,8 @@
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFBE3D6"/>
-      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFFFF2CC"/>
+      <rgbColor rgb="FFDEEBF7"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
@@ -1718,7 +1815,7 @@
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FFFBE3D6"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF92D050"/>
@@ -1751,9 +1848,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
-      <xdr:colOff>107640</xdr:colOff>
+      <xdr:colOff>107280</xdr:colOff>
       <xdr:row>10</xdr:row>
-      <xdr:rowOff>125640</xdr:rowOff>
+      <xdr:rowOff>125280</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1762,8 +1859,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7538760" y="905040"/>
-          <a:ext cx="7646400" cy="1030320"/>
+          <a:off x="7543800" y="905040"/>
+          <a:ext cx="7651080" cy="1029960"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1863,9 +1960,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>539640</xdr:colOff>
+      <xdr:colOff>539280</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>166320</xdr:rowOff>
+      <xdr:rowOff>165960</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1874,8 +1971,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13583520" y="402480"/>
-          <a:ext cx="8069760" cy="1030680"/>
+          <a:off x="13585680" y="402480"/>
+          <a:ext cx="8074440" cy="1030320"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1955,13 +2052,715 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>420840</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>108720</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>546120</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>118080</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="ZoneTexte 2"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="13114440" y="1310040"/>
+          <a:ext cx="6627600" cy="3260520"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="ffffff"/>
+        </a:solidFill>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0"/>
+        <a:fillRef idx="0"/>
+        <a:effectRef idx="0"/>
+        <a:fontRef idx="minor"/>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr horzOverflow="clip" vertOverflow="clip" lIns="90000" rIns="90000" tIns="45000" bIns="45000" anchor="t">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:p>
+          <a:pPr>
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>Indications pour remplir ces </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>informations :</a:t>
+          </a:r>
+          <a:endParaRPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+            <a:latin typeface="Times New Roman"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr>
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t> </a:t>
+          </a:r>
+          <a:endParaRPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+            <a:latin typeface="Times New Roman"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr>
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>- colonne </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>"SCENARIO_AGREGATION " :</a:t>
+          </a:r>
+          <a:endParaRPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+            <a:latin typeface="Times New Roman"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr>
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t> </a:t>
+          </a:r>
+          <a:endParaRPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+            <a:latin typeface="Times New Roman"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr>
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>&gt;&gt; mettre duration 1 si on </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>veut agréger par durée de </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>stock et zone de marché</a:t>
+          </a:r>
+          <a:endParaRPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+            <a:latin typeface="Times New Roman"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr>
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>&gt;&gt; mettre duration 2 si on </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>agrege par zone de marché</a:t>
+          </a:r>
+          <a:endParaRPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+            <a:latin typeface="Times New Roman"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr>
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t> </a:t>
+          </a:r>
+          <a:endParaRPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+            <a:latin typeface="Times New Roman"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr>
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>&gt;&gt; mettre class 1 si on veut </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>agréger par intervalle de </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>durée de stock et zone de </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>marché</a:t>
+          </a:r>
+          <a:endParaRPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+            <a:latin typeface="Times New Roman"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr>
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>&gt;&gt; mettre class 2 si on veut </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>agréger par intervalle zone de </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>marché</a:t>
+          </a:r>
+          <a:endParaRPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+            <a:latin typeface="Times New Roman"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr>
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t> </a:t>
+          </a:r>
+          <a:endParaRPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+            <a:latin typeface="Times New Roman"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr>
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>- colonne "REFERENCE" : sert à </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>paramétrer le nommage des </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>clusters (colonne NAME) :</a:t>
+          </a:r>
+          <a:endParaRPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+            <a:latin typeface="Times New Roman"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr>
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t> </a:t>
+          </a:r>
+          <a:endParaRPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+            <a:latin typeface="Times New Roman"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr>
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>&gt;&gt; si == HOUR_STO, le script </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>va agréger à la cellule de la </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>colonne NAME la durée de </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>stockage (ex : battery_2h)</a:t>
+          </a:r>
+          <a:endParaRPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+            <a:latin typeface="Times New Roman"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr>
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>&gt;&gt; si == TYPE, le script va </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>agréger à la cellule de la </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>colonne NAME l'intervalle de </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>stockage ("short", "middle" ou </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>"long")</a:t>
+          </a:r>
+          <a:endParaRPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+            <a:latin typeface="Times New Roman"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr>
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>  </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>- Si durée de stock =&gt;3h : la </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>batterie s'appellera </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>battery_short</a:t>
+          </a:r>
+          <a:endParaRPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+            <a:latin typeface="Times New Roman"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr>
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>  </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>- Si durée de stock [4,8h] : la </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>batterie s'appellera </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>battery_middle</a:t>
+          </a:r>
+          <a:endParaRPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+            <a:latin typeface="Times New Roman"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr>
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>  </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>- Si durée de stock &gt;8h : la </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>batterie s'appellera </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>battery_long</a:t>
+          </a:r>
+          <a:endParaRPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+            <a:latin typeface="Times New Roman"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr>
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t> </a:t>
+          </a:r>
+          <a:endParaRPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+            <a:latin typeface="Times New Roman"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr>
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>&gt;&gt; si cellule vide, le script va </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>prendre suelement la donnée </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>de la colonne NAME (ex : </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>battery_residential")</a:t>
+          </a:r>
+          <a:endParaRPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+            <a:latin typeface="Times New Roman"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr>
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+          </a:pPr>
+          <a:endParaRPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
+            <a:latin typeface="Times New Roman"/>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E109"/>
-  <sheetFormatPr defaultColWidth="10.6015625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.609375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="34.43"/>
@@ -3647,7 +4446,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B42"/>
-  <sheetFormatPr defaultColWidth="10.6015625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.609375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
@@ -4043,7 +4842,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B60"/>
-  <sheetFormatPr defaultColWidth="10.6015625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.609375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.43"/>
@@ -4546,7 +5345,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1048576"/>
-  <sheetFormatPr defaultColWidth="10.6015625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.609375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="69.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30.29"/>
@@ -10179,6 +10978,130 @@
     <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;Kffffff&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;KffffffPage &amp;P</oddFooter>
   </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="23.96"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34.32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="44.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10.95"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16.9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12.05"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="13" t="s">
+        <v>469</v>
+      </c>
+      <c r="B1" s="14" t="s">
+        <v>470</v>
+      </c>
+      <c r="C1" s="14" t="s">
+        <v>471</v>
+      </c>
+      <c r="D1" s="15" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1" s="15" t="s">
+        <v>473</v>
+      </c>
+      <c r="F1" s="15" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>475</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>476</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>478</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>479</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>481</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>482</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>483</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>484</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>485</v>
+      </c>
+      <c r="F3" s="3"/>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>486</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>487</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>478</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>479</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
+        <v>488</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>482</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>483</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>484</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>485</v>
+      </c>
+      <c r="F5" s="3"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
refactor: remove battery-related code and references from main parameters logic
</commit_message>
<xml_diff>
--- a/tests/antares/resources/MAIN_PARAMS_2025.xlsx
+++ b/tests/antares/resources/MAIN_PARAMS_2025.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="6"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="PAYS" sheetId="1" state="visible" r:id="rId2"/>
@@ -14,7 +14,6 @@
     <sheet name="CLUSTER" sheetId="4" state="visible" r:id="rId5"/>
     <sheet name="Common Data" sheetId="5" state="visible" r:id="rId6"/>
     <sheet name="PEAK_PARAMS" sheetId="6" state="visible" r:id="rId7"/>
-    <sheet name="BATTERIES" sheetId="7" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">CLUSTER!$A$1:$D$93</definedName>
@@ -29,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1244" uniqueCount="489">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1216" uniqueCount="469">
   <si>
     <t xml:space="preserve">Nom_pays</t>
   </si>
@@ -1436,66 +1435,6 @@
   </si>
   <si>
     <t xml:space="preserve">HP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SCENARIO_AGREGATION</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PEMMDB_PLANT_TYPE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OP_STAT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GROUP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NAME</t>
-  </si>
-  <si>
-    <t xml:space="preserve">REFERENCE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">duration 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Battery utility scale;Battery residential</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Available on market </t>
-  </si>
-  <si>
-    <t xml:space="preserve">battery</t>
-  </si>
-  <si>
-    <t xml:space="preserve">battery_</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HOUR_STO </t>
-  </si>
-  <si>
-    <t xml:space="preserve">duration 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Battery residential</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Out of market - for PV/battery dispatch optimization</t>
-  </si>
-  <si>
-    <t xml:space="preserve">battery_out</t>
-  </si>
-  <si>
-    <t xml:space="preserve">battery_residential</t>
-  </si>
-  <si>
-    <t xml:space="preserve">class 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Battery utility scale ; Battery residential</t>
-  </si>
-  <si>
-    <t xml:space="preserve">class 2</t>
   </si>
 </sst>
 </file>
@@ -1507,7 +1446,7 @@
     <numFmt numFmtId="165" formatCode="_-[$€-2]* #,##0.00_-;\-[$€-2]* #,##0.00_-;_-[$€-2]* \-??_-"/>
     <numFmt numFmtId="166" formatCode="0"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -1556,14 +1495,8 @@
       <name val="Times New Roman"/>
       <family val="0"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="0"/>
-    </font>
   </fonts>
-  <fills count="8">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1579,31 +1512,13 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFBE3D6"/>
-        <bgColor rgb="FFFFF2CC"/>
+        <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor rgb="FFFFFF00"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE7E6E6"/>
-        <bgColor rgb="FFDEEBF7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFDEEBF7"/>
-        <bgColor rgb="FFE7E6E6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
-        <bgColor rgb="FFFBE3D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -1673,7 +1588,7 @@
       <alignment horizontal="right" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="13">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1726,18 +1641,6 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
   </cellXfs>
   <cellStyles count="9">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1777,7 +1680,7 @@
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
-      <rgbColor rgb="FFE7E6E6"/>
+      <rgbColor rgb="FFFFFFFF"/>
       <rgbColor rgb="FFFF0000"/>
       <rgbColor rgb="FF00FF00"/>
       <rgbColor rgb="FF0000FF"/>
@@ -1794,8 +1697,8 @@
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFF2CC"/>
-      <rgbColor rgb="FFDEEBF7"/>
+      <rgbColor rgb="FFFBE3D6"/>
+      <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
@@ -1815,7 +1718,7 @@
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFBE3D6"/>
+      <rgbColor rgb="FFFFCC99"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF92D050"/>
@@ -1848,9 +1751,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
-      <xdr:colOff>107280</xdr:colOff>
+      <xdr:colOff>106920</xdr:colOff>
       <xdr:row>10</xdr:row>
-      <xdr:rowOff>125280</xdr:rowOff>
+      <xdr:rowOff>124920</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1859,8 +1762,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7543800" y="905040"/>
-          <a:ext cx="7651080" cy="1029960"/>
+          <a:off x="7548840" y="905040"/>
+          <a:ext cx="7655760" cy="1029600"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1960,9 +1863,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>539280</xdr:colOff>
+      <xdr:colOff>538920</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>165960</xdr:rowOff>
+      <xdr:rowOff>165600</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1971,8 +1874,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13585680" y="402480"/>
-          <a:ext cx="8074440" cy="1030320"/>
+          <a:off x="13587480" y="402480"/>
+          <a:ext cx="8079120" cy="1029960"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2052,715 +1955,13 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>420840</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>108720</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>546120</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>118080</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp>
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="2" name="ZoneTexte 2"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="13114440" y="1310040"/>
-          <a:ext cx="6627600" cy="3260520"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="ffffff"/>
-        </a:solidFill>
-        <a:ln w="0">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0"/>
-        <a:fillRef idx="0"/>
-        <a:effectRef idx="0"/>
-        <a:fontRef idx="minor"/>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr horzOverflow="clip" vertOverflow="clip" lIns="90000" rIns="90000" tIns="45000" bIns="45000" anchor="t">
-          <a:noAutofit/>
-        </a:bodyPr>
-        <a:p>
-          <a:pPr>
-            <a:lnSpc>
-              <a:spcPct val="100000"/>
-            </a:lnSpc>
-          </a:pPr>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>Indications pour remplir ces </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>informations :</a:t>
-          </a:r>
-          <a:endParaRPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-            <a:latin typeface="Times New Roman"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr>
-            <a:lnSpc>
-              <a:spcPct val="100000"/>
-            </a:lnSpc>
-          </a:pPr>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t> </a:t>
-          </a:r>
-          <a:endParaRPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-            <a:latin typeface="Times New Roman"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr>
-            <a:lnSpc>
-              <a:spcPct val="100000"/>
-            </a:lnSpc>
-          </a:pPr>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>- colonne </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>"SCENARIO_AGREGATION " :</a:t>
-          </a:r>
-          <a:endParaRPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-            <a:latin typeface="Times New Roman"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr>
-            <a:lnSpc>
-              <a:spcPct val="100000"/>
-            </a:lnSpc>
-          </a:pPr>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t> </a:t>
-          </a:r>
-          <a:endParaRPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-            <a:latin typeface="Times New Roman"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr>
-            <a:lnSpc>
-              <a:spcPct val="100000"/>
-            </a:lnSpc>
-          </a:pPr>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>&gt;&gt; mettre duration 1 si on </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>veut agréger par durée de </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>stock et zone de marché</a:t>
-          </a:r>
-          <a:endParaRPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-            <a:latin typeface="Times New Roman"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr>
-            <a:lnSpc>
-              <a:spcPct val="100000"/>
-            </a:lnSpc>
-          </a:pPr>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>&gt;&gt; mettre duration 2 si on </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>agrege par zone de marché</a:t>
-          </a:r>
-          <a:endParaRPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-            <a:latin typeface="Times New Roman"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr>
-            <a:lnSpc>
-              <a:spcPct val="100000"/>
-            </a:lnSpc>
-          </a:pPr>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t> </a:t>
-          </a:r>
-          <a:endParaRPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-            <a:latin typeface="Times New Roman"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr>
-            <a:lnSpc>
-              <a:spcPct val="100000"/>
-            </a:lnSpc>
-          </a:pPr>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>&gt;&gt; mettre class 1 si on veut </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>agréger par intervalle de </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>durée de stock et zone de </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>marché</a:t>
-          </a:r>
-          <a:endParaRPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-            <a:latin typeface="Times New Roman"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr>
-            <a:lnSpc>
-              <a:spcPct val="100000"/>
-            </a:lnSpc>
-          </a:pPr>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>&gt;&gt; mettre class 2 si on veut </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>agréger par intervalle zone de </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>marché</a:t>
-          </a:r>
-          <a:endParaRPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-            <a:latin typeface="Times New Roman"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr>
-            <a:lnSpc>
-              <a:spcPct val="100000"/>
-            </a:lnSpc>
-          </a:pPr>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t> </a:t>
-          </a:r>
-          <a:endParaRPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-            <a:latin typeface="Times New Roman"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr>
-            <a:lnSpc>
-              <a:spcPct val="100000"/>
-            </a:lnSpc>
-          </a:pPr>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>- colonne "REFERENCE" : sert à </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>paramétrer le nommage des </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>clusters (colonne NAME) :</a:t>
-          </a:r>
-          <a:endParaRPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-            <a:latin typeface="Times New Roman"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr>
-            <a:lnSpc>
-              <a:spcPct val="100000"/>
-            </a:lnSpc>
-          </a:pPr>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t> </a:t>
-          </a:r>
-          <a:endParaRPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-            <a:latin typeface="Times New Roman"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr>
-            <a:lnSpc>
-              <a:spcPct val="100000"/>
-            </a:lnSpc>
-          </a:pPr>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>&gt;&gt; si == HOUR_STO, le script </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>va agréger à la cellule de la </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>colonne NAME la durée de </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>stockage (ex : battery_2h)</a:t>
-          </a:r>
-          <a:endParaRPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-            <a:latin typeface="Times New Roman"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr>
-            <a:lnSpc>
-              <a:spcPct val="100000"/>
-            </a:lnSpc>
-          </a:pPr>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>&gt;&gt; si == TYPE, le script va </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>agréger à la cellule de la </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>colonne NAME l'intervalle de </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>stockage ("short", "middle" ou </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>"long")</a:t>
-          </a:r>
-          <a:endParaRPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-            <a:latin typeface="Times New Roman"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr>
-            <a:lnSpc>
-              <a:spcPct val="100000"/>
-            </a:lnSpc>
-          </a:pPr>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>  </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>- Si durée de stock =&gt;3h : la </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>batterie s'appellera </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>battery_short</a:t>
-          </a:r>
-          <a:endParaRPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-            <a:latin typeface="Times New Roman"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr>
-            <a:lnSpc>
-              <a:spcPct val="100000"/>
-            </a:lnSpc>
-          </a:pPr>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>  </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>- Si durée de stock [4,8h] : la </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>batterie s'appellera </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>battery_middle</a:t>
-          </a:r>
-          <a:endParaRPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-            <a:latin typeface="Times New Roman"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr>
-            <a:lnSpc>
-              <a:spcPct val="100000"/>
-            </a:lnSpc>
-          </a:pPr>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>  </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>- Si durée de stock &gt;8h : la </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>batterie s'appellera </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>battery_long</a:t>
-          </a:r>
-          <a:endParaRPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-            <a:latin typeface="Times New Roman"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr>
-            <a:lnSpc>
-              <a:spcPct val="100000"/>
-            </a:lnSpc>
-          </a:pPr>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t> </a:t>
-          </a:r>
-          <a:endParaRPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-            <a:latin typeface="Times New Roman"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr>
-            <a:lnSpc>
-              <a:spcPct val="100000"/>
-            </a:lnSpc>
-          </a:pPr>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>&gt;&gt; si cellule vide, le script va </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>prendre suelement la donnée </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>de la colonne NAME (ex : </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-            </a:rPr>
-            <a:t>battery_residential")</a:t>
-          </a:r>
-          <a:endParaRPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-            <a:latin typeface="Times New Roman"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr>
-            <a:lnSpc>
-              <a:spcPct val="100000"/>
-            </a:lnSpc>
-          </a:pPr>
-          <a:endParaRPr b="0" lang="fr-FR" sz="1100" spc="-1" strike="noStrike">
-            <a:latin typeface="Times New Roman"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E109"/>
-  <sheetFormatPr defaultColWidth="10.609375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.6171875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="34.43"/>
@@ -4446,7 +3647,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B42"/>
-  <sheetFormatPr defaultColWidth="10.609375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.6171875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
@@ -4842,7 +4043,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B60"/>
-  <sheetFormatPr defaultColWidth="10.609375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.6171875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.43"/>
@@ -5345,7 +4546,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1048576"/>
-  <sheetFormatPr defaultColWidth="10.609375" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.6171875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="69.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30.29"/>
@@ -10978,130 +10179,6 @@
     <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;Kffffff&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;KffffffPage &amp;P</oddFooter>
   </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:F5"/>
-  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="23.96"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34.32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="44.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10.95"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16.9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12.05"/>
-  </cols>
-  <sheetData>
-    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="13" t="s">
-        <v>469</v>
-      </c>
-      <c r="B1" s="14" t="s">
-        <v>470</v>
-      </c>
-      <c r="C1" s="14" t="s">
-        <v>471</v>
-      </c>
-      <c r="D1" s="15" t="s">
-        <v>472</v>
-      </c>
-      <c r="E1" s="15" t="s">
-        <v>473</v>
-      </c>
-      <c r="F1" s="15" t="s">
-        <v>474</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
-        <v>475</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>476</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>477</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>478</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>479</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>480</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
-        <v>481</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>482</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>483</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>484</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>485</v>
-      </c>
-      <c r="F3" s="3"/>
-    </row>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
-        <v>486</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>487</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>477</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>478</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>479</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
-        <v>488</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>482</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>483</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>484</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>485</v>
-      </c>
-      <c r="F5" s="3"/>
-    </row>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;Kffffff&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;KffffffPage &amp;P</oddFooter>
-  </headerFooter>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
BATTERIES : New features (#79)
</commit_message>
<xml_diff>
--- a/tests/antares/resources/MAIN_PARAMS_2025.xlsx
+++ b/tests/antares/resources/MAIN_PARAMS_2025.xlsx
@@ -1751,9 +1751,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
-      <xdr:colOff>107640</xdr:colOff>
+      <xdr:colOff>106920</xdr:colOff>
       <xdr:row>10</xdr:row>
-      <xdr:rowOff>125640</xdr:rowOff>
+      <xdr:rowOff>124920</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1762,8 +1762,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7538760" y="905040"/>
-          <a:ext cx="7646400" cy="1030320"/>
+          <a:off x="7548840" y="905040"/>
+          <a:ext cx="7655760" cy="1029600"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1863,9 +1863,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>539640</xdr:colOff>
+      <xdr:colOff>538920</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>166320</xdr:rowOff>
+      <xdr:rowOff>165600</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -1874,8 +1874,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13583520" y="402480"/>
-          <a:ext cx="8069760" cy="1030680"/>
+          <a:off x="13587480" y="402480"/>
+          <a:ext cx="8079120" cy="1029960"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1961,7 +1961,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E109"/>
-  <sheetFormatPr defaultColWidth="10.6015625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.6171875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="34.43"/>
@@ -3647,7 +3647,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B42"/>
-  <sheetFormatPr defaultColWidth="10.6015625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.6171875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
@@ -4043,7 +4043,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B60"/>
-  <sheetFormatPr defaultColWidth="10.6015625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.6171875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.43"/>
@@ -4546,7 +4546,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1048576"/>
-  <sheetFormatPr defaultColWidth="10.6015625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.6171875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="69.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30.29"/>

</xml_diff>